<commit_message>
:up: questoes do pdf 00 de RL
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:G95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -756,7 +756,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -792,7 +792,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -826,10 +826,10 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -866,7 +866,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -899,10 +899,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -936,7 +936,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -978,7 +978,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1015,7 +1015,7 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -1049,7 +1049,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -1089,7 +1089,7 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -1120,7 +1120,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -3720,9 +3720,188 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G90" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>91</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Engenharia de Métodos e Processos</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Subdivisão da Engenharia de Métodos</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Projeto de Métodos&lt;/li&gt;
+	&lt;li&gt;Padronização e Treinamento&lt;/li&gt;
+	&lt;li&gt;Medida do Trabalho&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>92</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Engenharia de Métodos e Processos</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Etapas para o estudo de métodos</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>&lt;ol&gt;
+	&lt;li&gt;Escolher o trabalho&lt;/li&gt;
+	&lt;li&gt;Registrar,&lt;/li&gt;
+	&lt;li&gt;Examinar com espírito crítico&lt;/li&gt;
+	&lt;li&gt;Desenvolver o método mais rápido&lt;/li&gt;
+	&lt;li&gt;Definir o novo método&lt;/li&gt;
+	&lt;li&gt;Implantar o novo método.&lt;/li&gt;
+	&lt;li&gt;Controlar o novo método&lt;/li&gt;
+&lt;/ol&gt;</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>93</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Ortografia Oficial</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Grafias Corretas</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Paralizado; Exceção; Adivinhar; Cabeleireiro</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>94</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Engenharia de Métodos e Processos</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Quesitos a serem levados em consideração para análise de operações</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Materias&lt;/li&gt;
+	&lt;li&gt;Manuseio de Materiais&lt;/li&gt;
+	&lt;li&gt;Ferramentas, Dispositivos e Gabaritos&lt;/li&gt;
+	&lt;li&gt;Máquina&lt;/li&gt;
+	&lt;li&gt;Operador&lt;/li&gt;
+	&lt;li&gt;Condições de Trabalho&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>95</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Engenharia de Métodos e Processos</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Perguntas fundamentais para a análise crítica de operações</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Qual é o objetivo?&lt;/li&gt;
+	&lt;li&gt;Por que é necessário?&lt;/li&gt;
+	&lt;li&gt;Onde, quando e como é feito?&lt;/li&gt;
+	&lt;li&gt;Quem executa?&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
:up: mais questões respondidas
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G99"/>
+  <dimension ref="A1:G100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -982,8 +982,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1007,7 +1009,7 @@
 	&lt;li&gt;Mapofluxograma;&lt;/li&gt;
 	&lt;li&gt;Carta de-para;&lt;/li&gt;
 	&lt;li&gt;Gráfico homem-máquina;&lt;/li&gt;
-	&lt;li&gt;Gráfico das duas mãos.&lt;/li&gt;
+	&lt;li&gt;Gráfico das duas mãos ou gráfico de operações.&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -4003,8 +4005,10 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="n">
-        <v>99</v>
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -4018,18 +4022,52 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Fórmula do Tempo Padrão</t>
+          <t>Fórmulas do Tempo Padrão</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Tempo padrão = tempo normal x fator de tolerância.</t>
+          <t>Tempo padrão = tempo normal x fator de tolerância.
+Tempo padrão = Tempo normal + Tolerâncias
+Tempo padrão = Tempo normal + (Tempo normal x tolerâncias, em %)</t>
         </is>
       </c>
       <c r="F99" t="n">
         <v>1</v>
       </c>
       <c r="G99" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>100</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Engenharia de Métodos e Processos</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Fórmula do Fator de Tolerância</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Fator de Tolerância = 1/(1-p)
+onde p é “tempo de intervalo/tempo de trabalho”</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
:up: mais questões respondidas, alguns flash criados e algumas questões salvas
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4320,6 +4320,99 @@
         <v>0</v>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>108</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Fórmula da Permutação com Repetição</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>P&lt;sub&gt;n&lt;/sub&gt;&lt;sup&gt;k&lt;sub&gt;1&lt;/sub&gt;,k&lt;sub&gt;2&lt;/sub&gt;,...k&lt;sub&gt;i&lt;/sub&gt;&lt;/sup&gt; = n!/(k&lt;sub&gt;1&lt;/sub&gt;! x k&lt;sub&gt;2&lt;/sub&gt;! x ... x k&lt;sub&gt;i&lt;/sub&gt;!)</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>109</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Fórmula da Permutação Circular</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>PC&lt;sub&gt;n&lt;/sub&gt; = (n - 1)!</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>110</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Fórmula da Combinhação com Repetiçao (ou Completa)</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>CR&lt;sup&gt;p&lt;/sup&gt;&lt;sub&gt;n&lt;/sub&gt; = P&lt;sup&gt;n-1,p&lt;/sup&gt;&lt;sub&gt;n-1+p&lt;/sub&gt; = [(n-1+p)!]/[(n-1)!xp!]</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>0</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: alguns cards de gestão do conhecimento adicionados
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4659,6 +4659,151 @@
         <v>0</v>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>118</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Abordagem Racional (Chun Wei Choo)</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Dados Quantitativos&lt;/li&gt;
+	&lt;li&gt;lógica&lt;/li&gt;
+	&lt;li&gt;objetividade&lt;/li&gt;
+	&lt;li&gt;máquina&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>119</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Abordagem Interpretativa (Chun Wei Choo)</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Dados Qualitativos&lt;/li&gt;
+	&lt;li&gt;Pessoas&lt;/li&gt;
+	&lt;li&gt;significados&lt;/li&gt;
+	&lt;li&gt;subjetividade&lt;/li&gt;
+	&lt;li&gt;cultura&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>120</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Processo de construção da Inteligência</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>&lt;ol&gt;
+	&lt;li&gt;Dado&lt;/li&gt;
+	&lt;li&gt;Informação&lt;/li&gt;
+	&lt;li&gt;Conhecimento&lt;/li&gt;
+	&lt;li&gt;Inteligência&lt;/li&gt;
+&lt;/ol&gt;</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>0</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>121</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Modelo SECI (Nonaka e Takeuchi)</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Socialização&lt;/li&gt;
+	&lt;li&gt;Externalização&lt;/li&gt;
+	&lt;li&gt;Combinação&lt;/li&gt;
+	&lt;li&gt;Internalização&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>0</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: alguns flashcards salvos - analise sintática
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G127"/>
+  <dimension ref="A1:G135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5099,6 +5099,292 @@
         <v>0</v>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>130</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Processo para análise sintática</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>&lt;ol&gt;
+	&lt;li&gt;ache o verbo&lt;/li&gt;
+	&lt;li&gt;tente colocar a sentença na ordem direta&lt;/li&gt;
+	&lt;li&gt;procurar o sujeito de cada verbo&lt;/li&gt;
+&lt;/ol&gt;</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>131</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>técnicas de indeterminação do sujeito</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;verbo na 3ª pessoa do plural, com omissão do agente que pratica a ação verbal&lt;/li&gt;
+	&lt;li&gt;uso da PIS&lt;/li&gt;
+	&lt;li&gt;uso do infinitivo impessoal&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>0</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>132</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Oração sem sujeito</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Fenômenos da natureza&lt;/li&gt;
+	&lt;li&gt;Verbos ser/estar/fazer/haver/parecer impessoais com sentido de fenômenos naturais, tempo ou estado&lt;/li&gt;
+	&lt;li&gt;verbo “haver” impessoal (com sentido de “existir”, “ocorrer” ou “tempo decorrido”)&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>0</v>
+      </c>
+      <c r="G130" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>133</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Casos de Objeto Direto Preposicionado</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Quando o objeto direto for um pronome oblíquo tônico ou “quem”&lt;/li&gt;
+	&lt;li&gt;Quando o objeto direto for verbo no infinitivo, com os verbos “ensinar” e “aprender”&lt;/li&gt;
+	&lt;li&gt;Quando houver dupla possibilidade de referente, ou seja, ambiguidade&lt;/li&gt;
+	&lt;li&gt;Quando o objeto indicar reciprocidade&lt;/li&gt;
+	&lt;li&gt;Com alguns pronomes indefinidos, sobretudo referentes a pessoas&lt;/li&gt;
+	&lt;li&gt;Quando o OD for um nome próprio&lt;/li&gt;
+	&lt;li&gt;Quando o objeto direto for a palavra “ambos”&lt;/li&gt;
+	&lt;li&gt;Quando houver reforço ou exaltação de um sentimento&lt;/li&gt;
+	&lt;li&gt;Em construções enfáticas, nas quais antecipamos o objeto direto para dar-lhe realce&lt;/li&gt;
+	&lt;li&gt;Em construções paralelas com pronomes oblíquos (átonos ou tônicos) do tipo&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>0</v>
+      </c>
+      <c r="G131" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>134</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Complemento Nominal</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;complemento de um nome que possua transitividade (substantivo, adjetivo ou advérbio), com preposição&lt;/li&gt;
+	&lt;li&gt;Parece um objeto indireto, com a diferença de que não completa o sentido de um verbo, mas sim de um nome.&lt;/li&gt;
+	&lt;li&gt;também pode ter forma de uma oração&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>0</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>135</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Adjunto Adnominal</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;acompanha substantivos concretos e abstratos para atribuir-lhes &lt;ul&gt; &lt;li&gt;características&lt;/li&gt; &lt;li&gt;qualidade ou&lt;/li&gt; &lt;li&gt;estado&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;têm função adjetiva, ou seja, modificam termo substantivo&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>0</v>
+      </c>
+      <c r="G133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>136</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Predicação Verbal</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Verbos de Ação/Movimento/Fenômeno &lt;ul&gt; &lt;li&gt;VI &lt;ul&gt; &lt;li&gt;É aquele que não precisa de complemento&lt;/li&gt; &lt;li&gt;Pode vir seguido de informações acessórias (Predicativo/Adj. Adverbial)&lt;/li&gt; &lt;/ul&gt; &lt;/li&gt; &lt;li&gt;VTD&lt;/li&gt; &lt;li&gt;VTI&lt;/li&gt; &lt;li&gt;VTDI&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Verbos de Estado/de Ligação&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>0</v>
+      </c>
+      <c r="G134" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>137</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Adjunto Adverbial</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Invariável&lt;/li&gt;
+	&lt;li&gt;Refere-se a verbo (Seta)&lt;/li&gt;
+	&lt;li&gt;Indica circunstância (Onde?/Quando?/Como?/...)&lt;/li&gt;
+	&lt;li&gt;Pode ser dispensado na frase&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>0</v>
+      </c>
+      <c r="G135" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: ultimo commit antes de tentar mudar o algoritmo do plano
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G156"/>
+  <dimension ref="A1:G158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6114,8 +6114,10 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="n">
-        <v>157</v>
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>157</t>
+        </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -6136,6 +6138,7 @@
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;"Termo que limita, individualiza a significação de um substantivo."&lt;/li&gt;
+        &lt;li&gt;Termo acessório&lt;/li&gt;
 	&lt;li&gt;Ex.: &lt;ul&gt; &lt;li&gt;&lt;b&gt;&lt;u&gt;Dois &lt;/u&gt;&lt;/b&gt;alunos; &lt;ul&gt; &lt;li&gt;(Numeral)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;O/&lt;b&gt;&lt;u&gt;Um &lt;/u&gt;&lt;/b&gt;aluno; &lt;ul&gt; &lt;li&gt;(Artigo)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;Aluno &lt;b&gt;&lt;u&gt;inteligente&lt;/u&gt;&lt;/b&gt;/&lt;b&gt;&lt;u&gt;de inteligência&lt;/u&gt;&lt;/b&gt; &lt;ul&gt; &lt;li&gt;(Adjetivo/Locução Adjetiva)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;&lt;b&gt;&lt;u&gt;Meu&lt;/u&gt;&lt;/b&gt; aluno; &lt;ul&gt; &lt;li&gt;(Pronome)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;Invasão &lt;b&gt;&lt;u&gt;dos mosquitos&lt;/u&gt;&lt;/b&gt; &lt;ul&gt; &lt;li&gt;(Locução Adjetiva)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 	&lt;li&gt;Classes gramaticais que, sintaticamente, podem exercer o papel de Adjunto Adnominal: &lt;ul&gt; &lt;li&gt;Numeral&lt;/li&gt; &lt;li&gt;Artigo&lt;/li&gt; &lt;li&gt;Pronome&lt;/li&gt; &lt;li&gt;Adjetivo&lt;/li&gt; &lt;li&gt;Locução Adjetiva&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 &lt;/ul&gt;</t>
@@ -6149,8 +6152,10 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" t="n">
-        <v>158</v>
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -6164,16 +6169,15 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Predicativo do Sujeito</t>
+          <t>Predicativos</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;Vem sempre no predicado&lt;/li&gt;
-	&lt;li&gt;Atribui característica ao sujeito &lt;ul&gt; &lt;li&gt;Vem no predicado e "manda seta" para o sujeito&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;Não vem apenas com verbo de ligação &lt;ul&gt; &lt;li&gt;Pode vir com qualquer verbo&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;Não é apenas adjetivo que pode ser predicativo do sujeito &lt;ul&gt; &lt;li&gt;Predicativo do sujeito pode ser (Substantivo/Adjetivo/Pronome/Numeral)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Vem &lt;b&gt;sempre&lt;/b&gt; no predicado&lt;/li&gt;
+	&lt;li&gt;Predicativo do Sujeito &lt;ul&gt; &lt;li&gt;Atribui característica ao sujeito &lt;ul&gt; &lt;li&gt;Vem no predicado e "manda seta" para o sujeito&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;Não vem apenas com verbo de ligação &lt;ul&gt; &lt;li&gt;Pode vir com qualquer verbo&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;Não é apenas adjetivo que pode ser predicativo do sujeito &lt;ul&gt; &lt;li&gt;Predicativo do sujeito pode ser (Substantivo/Adjetivo/Pronome/Numeral)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Predicativo do Objeto &lt;ul&gt; &lt;li&gt;Refere-se ao Objeto Direto ou Indireto&lt;/li&gt; &lt;li&gt;Se retirado, prejudica o sentido do Verbo&lt;/li&gt; &lt;li&gt;Ex.: &lt;ul&gt; &lt;li&gt;Achei-o &lt;b&gt;competente&lt;/b&gt;&lt;/li&gt; &lt;li&gt;Julguei as suas perguntas &lt;b&gt;tolas&lt;/b&gt;&lt;/li&gt; &lt;li&gt;Chamaram o delegado &lt;b&gt;de inquieto&lt;/b&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -6181,6 +6185,121 @@
         <v>0</v>
       </c>
       <c r="G156" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>159</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Passo a passo - distinguir Adjunto Adnominal de Predicativo do Objeto</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>&lt;ol&gt;
+	&lt;li&gt;Coloca a seta!&lt;/li&gt;
+	&lt;li&gt;Caso o termo se refira ao Objeto, poderá ser AA ou PO &lt;ul&gt; &lt;li&gt;Olhar para o Verbo&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Caso o termo não puder ser retirado (por "prejudicar" o verbo), será PO.&lt;/li&gt;
+&lt;/ol&gt;
+Dica: Quando é PO, você poderá deslocá-lo para perto do Verbo &lt;ul&gt; &lt;li&gt;pois sua conversa é com o verbo&lt;/li&gt; &lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>160</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Período Composto</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;&lt;strong&gt;Coordenação&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Orações Coordenadas Assindéticas (sem conectivo)&lt;/li&gt;
+			&lt;li&gt;Orações Coordenadas Sindéticas (com conectivo):
+				&lt;ul&gt;
+					&lt;li&gt;Aditivas&lt;/li&gt;
+					&lt;li&gt;Adversativas&lt;/li&gt;
+					&lt;li&gt;Alternativas&lt;/li&gt;
+					&lt;li&gt;Conclusivas&lt;/li&gt;
+					&lt;li&gt;Explicativas&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;strong&gt;Subordinação&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Orações Subordinadas Substantivas:
+				&lt;ul&gt;
+					&lt;li&gt;Subjetivas&lt;/li&gt;
+					&lt;li&gt;Objetivas Diretas&lt;/li&gt;
+					&lt;li&gt;Objetivas Indiretas&lt;/li&gt;
+					&lt;li&gt;Completivas Nominais&lt;/li&gt;
+					&lt;li&gt;Predicativas&lt;/li&gt;
+					&lt;li&gt;Apositivas&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Orações Subordinadas Adjetivas:
+				&lt;ul&gt;
+					&lt;li&gt;Restritivas&lt;/li&gt;
+					&lt;li&gt;Explicativas&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Orações Subordinadas Adverbiais:
+				&lt;ul&gt;
+					&lt;li&gt;Causais&lt;/li&gt;
+					&lt;li&gt;Comparativas&lt;/li&gt;
+					&lt;li&gt;Concessivas&lt;/li&gt;
+					&lt;li&gt;Condicionais&lt;/li&gt;
+					&lt;li&gt;Conformativas&lt;/li&gt;
+					&lt;li&gt;Consecutivas&lt;/li&gt;
+					&lt;li&gt;Finais&lt;/li&gt;
+					&lt;li&gt;Proporcionais&lt;/li&gt;
+					&lt;li&gt;Temporais&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
:up: algumas questões respondidas e organizadas
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G158"/>
+  <dimension ref="A1:G163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6299,6 +6299,181 @@
         <v>0</v>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Equação Fundamental da Contabilidade</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Ativo = Passivo + PL &lt;ul&gt; &lt;li&gt;Toda aplicação de recursos possui uma origem de igual valor&lt;/li&gt; &lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>162</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Termos Importantes</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Ativo: Bens e direitos
+Passivo: Obrigações
+Patrimônio: Líquido Capital próprio (dos sócios)
+Aplicação de recursos: Ativo
+Origem de recursos: Passivo e Patrimônio líquido
+Capital próprio: Patrimônio Líquido
+Capital de terceiros: Passivo
+Capital aplicado: Ativo</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>163</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Situação Líquida (Patrimônio Líquido) e Equação Fundamental do Patrimônio</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Ativo maior do que passivo &lt;ul&gt; &lt;li&gt;Ativo &gt; Passivo exigível&lt;/li&gt; &lt;li&gt;Situação líquida &gt; 0&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Ativo menor do que passivo &lt;ul&gt; &lt;li&gt;passivo a descoberto&lt;/li&gt; &lt;li&gt;patrimônio líquido negativo&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Ativo igual ao passivo &lt;ul&gt; &lt;li&gt;não existe capital próprio&lt;/li&gt; &lt;li&gt;Ativo = Passivo&lt;/li&gt; &lt;li&gt;Patrimônio Líquido = Zero&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Ativo igual à situação líquida &lt;ul&gt; &lt;li&gt;constituição da sociedade&lt;/li&gt; &lt;li&gt;Pode ser o caso também de uma entidade que somente trabalhe com recursos próprios&lt;/li&gt; &lt;li&gt;Ativo = Patrimônio Líquido&lt;/li&gt; &lt;li&gt;Passivo = Zero&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>164</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Atos e Fatos Contábeis</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Atos contábeis ou Atos Administrativos &lt;ul&gt; &lt;li&gt;não provocam alterações do patrimônio&lt;/li&gt; &lt;li&gt;ou apenas irão alterar o Patrimônio no futuro&lt;/li&gt; &lt;li&gt;Ex.: &lt;ul&gt; &lt;li&gt;admissão de empregados&lt;/li&gt; &lt;li&gt;assinatura de um contrato de compra&lt;/li&gt; &lt;li&gt;venda&lt;/li&gt; &lt;li&gt;o aval de um título de crédito&lt;/li&gt; &lt;li&gt;uma fiança prestada em favor de terceiros&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;Lei 6.404/76: Art. 176. (...) § 4º As demonstrações serão complementadas&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Fatos contábeis ou Fatos Administrativos &lt;ul&gt; &lt;li&gt;provocam variações no patrimônio da entidade&lt;/li&gt; &lt;li&gt;são contabilizados através &lt;ul&gt; &lt;li&gt;das contas patrimoniais (ativo, passivo, patrimônio líquido)&lt;/li&gt; &lt;li&gt;e/ou das contas de resultado (receitas e despesas)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>165</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Variações de Elementos Patrimoniais</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Subscrição do Capital Social &lt;ul&gt; &lt;li&gt;Comprometimento&lt;/li&gt; &lt;li&gt;Promessa&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Integralização do Capital Social &lt;ul&gt; &lt;li&gt;os sócios efetivamente entregam os recursos&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>0</v>
+      </c>
+      <c r="G163" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: mexer no cell terminado e algumas questões cadastradas
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -4324,7 +4324,7 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G106" t="n">
         <v>0</v>
@@ -4355,7 +4355,7 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G107" t="n">
         <v>0</v>
@@ -4391,7 +4391,7 @@
         <v>0</v>
       </c>
       <c r="G108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109">

</xml_diff>

<commit_message>
:up: algumas questões cadastradas - prova fub 2025
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -4579,7 +4579,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G113" t="n">
         <v>0</v>
@@ -4617,10 +4617,10 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G114" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115">
@@ -4653,10 +4653,10 @@
         </is>
       </c>
       <c r="F115" t="n">
+        <v>4</v>
+      </c>
+      <c r="G115" t="n">
         <v>2</v>
-      </c>
-      <c r="G115" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="116">
@@ -4689,7 +4689,7 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G116" t="n">
         <v>0</v>
@@ -4726,7 +4726,7 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G117" t="n">
         <v>0</v>
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G118" t="n">
         <v>0</v>
@@ -4798,10 +4798,10 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G120" t="n">
         <v>0</v>
@@ -4872,10 +4872,10 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G121" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="122">
@@ -4912,7 +4912,7 @@
         <v>0</v>
       </c>
       <c r="G122" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="123">
@@ -4946,10 +4946,10 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G123" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="124">
@@ -4984,7 +4984,7 @@
         <v>0</v>
       </c>
       <c r="G124" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="125">
@@ -5023,7 +5023,7 @@
         <v>0</v>
       </c>
       <c r="G125" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="126">
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G126" t="n">
         <v>1</v>
@@ -5093,7 +5093,7 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G127" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
:up: flashcards elevados - GC
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -4611,13 +4611,27 @@
           <t>&lt;ul&gt;
 	&lt;li&gt;reside nas pessoas&lt;/li&gt;
 	&lt;li&gt;é subjetivo, pessoal, difícil de formalizar&lt;/li&gt;
-	&lt;li&gt;dimensão técnica&lt;/li&gt;
-	&lt;li&gt;dimensão cognitiva&lt;/li&gt;
+	&lt;li&gt;dimensão técnica
+&lt;ul&gt;
+	&lt;li&gt;&lt;i&gt;know-how&lt;/i&gt;&lt;/li&gt;
+	&lt;li&gt;habilidades motoras&lt;/li&gt;
+	&lt;li&gt;perceptivas difíceis de verbalizar&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;dimensão cognitiva
+&lt;ul&gt;
+	&lt;li&gt;modelos mentais&lt;/li&gt;
+	&lt;li&gt;crenças&lt;/li&gt;
+	&lt;li&gt;crenças&lt;/li&gt;
+	&lt;li&gt;percepções&lt;/li&gt;
+	&lt;li&gt;intuições&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F114" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G114" t="n">
         <v>2</v>
@@ -4648,20 +4662,23 @@
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;pode ser formalizado&lt;/li&gt;
-	&lt;li&gt;é documentado, codificado e sistematizado&lt;/li&gt;
+	&lt;li&gt;é documentado, codificado e sistematizado em procedimentos, manuais, relatórios, sistemas de informação, bancos de dados&lt;/li&gt;
+&lt;li&gt;mais fácil de ser transferido entre pessoas, de ser replicado e armazenado&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G115" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="n">
-        <v>118</v>
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -4681,15 +4698,15 @@
       <c r="E116" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;Dados Quantitativos&lt;/li&gt;
-	&lt;li&gt;lógica&lt;/li&gt;
-	&lt;li&gt;objetividade&lt;/li&gt;
-	&lt;li&gt;máquina&lt;/li&gt;
+	&lt;li&gt;As decisões são tomadas com base em regras, lógica e análise objetiva da informação disponível.&lt;/li&gt;
+	&lt;li&gt;A organização é vista como uma máquina de processar dados&lt;/li&gt;
+	&lt;li&gt;eficiência e previsibilidade dos processos&lt;/li&gt;
+	&lt;li&gt;melhor escolha racional possível&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G116" t="n">
         <v>0</v>
@@ -4733,8 +4750,10 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="n">
-        <v>120</v>
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -4754,23 +4773,44 @@
       <c r="E118" t="inlineStr">
         <is>
           <t>&lt;ol&gt;
-	&lt;li&gt;Dado&lt;/li&gt;
-	&lt;li&gt;Informação&lt;/li&gt;
-	&lt;li&gt;Conhecimento&lt;/li&gt;
-	&lt;li&gt;Inteligência&lt;/li&gt;
+	&lt;li&gt;Dado
+ &lt;ul&gt;
+	&lt;li&gt;elemento isolado, desprovido de significado&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Informação
+&lt;ul&gt;
+	&lt;li&gt;dado que foi contextualizado, organizado e interpretado&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Conhecimento
+&lt;ul&gt;
+	&lt;li&gt;informação combinada com experiência, julgamento, intuição e valores&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Inteligência
+&lt;ul&gt;
+	&lt;li&gt;tomar decisões complexas,&lt;/li&gt;
+	&lt;li&gt;prever cenários futuros,&lt;/li&gt;
+	&lt;li&gt;inovar&lt;/li&gt;
+	&lt;li&gt;gerar vantagem competitiva&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
 &lt;/ol&gt;</t>
         </is>
       </c>
       <c r="F118" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G118" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="n">
-        <v>121</v>
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -4789,24 +4829,42 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>&lt;ul&gt;
-	&lt;li&gt;Socialização&lt;/li&gt;
-	&lt;li&gt;Externalização&lt;/li&gt;
-	&lt;li&gt;Combinação&lt;/li&gt;
+          <t>&lt;ol&gt;
+	&lt;li&gt;Socialização
+&lt;ul&gt;
+	&lt;li&gt;tácito → tácito&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Externalização
+&lt;ul&gt;
+	&lt;li&gt;tácito → explícito&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Combinação
+&lt;ul&gt;
+	&lt;li&gt;explícito → explícito
+&lt;ul&gt;
+	&lt;li&gt;explícito → tácito&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
 	&lt;li&gt;Internalização&lt;/li&gt;
-&lt;/ul&gt;</t>
+&lt;/ol&gt;</t>
         </is>
       </c>
       <c r="F119" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G119" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="n">
-        <v>122</v>
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>122</t>
+        </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -4826,26 +4884,69 @@
       <c r="E120" t="inlineStr">
         <is>
           <t>&lt;ol&gt;
-	&lt;li&gt;Identificação&lt;/li&gt;
-	&lt;li&gt;Captura&lt;/li&gt;
-	&lt;li&gt;Aquisição&lt;/li&gt;
-	&lt;li&gt;Armazenamento&lt;/li&gt;
-	&lt;li&gt;Compartilhamento&lt;/li&gt;
-	&lt;li&gt;Aplicação&lt;/li&gt;
-	&lt;li&gt;Avaliação&lt;/li&gt;
+	&lt;li&gt;Identificação
+&lt;ul&gt;
+	&lt;li&gt;Diagnóstico&lt;/li&gt;
+	&lt;li&gt;Mapeamento&lt;/li&gt;
+	&lt;li&gt;Localização&lt;/li&gt;
+	&lt;li&gt;Reconhecimento&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Captura
+&lt;ul&gt;
+	&lt;li&gt;Entrevistas&lt;/li&gt;
+	&lt;li&gt;Relatos&lt;/li&gt;
+	&lt;li&gt;Vídeos&lt;/li&gt;
+	&lt;li&gt;Sistematização&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Aquisição
+&lt;ul&gt;
+	&lt;li&gt;obtenção de conhecimento fora da organização&lt;/li&gt;
+	&lt;li&gt;é complementar à captura&lt;/li&gt;
+	&lt;li&gt;olha para fora&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Armazenamento
+&lt;ul&gt;
+	&lt;li&gt;Bases&lt;/li&gt;
+	&lt;li&gt;Sistemas&lt;/li&gt;
+	&lt;li&gt;Repositórios&lt;/li&gt;
+	&lt;li&gt;Documentação&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Compartilhamento
+Treinamentos
+Mentorias
+Comunidades
+Ferramentas
+&lt;/li&gt;
+	&lt;li&gt;Aplicação
+&lt;ul&gt;
+	&lt;li&gt;uso efetivo do conhecimento disponível&lt;/li&gt;
+	&lt;li&gt;O conhecimento aplicado precisa ser atualizado constantemente&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Avaliação
+&lt;ul&gt;
+	&lt;li&gt;Alguns indicadores possíveis: &lt;ul&gt; &lt;li&gt;Redução&lt;/li&gt; &lt;li&gt;Aumento&lt;/li&gt; &lt;li&gt;Nível&lt;/li&gt; &lt;li&gt;Quantidade&lt;/li&gt; &lt;li&gt;Tempo&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
 &lt;/ol&gt;</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G120" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="121">
-      <c r="A121" t="n">
-        <v>123</v>
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -4865,14 +4966,26 @@
       <c r="E121" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;Organizacionais&lt;/li&gt;
-	&lt;li&gt;Culturais&lt;/li&gt;
-	&lt;li&gt;Tecnológicas&lt;/li&gt;
+	&lt;li&gt;Organizacionais
+&lt;ul&gt;
+	&lt;li&gt;Alguns exemplos: &lt;ul&gt; &lt;li&gt;Hierarquias rígidas&lt;/li&gt; &lt;li&gt;Falta de tempo e recursos&lt;/li&gt; &lt;li&gt;Falta de processos formais de GC&lt;/li&gt; &lt;li&gt;Fragmentação departamental&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Culturais
+&lt;ul&gt;
+	&lt;li&gt;mais frequentes: &lt;ul&gt; &lt;li&gt;Resistência à mudança&lt;/li&gt; &lt;li&gt;Medo da exposição ou da obsolescência&lt;/li&gt; &lt;li&gt;Falta de confiança&lt;/li&gt; &lt;li&gt;Individualismo&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Tecnológicas
+&lt;ul&gt;
+	&lt;li&gt;mais comuns: &lt;ul&gt; &lt;li&gt;Falta de sistemas integrados&lt;/li&gt; &lt;li&gt;Baixa usabilidade&lt;/li&gt; &lt;li&gt;Falta de treinamento&lt;/li&gt; &lt;li&gt;Problemas de segurança da informação&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G121" t="n">
         <v>2</v>
@@ -4916,8 +5029,10 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" t="n">
-        <v>125</v>
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -4931,22 +5046,47 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>condições capacitadoras que sustentam "Ba" (espaço compartilhado onde ocorre a criação do conhecimento)</t>
+          <t>condições capacitadoras que sustentam o "Ba" (espaço compartilhado onde ocorre a criação do conhecimento)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;Intenção (Intentionality)&lt;/li&gt;
-	&lt;li&gt;Autonomia&lt;/li&gt;
-	&lt;li&gt;Flutuação e Caos Criativo&lt;/li&gt;
-	&lt;li&gt;Redundância&lt;/li&gt;
-	&lt;li&gt;Variedade de Requisitos (Variety of Requisite)&lt;/li&gt;
+	&lt;li&gt;Intenção (Intentionality)
+&lt;ul&gt;
+	&lt;li&gt;propósito organizacional claro e compartilhado&lt;/li&gt;
+	&lt;li&gt;orienta os esforços de geração e uso do conhecimento&lt;/li&gt;
+	&lt;li&gt;liderança tem papel central&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Autonomia
+&lt;ul&gt;
+	&lt;li&gt;permitir que os indivíduos se apropriem do conhecimento que produzem&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Flutuação e Caos Criativo
+&lt;ul&gt;
+	&lt;li&gt;certo grau de instabilidade, ambiguidade ou desafio pode estimular a criação de novas ideias&lt;/li&gt;
+	&lt;li&gt;Mudanças, crises ou dilemas geram oportunidades de inovação&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Redundância
+&lt;ul&gt;
+	&lt;li&gt;sobreposição de informações, funções e responsabilidades&lt;/li&gt;
+	&lt;li&gt;previne a perda de saberes em caso de desligamentos ou mudanças&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Variedade de Requisitos (Variety of Requisite)
+&lt;ul&gt;
+	&lt;li&gt;diversidade de perspectivas, linguagens e experiências&lt;/li&gt;
+	&lt;li&gt;Equipes multidisciplinares, com backgrounds diferentes, são mais propensas à inovação&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F123" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G123" t="n">
         <v>2</v>
@@ -5064,8 +5204,10 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="n">
-        <v>129</v>
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -5085,15 +5227,37 @@
       <c r="E127" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;Big Data&lt;/li&gt;
-	&lt;li&gt;Business Intelligence (BI)&lt;/li&gt;
-	&lt;li&gt;Machine Learning (ML)&lt;/li&gt;
-	&lt;li&gt;Inteligência Artificial (IA)&lt;/li&gt;
+	&lt;li&gt;Big Data
+&lt;ul&gt;
+	&lt;li&gt;grandes volumes de dados&lt;/li&gt;
+	&lt;li&gt;volume, variedade e velocidade&lt;/li&gt;
+	&lt;li&gt;No contexto da GC, o Big Data permite &lt;ul&gt; &lt;li&gt;Capturar&lt;/li&gt; &lt;li&gt;Detectar&lt;/li&gt; &lt;li&gt;Identificar&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Business Intelligence (BI)
+&lt;ul&gt;
+	&lt;li&gt;transformam dados brutos em informações úteis&lt;/li&gt;
+	&lt;li&gt;No contexto da GC, o BI: &lt;ul&gt; &lt;li&gt;Organiza&lt;/li&gt; &lt;li&gt;Apoia&lt;/li&gt; &lt;li&gt;Ajuda&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Machine Learning (ML)
+&lt;ul&gt;
+	&lt;li&gt;permite que os sistemas aprendam automaticamente com os dados&lt;/li&gt;
+	&lt;li&gt;Na GC, o ML pode: &lt;ul&gt; &lt;li&gt;Sugerir&lt;/li&gt; &lt;li&gt;Classificar&lt;/li&gt; &lt;li&gt;Detectar&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
+	&lt;li&gt;Inteligência Artificial (IA)
+&lt;ul&gt;
+	&lt;li&gt;aplicação mais abrangente&lt;/li&gt;
+	&lt;li&gt;uso de algoritmos para simular processos cognitivos humanos&lt;/li&gt;
+	&lt;li&gt;Dentro da GC, a IA: &lt;ul&gt; &lt;li&gt;Alimenta&lt;/li&gt; &lt;li&gt;Automatiza&lt;/li&gt; &lt;li&gt;Suporta&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F127" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G127" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
:up: algumas questões cadastradas - questoes extras - cebraspe
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -855,9 +855,9 @@
 	&lt;li&gt;Sistema de duas gavetas;&lt;/li&gt;
 	&lt;li&gt;Sistema dos máximos-mínimos;
 &lt;ul&gt;
-	&lt;li&gt;E min = ER + dt &lt;ul&gt; &lt;li&gt;d = consumo médio&lt;/li&gt; &lt;li&gt;t = tempo de espera médio, em dias, para reposição do material&lt;/li&gt; &lt;li&gt;ER = estoque de reserva ou de segurança&lt;/li&gt; &lt;/ul&gt; &lt;/li&gt;
-	&lt;li&gt;Emin = Emin + Lote de compra.&lt;/li&gt;
-	&lt;li&gt;ponto de ressuprimento ou ponto de pedido: &lt;ul&gt; &lt;li&gt;PR = (C X TR) + ES, onde &lt;ul&gt; &lt;li&gt;C = consumo médio do item&lt;/li&gt; &lt;li&gt;TR = tempo de reposição&lt;/li&gt; &lt;li&gt;ES = estoque mínimo ou de segurança&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;E&lt;sub&gt;min&lt;/sub&gt; = ER + dt &lt;ul&gt; &lt;li&gt;d = consumo médio&lt;/li&gt; &lt;li&gt;t = tempo de espera médio, em dias, para reposição do material&lt;/li&gt; &lt;li&gt;ER = estoque de reserva ou de segurança&lt;/li&gt; &lt;/ul&gt; &lt;/li&gt;
+	&lt;li&gt;E&lt;sub&gt;max&lt;/sub&gt; = E&lt;sub&gt;min&lt;/sub&gt; + Lote de compra.&lt;/li&gt;
+	&lt;li&gt;ponto de ressuprimento ou ponto de pedido: &lt;ul&gt; &lt;li&gt;PR = (d X TR) + RS, onde &lt;ul&gt; &lt;li&gt;d = consumo médio do item&lt;/li&gt; &lt;li&gt;TR = tempo de reposição&lt;/li&gt; &lt;li&gt;ER = estoque mínimo ou de segurança&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 &lt;/ul&gt;
 &lt;/li&gt;
 	&lt;li&gt;Sistema de reposições periódicas;
@@ -905,14 +905,13 @@
 	&lt;li&gt;FIFO&lt;/li&gt;
 	&lt;li&gt;Custo Médio&lt;/li&gt;
 	&lt;li&gt;Custo de Reposição.
+	CR= PU+ACR &lt;ul&gt; &lt;li&gt;onde:
 &lt;ul&gt;
-	&lt;li&gt;CR= PU+ACR onde:&lt;/li&gt;
-	&lt;li&gt;&lt;ul&gt;&lt;/li&gt;
-	&lt;li&gt;&lt;li&gt;CR = Custo de Reposição;&lt;/li&gt;&lt;/li&gt;
-	&lt;li&gt;&lt;li&gt;PU = Preço Unitário do material; e&lt;/li&gt;&lt;/li&gt;
-	&lt;li&gt;&lt;li&gt;ACR = Acréscimo do Custo de Reposição em porcentagem (%).&lt;/li&gt;&lt;/li&gt;
-	&lt;li&gt;&lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;CR = Custo de Reposição;&lt;/li&gt;
+	&lt;li&gt;PU = Preço Unitário do material; e&lt;/li&gt;
+	&lt;li&gt;ACR = Acréscimo do Custo de Reposição em porcentagem (%).&lt;/li&gt;
 &lt;/ul&gt;
+&lt;/li&gt; &lt;/ul&gt;
 &lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>

</xml_diff>

<commit_message>
:lady_beetle: função plano consertadas, agora recarrega todas aas configs
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G222"/>
+  <dimension ref="A1:G230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -719,7 +719,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -4323,7 +4323,7 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G106" t="n">
         <v>0</v>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G107" t="n">
         <v>0</v>
@@ -4390,7 +4390,7 @@
         <v>0</v>
       </c>
       <c r="G108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109">
@@ -8636,6 +8636,293 @@
         <v>0</v>
       </c>
     </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>226</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Gestão da Produção e Operações</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>produção intermitente</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;sistema de fabricação flexível&lt;/li&gt;
+	&lt;li&gt;organizado por lotes ou encomendas, em vez de um fluxo contínuo.&lt;/li&gt;
+	&lt;li&gt;alta variedade e baixo volume&lt;/li&gt;
+	&lt;li&gt;Produção puxada&lt;/li&gt;
+	&lt;li&gt;setup&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F223" t="n">
+        <v>0</v>
+      </c>
+      <c r="G223" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>227</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Gestão da Produção e Operações</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>cable belt (correia de cabo)</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;sistema de transporte de materiais de alta eficiência&lt;/li&gt;
+	&lt;li&gt;projetado para longas distâncias e terrenos difíceis&lt;/li&gt;
+	&lt;li&gt;separa a função de transporte da função de tração &lt;ul&gt; &lt;li&gt;cabos de aço laterais movem a correia&lt;/li&gt; &lt;li&gt;a correia apenas carrega o material&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Sinônimos/Termos Relacionados: &lt;ul&gt; &lt;li&gt;Correia transportadora de cabo&lt;/li&gt; &lt;li&gt;Cable Belt Conveyor&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F224" t="n">
+        <v>0</v>
+      </c>
+      <c r="G224" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>228</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Gestão de Projetos</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>KPIs (Key Performance Indicators) na Gestão de Projetos (Kerzner, 2009)</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;ul&gt;
+	&lt;li&gt;medem a qualidade do processo interno durante a execução&lt;/li&gt;
+	&lt;li&gt;KPIs tipicos &lt;ul&gt; &lt;li&gt;Uso da metodologia de gestão de projetos&lt;/li&gt; &lt;li&gt;Estabelecimento dos processos de controle&lt;/li&gt; &lt;li&gt;Uso de métricas intermediárias&lt;/li&gt; &lt;li&gt;Qualidade dos recursos atribuídos versus planejados&lt;/li&gt; &lt;li&gt;Envolvimento do cliente&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+</t>
+        </is>
+      </c>
+      <c r="F225" t="n">
+        <v>0</v>
+      </c>
+      <c r="G225" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>229</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Gestão de Projetos</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Planejamento Estratégico na Gestão de Projetos (Kerzner, 2015)</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;seleção e priorização de projetos &lt;ul&gt; &lt;li&gt;devem ser feitas com base na disponibilidade de recursos qualificados&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;modelos de planejamento &lt;ul&gt; &lt;li&gt;disponíveis para auxiliar na programação estratégica de recursos.&lt;/li&gt; &lt;li&gt;frequentemente chamados de modelos de planejamento agregado.&lt;/li&gt; &lt;li&gt;permitem que uma organização identifique o excesso de alocação de recursos&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Outro problema &lt;ul&gt; &lt;li&gt;determinar quais projetos exigem os melhores recursos.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Outro componente-chave &lt;ul&gt; &lt;li&gt;nível de tolerância ao risco da organização&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F226" t="n">
+        <v>0</v>
+      </c>
+      <c r="G226" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>230</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>BI (Business Intelligence)</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Dados estruturados&lt;/li&gt;
+	&lt;li&gt;Função: coletar, organizar, analisar e transformar dados em informações úteis para apoiar decisões estratégicas e operacionais.&lt;/li&gt;
+	&lt;li&gt;Exemplos: &lt;ul&gt; &lt;li&gt;Relatório de Vendas,&lt;/li&gt; &lt;li&gt;Dashboards de Desempenho,&lt;/li&gt; &lt;li&gt;Análise de Tendências de Mercado&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F227" t="n">
+        <v>0</v>
+      </c>
+      <c r="G227" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>231</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>licenciamento de patentes</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;proteção de ativos intelectuais &lt;ul&gt; &lt;li&gt;mapeamento de competências&lt;/li&gt; &lt;li&gt;proteção de PI (Propriedade Intelectual)&lt;/li&gt; &lt;li&gt;alinhamento com os objetivos de negócio&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;identificação de oportunidades de mercado&lt;/li&gt;
+	&lt;li&gt;licenciamento transforma pesquisa e desenvolvimento (P&amp;D) em ativos financeiros e parcerias estratégicas&lt;/li&gt;
+	&lt;li&gt;transferência de tecnologia&lt;/li&gt;
+	&lt;li&gt;mecanismo que coloca inovações desenvolvidas no mercado&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F228" t="n">
+        <v>0</v>
+      </c>
+      <c r="G228" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>232</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Gestão da Inovação</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Diferença entre modelos tradicionais e modelos modernos de inovação</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Modelos Lineares (Antigos): &lt;ul&gt; &lt;li&gt;Fundamentados em uma sequência lógica e rígida de etapas sucessivas.&lt;/li&gt; &lt;li&gt;Focam no fluxo unidirecional (ex: P&amp;D -&gt; Vendas).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Modelos Não Lineares (Recentes): &lt;ul&gt; &lt;li&gt;Processo interativo e dinâmico com sobreposição de fases.&lt;/li&gt; &lt;li&gt;Envolvem ciclos de feedback e colaboração entre múltiplos atores (internos e externos).&lt;/li&gt; &lt;li&gt;Referência: Manual de Oslo (OCDE).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F229" t="n">
+        <v>0</v>
+      </c>
+      <c r="G229" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>233</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Gestão de Investimentos e Risco</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Índices Financeiros</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;ul&gt;
+	&lt;li&gt;ÍNDICES DE LIQUIDEZ &lt;ul&gt; &lt;li&gt;Índice de liquidez corrente = Ativo circulante/Passivo circulante&lt;/li&gt; &lt;li&gt;Indice de liquidez seca = (Ativo circulante – Estoques)/Passivo circulante&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;ÍNDICES DE ATIVIDADE &lt;ul&gt; &lt;li&gt;Giro do estoque = Custo das mercadorias vendidas/Estoque&lt;/li&gt; &lt;li&gt;Prazo médio de recebimento = Contas a receber de clientes/Valor diário médio das vendas&lt;/li&gt; &lt;li&gt;Prazo médio de recebimento = (Contas a receber de clientes x 360)/Vendas anuais&lt;/li&gt; &lt;li&gt;Prazo médio de pagamento = Fornecedores/Valor diário médio das compras&lt;/li&gt; &lt;li&gt;Prazo médio de pagamento = (Fornecedore x 360)/Compras anuais&lt;/li&gt; &lt;li&gt;Giro do ativo total = Vendas/Ativo total&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;ÍNDICES DE ENDIVIDAMENTO &lt;ul&gt; &lt;li&gt;Índice de endividamento geral = Passivo total/Ativo total&lt;/li&gt; &lt;li&gt;Índice de cobertura de juros = Lucro antes de juros e imposto de renda/Juros&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;ÍNDICES DE RENTABILIDADE &lt;ul&gt; &lt;li&gt;Margem de lucro bruto = (Receita de vendas – Custo das mercadorias vendidas)/Receita de vendas = Lucro bruto/Receita de vendas&lt;/li&gt; &lt;li&gt;Margem de lucro operacional = Lucro operacional/Receita de vendas&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+</t>
+        </is>
+      </c>
+      <c r="F230" t="n">
+        <v>0</v>
+      </c>
+      <c r="G230" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: novo plano montado e salvo
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G230"/>
+  <dimension ref="A1:G229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7108,7 +7108,7 @@
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -7122,12 +7122,12 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Translineação</t>
+          <t>Rasuras</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>asdg</t>
+          <t>apenas fazer um traço simples na palavra</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -7139,7 +7139,7 @@
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -7153,41 +7153,10 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Rasuras</t>
+          <t>Siglas e abreviaturas</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
-        <is>
-          <t>apenas fazer um traço simples na palavra</t>
-        </is>
-      </c>
-      <c r="F179" t="n">
-        <v>0</v>
-      </c>
-      <c r="G179" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="n">
-        <v>183</v>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>Discursiva</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>Teoria Geral da Produção Textual</t>
-        </is>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>Siglas e abreviaturas</t>
-        </is>
-      </c>
-      <c r="E180" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;mencionadas pela primeira vez &lt;ul&gt; &lt;li&gt;forma por extenso, seguida da sigla entre parênteses, ou separada por hífen.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
@@ -7201,8 +7170,39 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="F179" t="n">
+        <v>0</v>
+      </c>
+      <c r="G179" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>184</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Discursiva</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Teoria Geral da Produção Textual</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Posso pular linhas?</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>A resposta é, definitivamente, NÃO!</t>
+        </is>
+      </c>
       <c r="F180" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G180" t="n">
         <v>0</v>
@@ -7210,7 +7210,7 @@
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -7224,41 +7224,10 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Posso pular linhas?</t>
+          <t>Como Utilizar Números em Provas Discursivas</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
-        <is>
-          <t>A resposta é, definitivamente, NÃO!</t>
-        </is>
-      </c>
-      <c r="F181" t="n">
-        <v>0</v>
-      </c>
-      <c r="G181" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="n">
-        <v>185</v>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>Discursiva</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>Teoria Geral da Produção Textual</t>
-        </is>
-      </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>Como Utilizar Números em Provas Discursivas</t>
-        </is>
-      </c>
-      <c r="E182" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;ul&gt;
 	&lt;li&gt;forma extensa &lt;ul&gt; &lt;li&gt;formar apenas uma palavra &lt;ul&gt; &lt;li&gt;será grafado apenas por extenso.&lt;/li&gt; &lt;li&gt;Exemplo: &lt;ul&gt; &lt;li&gt;doze,&lt;/li&gt; &lt;li&gt;vinte,&lt;/li&gt; &lt;li&gt;nove.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;formar duas ou mais palavras &lt;ul&gt; &lt;li&gt;deverá constar o número cardinal seguido do extenso entre parênteses.&lt;/li&gt; &lt;li&gt;Exemplo: &lt;ul&gt; &lt;li&gt;21 (vinte e um),&lt;/li&gt; &lt;li&gt;34 (trinta e quatro).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
@@ -7267,35 +7236,35 @@
 </t>
         </is>
       </c>
-      <c r="F182" t="n">
-        <v>0</v>
-      </c>
-      <c r="G182" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
+      <c r="F181" t="n">
+        <v>0</v>
+      </c>
+      <c r="G181" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
         <is>
           <t>186</t>
         </is>
       </c>
-      <c r="B183" t="inlineStr">
+      <c r="B182" t="inlineStr">
         <is>
           <t>Raciocínio Lógico</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr">
+      <c r="C182" t="inlineStr">
         <is>
           <t>Equivalências e Negações Lógicas</t>
         </is>
       </c>
-      <c r="D183" t="inlineStr">
+      <c r="D182" t="inlineStr">
         <is>
           <t>Equivalências lógicas</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr">
+      <c r="E182" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;Equivalência contrapositiva &lt;ul&gt; &lt;li&gt;p→q ≡ ~q→~p&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
@@ -7304,33 +7273,33 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F183" t="n">
-        <v>0</v>
-      </c>
-      <c r="G183" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="n">
+      <c r="F182" t="n">
+        <v>0</v>
+      </c>
+      <c r="G182" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
         <v>187</v>
       </c>
-      <c r="B184" t="inlineStr">
+      <c r="B183" t="inlineStr">
         <is>
           <t>Raciocínio Lógico</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr">
+      <c r="C183" t="inlineStr">
         <is>
           <t>Equivalências e Negações Lógicas</t>
         </is>
       </c>
-      <c r="D184" t="inlineStr">
+      <c r="D183" t="inlineStr">
         <is>
           <t>Negações lógicas</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr">
+      <c r="E183" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;Negação da conjunção e da disjunção inclusiva (Leis de De Morgan) &lt;ul&gt; &lt;li&gt;~(p∧q) ≡ ~p∨~q&lt;/li&gt; &lt;li&gt;~(p∨q) ≡ ~p∧~q&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
@@ -7338,35 +7307,35 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F184" t="n">
-        <v>0</v>
-      </c>
-      <c r="G184" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
+      <c r="F183" t="n">
+        <v>0</v>
+      </c>
+      <c r="G183" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
         <is>
           <t>188</t>
         </is>
       </c>
-      <c r="B185" t="inlineStr">
+      <c r="B184" t="inlineStr">
         <is>
           <t>Contabilidade Gerencial</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr">
+      <c r="C184" t="inlineStr">
         <is>
           <t>Aspectos Introdutórios</t>
         </is>
       </c>
-      <c r="D185" t="inlineStr">
+      <c r="D184" t="inlineStr">
         <is>
           <t>Definição oficial de contabilidade</t>
         </is>
       </c>
-      <c r="E185" t="inlineStr">
+      <c r="E184" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;caráter científico  (1º Congresso Brasileiro de Contabilidade/1924)&lt;ul&gt; &lt;li&gt;ciência que estuda e pratica as funções de orientação&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
@@ -7374,6 +7343,37 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="F184" t="n">
+        <v>0</v>
+      </c>
+      <c r="G184" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>189</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Escrituração</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>técnica contábil que reúne todos os documentos</t>
+        </is>
+      </c>
       <c r="F185" t="n">
         <v>0</v>
       </c>
@@ -7383,7 +7383,7 @@
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -7397,12 +7397,12 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Escrituração</t>
+          <t>objeto de estudo da contabilidade</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>técnica contábil que reúne todos os documentos</t>
+          <t>patrimônio</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -7413,8 +7413,10 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" t="n">
-        <v>190</v>
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -7428,43 +7430,10 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>objeto de estudo da contabilidade</t>
+          <t>campo de aplicação da Contabilidade</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
-        <is>
-          <t>patrimônio</t>
-        </is>
-      </c>
-      <c r="F187" t="n">
-        <v>0</v>
-      </c>
-      <c r="G187" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>191</t>
-        </is>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>Contabilidade Gerencial</t>
-        </is>
-      </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>Aspectos Introdutórios</t>
-        </is>
-      </c>
-      <c r="D188" t="inlineStr">
-        <is>
-          <t>campo de aplicação da Contabilidade</t>
-        </is>
-      </c>
-      <c r="E188" t="inlineStr">
         <is>
           <t>Aziendas &lt;ul&gt; 
 &lt;li&gt;patrimônio de uma pessoa que é gerido de maneira organizada&lt;/li&gt;
@@ -7474,6 +7443,37 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="F187" t="n">
+        <v>0</v>
+      </c>
+      <c r="G187" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>192</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>finalidade principal da ciência contábil ou objetivo</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>fornecer informações sobre a situação patrimonial e financeira</t>
+        </is>
+      </c>
       <c r="F188" t="n">
         <v>0</v>
       </c>
@@ -7483,7 +7483,7 @@
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -7497,12 +7497,15 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>finalidade principal da ciência contábil ou objetivo</t>
+          <t>usuários das demonstrações contábeis externos ou internos</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>fornecer informações sobre a situação patrimonial e financeira</t>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Usuários internos (nível estratégico) &lt;ul&gt; &lt;li&gt;Alta e Média Gerência da empresa&lt;/li&gt; &lt;li&gt;Conselho de Administração&lt;/li&gt; &lt;li&gt;Acionistas Controladores&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Usuários externos &lt;ul&gt; &lt;li&gt;Empregados&lt;/li&gt; &lt;li&gt;Investidores&lt;/li&gt; &lt;li&gt;Credores por empréstimos&lt;/li&gt; &lt;li&gt;Fornecedores&lt;/li&gt; &lt;li&gt;Clientes&lt;/li&gt; &lt;li&gt;Governo e suas agências&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -7514,7 +7517,7 @@
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -7528,15 +7531,12 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>usuários das demonstrações contábeis externos ou internos</t>
+          <t>COMITÊ DE PRONUNCIAMENTOS CONTÁBEIS - 00, Item 1.5</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>&lt;ul&gt;
-	&lt;li&gt;Usuários internos (nível estratégico) &lt;ul&gt; &lt;li&gt;Alta e Média Gerência da empresa&lt;/li&gt; &lt;li&gt;Conselho de Administração&lt;/li&gt; &lt;li&gt;Acionistas Controladores&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;Usuários externos &lt;ul&gt; &lt;li&gt;Empregados&lt;/li&gt; &lt;li&gt;Investidores&lt;/li&gt; &lt;li&gt;Credores por empréstimos&lt;/li&gt; &lt;li&gt;Fornecedores&lt;/li&gt; &lt;li&gt;Clientes&lt;/li&gt; &lt;li&gt;Governo e suas agências&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-&lt;/ul&gt;</t>
+          <t>Muitos investidores, credores por empréstimos e outros credores</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -7548,26 +7548,29 @@
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Contabilidade Gerencial</t>
+          <t>Conhecimentos Específicos</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Aspectos Introdutórios</t>
+          <t>Gestão de Estoques</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>COMITÊ DE PRONUNCIAMENTOS CONTÁBEIS - 00, Item 1.5</t>
+          <t>índice de rotatividade mensal para os produtos acabados (ou giro de estoque)</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Muitos investidores, credores por empréstimos e outros credores</t>
+          <t>&lt;ul&gt;
+	&lt;li&gt;mede a velocidade com que o estoque é vendido&lt;/li&gt;
+	&lt;li&gt;Fórmula: &lt;ul&gt; &lt;li&gt;Índice de Rotatividade = Custo de Produtos Vendidos/Custo Médio Mensal de Estoque&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F191" t="n">
@@ -7579,7 +7582,7 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -7593,14 +7596,14 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>índice de rotatividade mensal para os produtos acabados (ou giro de estoque)</t>
+          <t>Como determinar o estoque mínimo</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;mede a velocidade com que o estoque é vendido&lt;/li&gt;
-	&lt;li&gt;Fórmula: &lt;ul&gt; &lt;li&gt;Índice de Rotatividade = Custo de Produtos Vendidos/Custo Médio Mensal de Estoque&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Projeção mínima de consumo: &lt;ul&gt; &lt;li&gt;consumo histórico ou previsões de uso durante o período de reposição, considerando uma margem de segurança.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Cálculo estatístico: &lt;ul&gt; &lt;li&gt;dados históricos, médias de consumo e variação de demanda, aplicando fórmulas estatísticas para definir o nível mínimo, conforme orientações de manuais de administração de materiais (vide Manuais do Ministério da Economia/Governo Federal e autores como Chiavenato).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -7613,7 +7616,7 @@
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -7622,19 +7625,19 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Gestão de Estoques</t>
+          <t>Engenharia do Trabalho</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Como determinar o estoque mínimo</t>
+          <t>Constituição Federal de 1988, Art. 7º</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;Projeção mínima de consumo: &lt;ul&gt; &lt;li&gt;consumo histórico ou previsões de uso durante o período de reposição, considerando uma margem de segurança.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;Cálculo estatístico: &lt;ul&gt; &lt;li&gt;dados históricos, médias de consumo e variação de demanda, aplicando fórmulas estatísticas para definir o nível mínimo, conforme orientações de manuais de administração de materiais (vide Manuais do Ministério da Economia/Governo Federal e autores como Chiavenato).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;redução dos riscos inerentes ao trabalho, por meio de normas de &lt;ul&gt; &lt;li&gt;saúde&lt;/li&gt; &lt;li&gt;higiene&lt;/li&gt; &lt;li&gt;segurança.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Adicional de remuneração para as atividades penosas, insalubres ou perigosas, na forma da lei;&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -7647,7 +7650,7 @@
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -7661,44 +7664,10 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Constituição Federal de 1988, Art. 7º</t>
+          <t>Consolidação das leis do Trabalho, Capítulo V</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
-        <is>
-          <t>&lt;ul&gt;
-	&lt;li&gt;redução dos riscos inerentes ao trabalho, por meio de normas de &lt;ul&gt; &lt;li&gt;saúde&lt;/li&gt; &lt;li&gt;higiene&lt;/li&gt; &lt;li&gt;segurança.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;Adicional de remuneração para as atividades penosas, insalubres ou perigosas, na forma da lei;&lt;/li&gt;
-&lt;/ul&gt;</t>
-        </is>
-      </c>
-      <c r="F194" t="n">
-        <v>0</v>
-      </c>
-      <c r="G194" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="n">
-        <v>198</v>
-      </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>Engenharia do Trabalho</t>
-        </is>
-      </c>
-      <c r="D195" t="inlineStr">
-        <is>
-          <t>Consolidação das leis do Trabalho, Capítulo V</t>
-        </is>
-      </c>
-      <c r="E195" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;responsabilidades dos órgãos&lt;/li&gt;
@@ -7708,6 +7677,37 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="F194" t="n">
+        <v>0</v>
+      </c>
+      <c r="G194" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>199</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Autosserviço</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Acesso pelo cidadão a serviço público</t>
+        </is>
+      </c>
       <c r="F195" t="n">
         <v>0</v>
       </c>
@@ -7717,7 +7717,7 @@
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -7731,12 +7731,12 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Autosserviço</t>
+          <t>Base nacional de serviços públicos</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Acesso pelo cidadão a serviço público</t>
+          <t>Base de dados que contém as informações</t>
         </is>
       </c>
       <c r="F196" t="n">
@@ -7748,7 +7748,7 @@
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -7762,12 +7762,12 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Base nacional de serviços públicos</t>
+          <t>Dados abertos</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Base de dados que contém as informações</t>
+          <t>Dados acessíveis ao público</t>
         </is>
       </c>
       <c r="F197" t="n">
@@ -7779,7 +7779,7 @@
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -7793,12 +7793,12 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Dados abertos</t>
+          <t>Dado acessível ao público</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Dados acessíveis ao público</t>
+          <t>Qualquer dado gerado ou acumulado</t>
         </is>
       </c>
       <c r="F198" t="n">
@@ -7810,7 +7810,7 @@
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -7824,12 +7824,12 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Dado acessível ao público</t>
+          <t>Formato aberto</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Qualquer dado gerado ou acumulado</t>
+          <t>Formato de arquivo não proprietário</t>
         </is>
       </c>
       <c r="F199" t="n">
@@ -7841,7 +7841,7 @@
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -7855,12 +7855,12 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Formato aberto</t>
+          <t>Governo como plataforma</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Formato de arquivo não proprietário</t>
+          <t>Infraestrutura tecnológica que facilite</t>
         </is>
       </c>
       <c r="F200" t="n">
@@ -7872,7 +7872,7 @@
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
@@ -7886,12 +7886,12 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Governo como plataforma</t>
+          <t>Laboratório de inovação</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Infraestrutura tecnológica que facilite</t>
+          <t>Espaço aberto à participação</t>
         </is>
       </c>
       <c r="F201" t="n">
@@ -7903,7 +7903,7 @@
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -7917,12 +7917,12 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Laboratório de inovação</t>
+          <t>Plataformas de governo digital</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Espaço aberto à participação</t>
+          <t>Ferramentas digitais e serviços comuns aos órgãos</t>
         </is>
       </c>
       <c r="F202" t="n">
@@ -7934,7 +7934,7 @@
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -7948,12 +7948,12 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Plataformas de governo digital</t>
+          <t>Registros de referência</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Ferramentas digitais e serviços comuns aos órgãos</t>
+          <t>Informação íntegra e precisa</t>
         </is>
       </c>
       <c r="F203" t="n">
@@ -7965,7 +7965,7 @@
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -7979,12 +7979,12 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Registros de referência</t>
+          <t>Transparência ativa</t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Informação íntegra e precisa</t>
+          <t>Disponibilização de dados pela administração pública</t>
         </is>
       </c>
       <c r="F204" t="n">
@@ -7996,7 +7996,7 @@
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
@@ -8010,41 +8010,10 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Transparência ativa</t>
+          <t>Governo Digital</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
-        <is>
-          <t>Disponibilização de dados pela administração pública</t>
-        </is>
-      </c>
-      <c r="F205" t="n">
-        <v>0</v>
-      </c>
-      <c r="G205" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="n">
-        <v>209</v>
-      </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>Informática</t>
-        </is>
-      </c>
-      <c r="C206" t="inlineStr">
-        <is>
-          <t>Lei nº 14.129-2021</t>
-        </is>
-      </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>Governo Digital</t>
-        </is>
-      </c>
-      <c r="E206" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;a administração pública deve utilizar soluções digitais&lt;/li&gt;
@@ -8058,35 +8027,35 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F206" t="n">
-        <v>0</v>
-      </c>
-      <c r="G206" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
+      <c r="F205" t="n">
+        <v>0</v>
+      </c>
+      <c r="G205" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
         <is>
           <t>210</t>
         </is>
       </c>
-      <c r="B207" t="inlineStr">
+      <c r="B206" t="inlineStr">
         <is>
           <t>Informática</t>
         </is>
       </c>
-      <c r="C207" t="inlineStr">
+      <c r="C206" t="inlineStr">
         <is>
           <t>Lei nº 14.129-2021</t>
         </is>
       </c>
-      <c r="D207" t="inlineStr">
+      <c r="D206" t="inlineStr">
         <is>
           <t>Redes de Conhecimento</t>
         </is>
       </c>
-      <c r="E207" t="inlineStr">
+      <c r="E206" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;Criadas pelo Poder Executivo federal&lt;/li&gt;
@@ -8096,35 +8065,35 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F207" t="n">
-        <v>0</v>
-      </c>
-      <c r="G207" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
+      <c r="F206" t="n">
+        <v>0</v>
+      </c>
+      <c r="G206" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
         <is>
           <t>211</t>
         </is>
       </c>
-      <c r="B208" t="inlineStr">
+      <c r="B207" t="inlineStr">
         <is>
           <t>Informática</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr">
+      <c r="C207" t="inlineStr">
         <is>
           <t>Lei nº 14.129-2021</t>
         </is>
       </c>
-      <c r="D208" t="inlineStr">
+      <c r="D207" t="inlineStr">
         <is>
           <t>Componentes do Governo Digital</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr">
+      <c r="E207" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;Base Nacional de Serviços Públicos&lt;/li&gt;
@@ -8135,33 +8104,33 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F208" t="n">
-        <v>0</v>
-      </c>
-      <c r="G208" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="n">
+      <c r="F207" t="n">
+        <v>0</v>
+      </c>
+      <c r="G207" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
         <v>212</v>
       </c>
-      <c r="B209" t="inlineStr">
+      <c r="B208" t="inlineStr">
         <is>
           <t>Informática</t>
         </is>
       </c>
-      <c r="C209" t="inlineStr">
+      <c r="C208" t="inlineStr">
         <is>
           <t>Lei nº 14.129-2021</t>
         </is>
       </c>
-      <c r="D209" t="inlineStr">
+      <c r="D208" t="inlineStr">
         <is>
           <t>Princípios do governo digital</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr">
+      <c r="E208" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;acesso centralizado&lt;/li&gt;
@@ -8174,33 +8143,33 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F209" t="n">
-        <v>0</v>
-      </c>
-      <c r="G209" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="n">
+      <c r="F208" t="n">
+        <v>0</v>
+      </c>
+      <c r="G208" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
         <v>213</v>
       </c>
-      <c r="B210" t="inlineStr">
+      <c r="B209" t="inlineStr">
         <is>
           <t>Informática</t>
         </is>
       </c>
-      <c r="C210" t="inlineStr">
+      <c r="C209" t="inlineStr">
         <is>
           <t>Lei nº 14.129-2021</t>
         </is>
       </c>
-      <c r="D210" t="inlineStr">
+      <c r="D209" t="inlineStr">
         <is>
           <t>Base Nacional de Serviços Públicos</t>
         </is>
       </c>
-      <c r="E210" t="inlineStr">
+      <c r="E209" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;estrutura destinada a concentrar informações essenciais sobre a oferta de serviços públicos&lt;/li&gt;
@@ -8209,39 +8178,72 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F210" t="n">
-        <v>0</v>
-      </c>
-      <c r="G210" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="n">
+      <c r="F209" t="n">
+        <v>0</v>
+      </c>
+      <c r="G209" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
         <v>214</v>
       </c>
-      <c r="B211" t="inlineStr">
+      <c r="B210" t="inlineStr">
         <is>
           <t>Informática</t>
         </is>
       </c>
-      <c r="C211" t="inlineStr">
+      <c r="C210" t="inlineStr">
         <is>
           <t>Lei nº 14.129-2021</t>
         </is>
       </c>
-      <c r="D211" t="inlineStr">
+      <c r="D210" t="inlineStr">
         <is>
           <t>Plataformas de Governo Digital</t>
         </is>
       </c>
-      <c r="E211" t="inlineStr">
+      <c r="E210" t="inlineStr">
         <is>
           <t xml:space="preserve">instrumentos para os entes federativos disponibilizem seus serviços públicos
 devem oferecer, no mínimo, uma ferramenta que permita &lt;ul&gt; &lt;li&gt;a solicitação&lt;/li&gt; &lt;li&gt;e o acompanhamento dos serviços e um painel destinado ao monitoramento do desempenho&lt;/li&gt; &lt;/ul&gt;
 padrões de interoperabilidade e integrar dados entre órgãos e entidades </t>
         </is>
       </c>
+      <c r="F210" t="n">
+        <v>0</v>
+      </c>
+      <c r="G210" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Prestação Digital dos Serviços Públicos</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Os órgãos e entidades devem adotar ações para garantir eficiência, qualidade e atualização contínua &lt;ul&gt; &lt;li&gt;manter atualizadas &lt;ul&gt; &lt;li&gt;Cartas de Serviços ao Usuário&lt;/li&gt; &lt;li&gt;Base Nacional de Serviços Públicos&lt;/li&gt; &lt;li&gt;Plataformas de Governo Digital&lt;/li&gt; &lt;li&gt;informações institucionais&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;melhoria dos serviços&lt;/li&gt; &lt;li&gt;integração dos serviços&lt;/li&gt; &lt;li&gt;exigências simplificadas&lt;/li&gt; &lt;li&gt;evitar a duplicação de registros&lt;/li&gt; &lt;li&gt;dados interoperáveis&lt;/li&gt; &lt;li&gt;políticas públicas com base em dados e evidências&lt;/li&gt; &lt;/ul&gt;</t>
+        </is>
+      </c>
       <c r="F211" t="n">
         <v>0</v>
       </c>
@@ -8250,58 +8252,25 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>215</t>
-        </is>
+      <c r="A212" t="n">
+        <v>216</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Informática</t>
+          <t>Conhecimentos Específicos</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Lei nº 14.129-2021</t>
+          <t>Engenharia do Trabalho</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Prestação Digital dos Serviços Públicos</t>
+          <t>Normas Regulamentadoras do Trabalho</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
-        <is>
-          <t>Os órgãos e entidades devem adotar ações para garantir eficiência, qualidade e atualização contínua &lt;ul&gt; &lt;li&gt;manter atualizadas &lt;ul&gt; &lt;li&gt;Cartas de Serviços ao Usuário&lt;/li&gt; &lt;li&gt;Base Nacional de Serviços Públicos&lt;/li&gt; &lt;li&gt;Plataformas de Governo Digital&lt;/li&gt; &lt;li&gt;informações institucionais&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;melhoria dos serviços&lt;/li&gt; &lt;li&gt;integração dos serviços&lt;/li&gt; &lt;li&gt;exigências simplificadas&lt;/li&gt; &lt;li&gt;evitar a duplicação de registros&lt;/li&gt; &lt;li&gt;dados interoperáveis&lt;/li&gt; &lt;li&gt;políticas públicas com base em dados e evidências&lt;/li&gt; &lt;/ul&gt;</t>
-        </is>
-      </c>
-      <c r="F212" t="n">
-        <v>0</v>
-      </c>
-      <c r="G212" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="n">
-        <v>216</v>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C213" t="inlineStr">
-        <is>
-          <t>Engenharia do Trabalho</t>
-        </is>
-      </c>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>Normas Regulamentadoras do Trabalho</t>
-        </is>
-      </c>
-      <c r="E213" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;obrigações, direitos e deveres&lt;/li&gt;
@@ -8310,35 +8279,35 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F213" t="n">
-        <v>0</v>
-      </c>
-      <c r="G213" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
+      <c r="F212" t="n">
+        <v>0</v>
+      </c>
+      <c r="G212" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
         <is>
           <t>217</t>
         </is>
       </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C214" t="inlineStr">
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
         <is>
           <t>Engenharia do Trabalho</t>
         </is>
       </c>
-      <c r="D214" t="inlineStr">
+      <c r="D213" t="inlineStr">
         <is>
           <t>NR 1</t>
         </is>
       </c>
-      <c r="E214" t="inlineStr">
+      <c r="E213" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 &lt;li&gt;Disposições Gerais e Gerenciamento de Riscos Ocupacionais&lt;/li&gt;
@@ -8349,6 +8318,37 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="F213" t="n">
+        <v>0</v>
+      </c>
+      <c r="G213" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>218</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>NR 2</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Inspeção Prévia</t>
+        </is>
+      </c>
       <c r="F214" t="n">
         <v>0</v>
       </c>
@@ -8358,7 +8358,7 @@
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
@@ -8372,41 +8372,10 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>NR 2</t>
+          <t>NR 3</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
-        <is>
-          <t>Inspeção Prévia</t>
-        </is>
-      </c>
-      <c r="F215" t="n">
-        <v>0</v>
-      </c>
-      <c r="G215" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="n">
-        <v>219</v>
-      </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>Engenharia do Trabalho</t>
-        </is>
-      </c>
-      <c r="D216" t="inlineStr">
-        <is>
-          <t>NR 3</t>
-        </is>
-      </c>
-      <c r="E216" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;Embargo e Interdição&lt;/li&gt;
@@ -8416,6 +8385,40 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="F215" t="n">
+        <v>0</v>
+      </c>
+      <c r="G215" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>220</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>NR 4</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;SERVIÇOS ESPECIALIZADOS EM ENGENHARIA DE SEGURANÇA E EM MEDICINA DO TRABALHO&lt;/li&gt;
+	&lt;li&gt;Profissionais do SESMT &lt;ul&gt; &lt;li&gt;Médico do Trabalho;&lt;/li&gt; &lt;li&gt;Engenheiro de Segurança do Trabalho;&lt;/li&gt; &lt;li&gt;Técnico de Segurança do Trabalho;&lt;/li&gt; &lt;li&gt;Enfermeiro do Trabalho e&lt;/li&gt; &lt;li&gt;Auxiliar ou Técnico em Enfermagem do Trabalho.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
       <c r="F216" t="n">
         <v>0</v>
       </c>
@@ -8425,7 +8428,7 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -8439,15 +8442,12 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>NR 4</t>
+          <t>NR 5</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>&lt;ul&gt;
-	&lt;li&gt;SERVIÇOS ESPECIALIZADOS EM ENGENHARIA DE SEGURANÇA E EM MEDICINA DO TRABALHO&lt;/li&gt;
-	&lt;li&gt;Profissionais do SESMT &lt;ul&gt; &lt;li&gt;Médico do Trabalho;&lt;/li&gt; &lt;li&gt;Engenheiro de Segurança do Trabalho;&lt;/li&gt; &lt;li&gt;Técnico de Segurança do Trabalho;&lt;/li&gt; &lt;li&gt;Enfermeiro do Trabalho e&lt;/li&gt; &lt;li&gt;Auxiliar ou Técnico em Enfermagem do Trabalho.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-&lt;/ul&gt;</t>
+          <t>COMISSÃO INTERNA DE PREVENÇÃO DE ACIDENTES</t>
         </is>
       </c>
       <c r="F217" t="n">
@@ -8459,7 +8459,7 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -8473,41 +8473,10 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>NR 5</t>
+          <t>NR 6</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
-        <is>
-          <t>COMISSÃO INTERNA DE PREVENÇÃO DE ACIDENTES</t>
-        </is>
-      </c>
-      <c r="F218" t="n">
-        <v>0</v>
-      </c>
-      <c r="G218" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="n">
-        <v>222</v>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C219" t="inlineStr">
-        <is>
-          <t>Engenharia do Trabalho</t>
-        </is>
-      </c>
-      <c r="D219" t="inlineStr">
-        <is>
-          <t>NR 6</t>
-        </is>
-      </c>
-      <c r="E219" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;EQUIPAMENTO DE PROTEÇÃO INDIVIDUAL - EPI&lt;/li&gt;
@@ -8520,33 +8489,33 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F219" t="n">
-        <v>0</v>
-      </c>
-      <c r="G219" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="n">
+      <c r="F218" t="n">
+        <v>0</v>
+      </c>
+      <c r="G218" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
         <v>223</v>
       </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr">
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
         <is>
           <t>Engenharia do Trabalho</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr">
+      <c r="D219" t="inlineStr">
         <is>
           <t>NR 7</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr">
+      <c r="E219" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;PROGRAMA DE CONTROLE MÉDICO DE SAÚDE OCUPACIONAL&lt;/li&gt;
@@ -8554,35 +8523,35 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F220" t="n">
-        <v>0</v>
-      </c>
-      <c r="G220" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
+      <c r="F219" t="n">
+        <v>0</v>
+      </c>
+      <c r="G219" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
         <is>
           <t>224</t>
         </is>
       </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr">
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
         <is>
           <t>Engenharia do Trabalho</t>
         </is>
       </c>
-      <c r="D221" t="inlineStr">
+      <c r="D220" t="inlineStr">
         <is>
           <t>NR 8</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr">
+      <c r="E220" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;ul&gt;
 	&lt;li&gt;EDIFICAÇÕES&lt;/li&gt;
@@ -8591,33 +8560,33 @@
 </t>
         </is>
       </c>
-      <c r="F221" t="n">
-        <v>0</v>
-      </c>
-      <c r="G221" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="n">
+      <c r="F220" t="n">
+        <v>0</v>
+      </c>
+      <c r="G220" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
         <v>225</v>
       </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr">
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
         <is>
           <t>Engenharia do Trabalho</t>
         </is>
       </c>
-      <c r="D222" t="inlineStr">
+      <c r="D221" t="inlineStr">
         <is>
           <t>NR 9</t>
         </is>
       </c>
-      <c r="E222" t="inlineStr">
+      <c r="E221" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;AVALIAÇÃO E CONTROLE DAS EXPOSIÇÕES OCUPACIONAIS A AGENTES FÍSICOS, QUÍMICOS E BIOLÓGICOS&lt;/li&gt;
@@ -8629,33 +8598,33 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F222" t="n">
-        <v>0</v>
-      </c>
-      <c r="G222" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="n">
+      <c r="F221" t="n">
+        <v>0</v>
+      </c>
+      <c r="G221" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
         <v>226</v>
       </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr">
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
         <is>
           <t>Gestão da Produção e Operações</t>
         </is>
       </c>
-      <c r="D223" t="inlineStr">
+      <c r="D222" t="inlineStr">
         <is>
           <t>produção intermitente</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr">
+      <c r="E222" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;sistema de fabricação flexível&lt;/li&gt;
@@ -8666,33 +8635,33 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F223" t="n">
-        <v>0</v>
-      </c>
-      <c r="G223" t="n">
+      <c r="F222" t="n">
+        <v>0</v>
+      </c>
+      <c r="G222" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="224">
-      <c r="A224" t="n">
+    <row r="223">
+      <c r="A223" t="n">
         <v>227</v>
       </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C224" t="inlineStr">
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
         <is>
           <t>Gestão da Produção e Operações</t>
         </is>
       </c>
-      <c r="D224" t="inlineStr">
+      <c r="D223" t="inlineStr">
         <is>
           <t>cable belt (correia de cabo)</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr">
+      <c r="E223" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;sistema de transporte de materiais de alta eficiência&lt;/li&gt;
@@ -8702,33 +8671,33 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F224" t="n">
-        <v>0</v>
-      </c>
-      <c r="G224" t="n">
+      <c r="F223" t="n">
+        <v>0</v>
+      </c>
+      <c r="G223" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="225">
-      <c r="A225" t="n">
+    <row r="224">
+      <c r="A224" t="n">
         <v>228</v>
       </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C225" t="inlineStr">
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
         <is>
           <t>Gestão de Projetos</t>
         </is>
       </c>
-      <c r="D225" t="inlineStr">
+      <c r="D224" t="inlineStr">
         <is>
           <t>KPIs (Key Performance Indicators) na Gestão de Projetos (Kerzner, 2009)</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr">
+      <c r="E224" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;ul&gt;
 	&lt;li&gt;medem a qualidade do processo interno durante a execução&lt;/li&gt;
@@ -8737,33 +8706,33 @@
 </t>
         </is>
       </c>
-      <c r="F225" t="n">
-        <v>0</v>
-      </c>
-      <c r="G225" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="n">
+      <c r="F224" t="n">
+        <v>0</v>
+      </c>
+      <c r="G224" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
         <v>229</v>
       </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C226" t="inlineStr">
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
         <is>
           <t>Gestão de Projetos</t>
         </is>
       </c>
-      <c r="D226" t="inlineStr">
+      <c r="D225" t="inlineStr">
         <is>
           <t>Planejamento Estratégico na Gestão de Projetos (Kerzner, 2015)</t>
         </is>
       </c>
-      <c r="E226" t="inlineStr">
+      <c r="E225" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;seleção e priorização de projetos &lt;ul&gt; &lt;li&gt;devem ser feitas com base na disponibilidade de recursos qualificados&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
@@ -8773,33 +8742,33 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F226" t="n">
-        <v>0</v>
-      </c>
-      <c r="G226" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="n">
+      <c r="F225" t="n">
+        <v>0</v>
+      </c>
+      <c r="G225" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
         <v>230</v>
       </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr">
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
         <is>
           <t>Gestão da Tecnologia</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr">
+      <c r="D226" t="inlineStr">
         <is>
           <t>BI (Business Intelligence)</t>
         </is>
       </c>
-      <c r="E227" t="inlineStr">
+      <c r="E226" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;Dados estruturados&lt;/li&gt;
@@ -8808,33 +8777,33 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
-      <c r="F227" t="n">
-        <v>0</v>
-      </c>
-      <c r="G227" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="n">
+      <c r="F226" t="n">
+        <v>0</v>
+      </c>
+      <c r="G226" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
         <v>231</v>
       </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
         <is>
           <t>Gestão da Tecnologia</t>
         </is>
       </c>
-      <c r="D228" t="inlineStr">
+      <c r="D227" t="inlineStr">
         <is>
           <t>licenciamento de patentes</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr">
+      <c r="E227" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;proteção de ativos intelectuais &lt;ul&gt; &lt;li&gt;mapeamento de competências&lt;/li&gt; &lt;li&gt;proteção de PI (Propriedade Intelectual)&lt;/li&gt; &lt;li&gt;alinhamento com os objetivos de negócio&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
@@ -8845,6 +8814,40 @@
 &lt;/ul&gt;</t>
         </is>
       </c>
+      <c r="F227" t="n">
+        <v>0</v>
+      </c>
+      <c r="G227" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>232</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Gestão da Inovação</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Diferença entre modelos tradicionais e modelos modernos de inovação</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Modelos Lineares (Antigos): &lt;ul&gt; &lt;li&gt;Fundamentados em uma sequência lógica e rígida de etapas sucessivas.&lt;/li&gt; &lt;li&gt;Focam no fluxo unidirecional (ex: P&amp;D -&gt; Vendas).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Modelos Não Lineares (Recentes): &lt;ul&gt; &lt;li&gt;Processo interativo e dinâmico com sobreposição de fases.&lt;/li&gt; &lt;li&gt;Envolvem ciclos de feedback e colaboração entre múltiplos atores (internos e externos).&lt;/li&gt; &lt;li&gt;Referência: Manual de Oslo (OCDE).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
       <c r="F228" t="n">
         <v>0</v>
       </c>
@@ -8854,7 +8857,7 @@
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
@@ -8863,49 +8866,15 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Gestão da Inovação</t>
+          <t>Gestão de Investimentos e Risco</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Diferença entre modelos tradicionais e modelos modernos de inovação</t>
+          <t>Índices Financeiros</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
-        <is>
-          <t>&lt;ul&gt;
-	&lt;li&gt;Modelos Lineares (Antigos): &lt;ul&gt; &lt;li&gt;Fundamentados em uma sequência lógica e rígida de etapas sucessivas.&lt;/li&gt; &lt;li&gt;Focam no fluxo unidirecional (ex: P&amp;D -&gt; Vendas).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;Modelos Não Lineares (Recentes): &lt;ul&gt; &lt;li&gt;Processo interativo e dinâmico com sobreposição de fases.&lt;/li&gt; &lt;li&gt;Envolvem ciclos de feedback e colaboração entre múltiplos atores (internos e externos).&lt;/li&gt; &lt;li&gt;Referência: Manual de Oslo (OCDE).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-&lt;/ul&gt;</t>
-        </is>
-      </c>
-      <c r="F229" t="n">
-        <v>0</v>
-      </c>
-      <c r="G229" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="n">
-        <v>233</v>
-      </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>Conhecimentos Específicos</t>
-        </is>
-      </c>
-      <c r="C230" t="inlineStr">
-        <is>
-          <t>Gestão de Investimentos e Risco</t>
-        </is>
-      </c>
-      <c r="D230" t="inlineStr">
-        <is>
-          <t>Índices Financeiros</t>
-        </is>
-      </c>
-      <c r="E230" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;ul&gt;
 	&lt;li&gt;ÍNDICES DE LIQUIDEZ &lt;ul&gt; &lt;li&gt;Índice de liquidez corrente = Ativo circulante/Passivo circulante&lt;/li&gt; &lt;li&gt;Indice de liquidez seca = (Ativo circulante – Estoques)/Passivo circulante&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
@@ -8916,10 +8885,10 @@
 </t>
         </is>
       </c>
-      <c r="F230" t="n">
-        <v>0</v>
-      </c>
-      <c r="G230" t="n">
+      <c r="F229" t="n">
+        <v>0</v>
+      </c>
+      <c r="G229" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
:up: algumas questões cadastradas - FUB-q62
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G233"/>
+  <dimension ref="A1:G244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,7 +485,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -530,7 +530,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -719,7 +719,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -1032,7 +1032,7 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -1072,7 +1072,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -1355,7 +1355,7 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1427,7 +1427,7 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -1540,7 +1540,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -1837,7 +1837,7 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -1871,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -1984,7 +1984,7 @@
         <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44" t="n">
         <v>0</v>
@@ -2081,7 +2081,7 @@
         <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -2245,7 +2245,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G49" t="n">
         <v>0</v>
@@ -2295,7 +2295,7 @@
         <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -2531,7 +2531,7 @@
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -2617,7 +2617,7 @@
         <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -2656,7 +2656,7 @@
         <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
@@ -2799,7 +2799,7 @@
         <v>0</v>
       </c>
       <c r="G63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -2870,7 +2870,7 @@
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -2903,7 +2903,7 @@
         <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -2934,7 +2934,7 @@
         <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G68" t="n">
         <v>1</v>
@@ -3034,7 +3034,7 @@
         <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="71">
@@ -3175,7 +3175,7 @@
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75">
@@ -3251,7 +3251,7 @@
         <v>0</v>
       </c>
       <c r="G76" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77">
@@ -3288,7 +3288,7 @@
         <v>0</v>
       </c>
       <c r="G77" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78">
@@ -3360,7 +3360,7 @@
         <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80">
@@ -3428,7 +3428,7 @@
         <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
@@ -4466,7 +4466,7 @@
         <v>2</v>
       </c>
       <c r="G110" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111">
@@ -8425,7 +8425,7 @@
         <v>0</v>
       </c>
       <c r="G216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217">
@@ -9040,6 +9040,399 @@
         <v>0</v>
       </c>
     </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>238</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Hierarquia na Aquisição de Tecnologia</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;1º Requisitos de Negócio: Consulta ao Gestor da Área (o que precisa ser feito).&lt;/li&gt;
+	&lt;li&gt;2º Especificações Técnicas: Descrição da Engenharia/TI (como será feito tecnicamente).&lt;/li&gt;
+	&lt;li&gt;Alinhamento: A definição do negócio deve preceder a definição técnica para garantir que a tecnologia sirva ao processo.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F234" t="n">
+        <v>0</v>
+      </c>
+      <c r="G234" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>239</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Processos Decisórios</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Critérios de Decisão no AHP</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Devem ser completos, operacionais e NÃO REDUNDANTES&lt;/li&gt;
+	&lt;li&gt;Hierarquia em níveis (Objetivo -&gt; Critérios -&gt; Subcritérios -&gt; Alternativas) com comparações paridárias (Matriz de Saaty).&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F235" t="n">
+        <v>0</v>
+      </c>
+      <c r="G235" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>240</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Tendências e Tecnologias em Gestão da Informação</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Computação em Nuvem (Cloud Computing)&lt;/li&gt;
+	&lt;li&gt;SaaS (Software as a Service)&lt;/li&gt;
+	&lt;li&gt;Plataformas Móveis Digitais&lt;/li&gt;
+	&lt;li&gt;Impacto &lt;ul&gt; &lt;li&gt;agilidade&lt;/li&gt; &lt;li&gt;custos&lt;/li&gt; &lt;li&gt;modelo de negócio&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F236" t="n">
+        <v>0</v>
+      </c>
+      <c r="G236" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>241</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Gestão da Inovação</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>EDI (Electronic Data Interchange)</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Troca eletrônica de documentos comerciais entre sistemas em um formato padrão (sem papel).&lt;/li&gt;
+	&lt;li&gt;Automatiza o envio de pedidos, faturas e avisos de expedição.&lt;/li&gt;
+	&lt;li&gt;Impacto na Produção: &lt;ul&gt; &lt;li&gt;Ferramenta de integração da Cadeia de Suprimentos (SCM)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Permite orientar e monitorar o processo produtivo em relação aos pedidos, pois provê visibilidade e dados em tempo real entre os elos da cadeia.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F237" t="n">
+        <v>0</v>
+      </c>
+      <c r="G237" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>242</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Processos Decisórios</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Técnica Nominal de Grupo (TNG)</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Processo estruturado de tomada de decisão em grupo que combina geração individual de ideias com julgamento coletivo.&lt;/li&gt;
+	&lt;li&gt;Diferente do Brainstorming livre &lt;ul&gt; &lt;li&gt;tiliza votação/ranking silencioso para priorizar opções.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Quando usar &lt;ul&gt; &lt;li&gt;alguns membros dominam a discussão.&lt;/li&gt; &lt;li&gt;problemas complexos onde o conhecimento está fragmentado entre os membros.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Objetivo: Potencializar a criatividade e garantir que todas as vozes sejam pesadas igualmente na decisão final.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F238" t="n">
+        <v>0</v>
+      </c>
+      <c r="G238" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>243</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Processos Decisórios</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Delphi x Brainstorming x TNG (Técnica nominal de grupo)</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;&lt;b&gt;Delphi&lt;/b&gt;: Especialistas anônimos, não se encontram, várias rodadas.&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Brainstorming&lt;/b&gt;: Livre, foco em quantidade, pode ser caótico.&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;TNG&lt;/b&gt;: Estruturada, encontro presencial (geralmente), foco em priorização/votação.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F239" t="n">
+        <v>0</v>
+      </c>
+      <c r="G239" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>244</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Gestão Ambiental: Reativa vs. Proativa</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;&lt;b&gt;Reativa (Controle)&lt;/b&gt;: Foco no "fim de linha" (end-of-pipe). Preocupação com tratamento de efluentes e disposição de resíduos.&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Proativa (Gestão)&lt;/b&gt;: Foco na Prevenção na Fonte, Ecoeficiência e Análise de Ciclo de Vida.&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Principal Diferença&lt;/b&gt;: A proativa busca eliminar a causa da poluição no projeto/processo, enquanto a reativa foca apenas em mitigar o dano já gerado.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F240" t="n">
+        <v>1</v>
+      </c>
+      <c r="G240" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>245</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Variável Ambiental no Negócio</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Fator Crítico: Depende do grau de conscientização e comprometimento da Alta Administração.&lt;/li&gt;
+	&lt;li&gt;Base Normativa: ISO 14001 (Requisito de Liderança).&lt;/li&gt;
+	&lt;li&gt;Lógica: Sem o suporte estratégico do topo, as metas ecológicas não recebem recursos nem integração com os processos de negócio da firma.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F241" t="n">
+        <v>0</v>
+      </c>
+      <c r="G241" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>246</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Classificação de Resíduos Sólidos (NBR 10.004)</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Classe I (Perigosos): Apresentam periculosidade (inflamabilidade, corrosividade, toxicidade, etc.).&lt;/li&gt;
+	&lt;li&gt;Classe II-A (Não Inertes): Podem ter propriedades como biodegradabilidade ou solubilidade em água (não são perigosos, mas reagem).&lt;/li&gt;
+	&lt;li&gt;Classe II-B (Inertes): Não se degradam nem se solubilizam (ex: lama de minério de ferro pura, entulho).&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F242" t="n">
+        <v>0</v>
+      </c>
+      <c r="G242" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>247</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Ordem de Prioridade PNRS (Lei 12.305)</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>&lt;ol&gt;
+	&lt;li&gt;Não geração.&lt;/li&gt;
+	&lt;li&gt;Redução.&lt;/li&gt;
+	&lt;li&gt;Reutilização.&lt;/li&gt;
+	&lt;li&gt;Reciclagem.&lt;/li&gt;
+	&lt;li&gt;Compostagem.&lt;/li&gt;
+	&lt;li&gt;Recuperação energética.&lt;/li&gt;
+	&lt;li&gt;Disposição final (Rejeitos).&lt;/li&gt;
+&lt;/ol&gt;</t>
+        </is>
+      </c>
+      <c r="F243" t="n">
+        <v>0</v>
+      </c>
+      <c r="G243" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>248</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Diferença entre Estéril e Rejeito (Mineração) e Métodos de Disposição</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;&lt;b&gt;Estéril&lt;/b&gt;: Material removido para acessar a jazida. NÃO passa pelo processo de beneficiamento (é rocha/solo "bruto").&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Rejeito&lt;/b&gt;: Sobra do processo de beneficiamento (onde se separa o mineral de interesse da rocha). É o que ficava nas barragens de Mariana.&lt;/li&gt;
+	&lt;li&gt;Barragens/Diques de alteamento são o método mais comum no Brasil (baixo custo), mas são considerados menos adequados por serem mais instáveis comparados ao empilhamento a seco.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F244" t="n">
+        <v>0</v>
+      </c>
+      <c r="G244" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questões cadastradas - FUB-q93
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G244"/>
+  <dimension ref="A1:G245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9433,6 +9433,43 @@
         <v>0</v>
       </c>
     </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>249</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Cadeia de Valor (Michael Porter)</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>D&lt;ul&gt;
+	&lt;li&gt;esagregação da organização em atividades estrategicamente relevantes.&lt;/li&gt;
+	&lt;li&gt;Foco: Identificar fontes de vantagem competitiva (custo ou diferenciação).&lt;/li&gt;
+	&lt;li&gt;Margem: Diferença entre o Valor Total (o que o cliente está disposto a pagar) e o Custo Coletivo das atividades executadas.&lt;/li&gt;
+	&lt;li&gt;Atividades Primárias &lt;ul&gt; &lt;li&gt;Logística Interna&lt;/li&gt; &lt;li&gt;Operações&lt;/li&gt; &lt;li&gt;Logística Externa&lt;/li&gt; &lt;li&gt;Marketing e Vendas&lt;/li&gt; &lt;li&gt;Serviços&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Atividades de Apoio &lt;ul&gt; &lt;li&gt;Aquisição (Compras)&lt;/li&gt; &lt;li&gt;Desenvolvimento de Tecnologia&lt;/li&gt; &lt;li&gt;Gerência de Recursos Humanos&lt;/li&gt; &lt;li&gt;Infraestrutura da Empresa&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F245" t="n">
+        <v>0</v>
+      </c>
+      <c r="G245" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questões cadastradas - FUB-q120
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G245"/>
+  <dimension ref="A1:G246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9470,6 +9470,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>250</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Número suficiente para identificação</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;CPF e CNPJ &lt;ul&gt; &lt;li&gt;número suficiente para identificação&lt;/li&gt; &lt;li&gt;gratuidade da inscrição e das alterações nesses cadastros.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;CPF &lt;ul&gt; &lt;li&gt;constar em diversos cadastros e documentos emitidos&lt;/li&gt; &lt;li&gt;Se requerente não inscrito &lt;ul&gt; &lt;li&gt;próprio órgão de identificação realiza inscrição &lt;ul&gt; &lt;li&gt;Se possui integração com a base da Receita&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F246" t="n">
+        <v>0</v>
+      </c>
+      <c r="G246" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questões cadastradas - MF - AI
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G246"/>
+  <dimension ref="A1:G248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9504,6 +9504,73 @@
         <v>0</v>
       </c>
     </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>251</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Análise de Investimentos</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Relação entre TIR e VPL</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;São análises independentes.&lt;/li&gt;
+	&lt;li&gt;Um projeto pode ter a TIR maior que outro projeto e VPL menor.&lt;/li&gt;
+	&lt;li&gt;Assim como pode ter a TIR menor e o VPL maior.&lt;/li&gt;
+	&lt;li&gt;Logo, as diferenças da TIR dos dois projetos não dizem nada sobre o valor presente líquido, VPL.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F247" t="n">
+        <v>0</v>
+      </c>
+      <c r="G247" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>252</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Análise de Investimentos</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>método da TIR</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>pressupõe que o fluxo de caixa seja reinvestido com base na própria Taxa Interna de Retorno.</t>
+        </is>
+      </c>
+      <c r="F248" t="n">
+        <v>0</v>
+      </c>
+      <c r="G248" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questões respondidas e cadastradas
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G260"/>
+  <dimension ref="A1:G266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
         <v>3</v>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
         <v>4</v>
@@ -1072,7 +1072,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
@@ -1103,7 +1103,7 @@
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
@@ -3709,7 +3709,7 @@
         <v>0</v>
       </c>
       <c r="G89" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="90">
@@ -3748,7 +3748,7 @@
         <v>0</v>
       </c>
       <c r="G90" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="91">
@@ -3817,7 +3817,7 @@
         <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93">
@@ -3853,7 +3853,7 @@
         <v>0</v>
       </c>
       <c r="G93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94">
@@ -3950,7 +3950,7 @@
         <v>0</v>
       </c>
       <c r="G96" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="97">
@@ -3985,7 +3985,7 @@
         <v>1</v>
       </c>
       <c r="G97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="98">
@@ -4014,7 +4014,7 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G98" t="n">
         <v>2</v>
@@ -4670,7 +4670,7 @@
         <v>5</v>
       </c>
       <c r="G115" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="116">
@@ -4708,12 +4708,14 @@
         <v>5</v>
       </c>
       <c r="G116" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="n">
-        <v>119</v>
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -4733,16 +4735,15 @@
       <c r="E117" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;Dados Qualitativos&lt;/li&gt;
-	&lt;li&gt;Pessoas&lt;/li&gt;
-	&lt;li&gt;significados&lt;/li&gt;
-	&lt;li&gt;subjetividade&lt;/li&gt;
-	&lt;li&gt;cultura&lt;/li&gt;
+	&lt;li&gt;organização como um sistema social e simbólico&lt;/li&gt;
+	&lt;li&gt;informação é interpretada por pessoas&lt;/li&gt;
+	&lt;li&gt;com base em seus &lt;ul&gt; &lt;li&gt;contextos, experiências e valores&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;tomada de decisão considera múltiplos significados possíveis&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G117" t="n">
         <v>1</v>
@@ -4853,7 +4854,7 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G119" t="n">
         <v>1</v>
@@ -4938,7 +4939,7 @@
         <v>6</v>
       </c>
       <c r="G120" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="121">
@@ -5088,7 +5089,7 @@
         <v>2</v>
       </c>
       <c r="G123" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124">
@@ -5123,7 +5124,7 @@
         <v>0</v>
       </c>
       <c r="G124" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="125">
@@ -7711,10 +7712,10 @@
         </is>
       </c>
       <c r="F195" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G195" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="196">
@@ -7745,7 +7746,7 @@
         <v>0</v>
       </c>
       <c r="G196" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="197">
@@ -7776,7 +7777,7 @@
         <v>0</v>
       </c>
       <c r="G197" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="198">
@@ -7807,7 +7808,7 @@
         <v>0</v>
       </c>
       <c r="G198" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="199">
@@ -7838,7 +7839,7 @@
         <v>0</v>
       </c>
       <c r="G199" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="200">
@@ -7866,10 +7867,10 @@
         </is>
       </c>
       <c r="F200" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G200" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201">
@@ -7900,7 +7901,7 @@
         <v>0</v>
       </c>
       <c r="G201" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="202">
@@ -7931,7 +7932,7 @@
         <v>0</v>
       </c>
       <c r="G202" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="203">
@@ -7962,7 +7963,7 @@
         <v>0</v>
       </c>
       <c r="G203" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="204">
@@ -7993,12 +7994,14 @@
         <v>0</v>
       </c>
       <c r="G204" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="n">
-        <v>209</v>
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
@@ -8018,14 +8021,79 @@
       <c r="E205" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;a administração pública deve utilizar soluções digitais&lt;/li&gt;
-	&lt;li&gt;processos administrativos eletrônicos&lt;/li&gt;
-	&lt;li&gt;documentos e atos processuais praticados em meio digital&lt;/li&gt;
-	&lt;li&gt;realização dos atos processuais em meio eletrônico&lt;/li&gt;
-	&lt;li&gt;acesso do interessado ao processo administrativo&lt;/li&gt;
-	&lt;li&gt;formato e o armazenamento dos documentos digitais&lt;/li&gt;
-	&lt;li&gt;prestação digital dos serviços públicos&lt;/li&gt;
-	&lt;li&gt;Cada ente federado&lt;/li&gt;
+  &lt;li&gt;operação padrão digital
+    &lt;ul&gt;
+      &lt;li&gt;gestão de políticas e processos&lt;/li&gt;
+      &lt;li&gt;documentos com validade legal
+        &lt;ul&gt;
+          &lt;li&gt;assinados eletronicamente&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;atos processuais
+    &lt;ul&gt;
+      &lt;li&gt;meio digital
+        &lt;ul&gt;
+          &lt;li&gt;exceções
+            &lt;ul&gt;
+              &lt;li&gt;solicitação do usuário&lt;/li&gt;
+              &lt;li&gt;inviabilidade técnica ou indisponibilidade&lt;/li&gt;
+              &lt;li&gt;risco à celeridade&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;validade
+        &lt;ul&gt;
+          &lt;li&gt;preservados parâmetros de segurança&lt;/li&gt;
+          &lt;li&gt;não se aplica ao anonimato&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;contagem de prazo
+        &lt;ul&gt;
+          &lt;li&gt;dia e hora do recebimento&lt;/li&gt;
+          &lt;li&gt;tempestivos até as 23h59 do último dia
+            &lt;ul&gt;
+              &lt;li&gt;horário de Brasília&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;acesso e arquivamento
+    &lt;ul&gt;
+      &lt;li&gt;sistemas informatizados ou cópias&lt;/li&gt;
+      &lt;li&gt;classificação conforme a LAI&lt;/li&gt;
+      &lt;li&gt;assegurar preservação e acesso
+        &lt;ul&gt;
+          &lt;li&gt;normas arquivísticas&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;prestação digital de serviços
+    &lt;ul&gt;
+      &lt;li&gt;tecnologias acessíveis&lt;/li&gt;
+      &lt;li&gt;atendimento presencial
+        &lt;ul&gt;
+          &lt;li&gt;permanece como direito&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;preferência pelo autosserviço&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Estratégia de Governo Digital
+    &lt;ul&gt;
+      &lt;li&gt;atuação integrada e cooperativa&lt;/li&gt;
+      &lt;li&gt;entes federados podem elaborar a própria
+        &lt;ul&gt;
+          &lt;li&gt;alinhada à nacional&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -8033,7 +8101,7 @@
         <v>0</v>
       </c>
       <c r="G205" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="206">
@@ -8071,7 +8139,7 @@
         <v>0</v>
       </c>
       <c r="G206" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="207">
@@ -8110,7 +8178,7 @@
         <v>0</v>
       </c>
       <c r="G207" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="208">
@@ -8149,7 +8217,7 @@
         <v>0</v>
       </c>
       <c r="G208" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="209">
@@ -8184,7 +8252,7 @@
         <v>0</v>
       </c>
       <c r="G209" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="210">
@@ -8217,7 +8285,7 @@
         <v>0</v>
       </c>
       <c r="G210" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="211">
@@ -8250,7 +8318,7 @@
         <v>0</v>
       </c>
       <c r="G211" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="212">
@@ -9501,7 +9569,7 @@
         <v>0</v>
       </c>
       <c r="G246" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="247">
@@ -10201,6 +10269,464 @@
         <v>0</v>
       </c>
     </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>265</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Interoperabilidade de Dados entre Órgãos Públicos</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;interoperabilidade de dados
+    &lt;ul&gt;
+      &lt;li&gt;elemento central&lt;/li&gt;
+      &lt;li&gt;órgãos e entidades
+        &lt;ul&gt;
+          &lt;li&gt;administrar ferramentas&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;observar
+        &lt;ul&gt;
+          &lt;li&gt;LGPD&lt;/li&gt;
+          &lt;li&gt;restrições legais&lt;/li&gt;
+          &lt;li&gt;requisitos de segurança&lt;/li&gt;
+          &lt;li&gt;limitações tecnológicas&lt;/li&gt;
+          &lt;li&gt;custo-benefício&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;otimização
+        &lt;ul&gt;
+          &lt;li&gt;custos de acesso&lt;/li&gt;
+          &lt;li&gt;infraestruturas existentes&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;mecanismo de interoperabilidade
+    &lt;ul&gt;
+      &lt;li&gt;aprimorar gestão e fortalecer confiabilidade&lt;/li&gt;
+      &lt;li&gt;assegurar
+        &lt;ul&gt;
+          &lt;li&gt;integridade e segurança&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;viabilizar
+        &lt;ul&gt;
+          &lt;li&gt;identificação unificada&lt;/li&gt;
+          &lt;li&gt;partilha de dados&lt;/li&gt;
+          &lt;li&gt;tratamento com base no CPF&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;registros de referência
+    &lt;ul&gt;
+      &lt;li&gt;órgãos responsáveis pela publicidade&lt;/li&gt;
+      &lt;li&gt;pessoas físicas e jurídicas
+        &lt;ul&gt;
+          &lt;li&gt;verificar dados&lt;/li&gt;
+          &lt;li&gt;monitorar acessos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;criação de novas bases
+    &lt;ul&gt;
+      &lt;li&gt;apenas em caso de impossibilidade de uso das existentes
+        &lt;ul&gt;
+          &lt;li&gt;evitar redundância e promover eficiência&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F261" t="n">
+        <v>0</v>
+      </c>
+      <c r="G261" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>266</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Domicílio Eletrônico</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;comunicações, notificações e intimações por meios digitais
+    &lt;ul&gt;
+      &lt;li&gt;opção do usuário
+        &lt;ul&gt;
+          &lt;li&gt;não constitui direito se indisponível&lt;/li&gt;
+          &lt;li&gt;pode encerrar recebimento a qualquer momento&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;ente público pode utilizar ferramentas de outro ente&lt;/li&gt;
+  &lt;li&gt;requisitos das ferramentas
+    &lt;ul&gt;
+      &lt;li&gt;garantir segurança, transparência e confiabilidade&lt;/li&gt;
+      &lt;li&gt;comprovar autoria&lt;/li&gt;
+      &lt;li&gt;registrar emissão e recebimento&lt;/li&gt;
+      &lt;li&gt;passíveis de auditoria&lt;/li&gt;
+      &lt;li&gt;preservar dados
+        &lt;ul&gt;
+          &lt;li&gt;mínimo de cinco anos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;aplicabilidade
+    &lt;ul&gt;
+      &lt;li&gt;mesmo quando a legislação mencionar formas tradicionais&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F262" t="n">
+        <v>0</v>
+      </c>
+      <c r="G262" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>267</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Laboratórios de Inovação</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;instituídos pelos entes públicos
+    &lt;ul&gt;
+      &lt;li&gt;espaços voltados ao desenvolvimento e à experimentação
+        &lt;ul&gt;
+          &lt;li&gt;ideias, métodos e ferramentas&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;abertos à participação e à colaboração
+        &lt;ul&gt;
+          &lt;li&gt;sociedade, especialistas e instituições&lt;/li&gt;
+          &lt;li&gt;contribuir para
+            &lt;ul&gt;
+              &lt;li&gt;melhoria dos serviços públicos&lt;/li&gt;
+              &lt;li&gt;aprimoramento do tratamento de dados&lt;/li&gt;
+              &lt;li&gt;fortalecimento do controle social&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;diretrizes
+    &lt;ul&gt;
+      &lt;li&gt;colaboração institucional e social&lt;/li&gt;
+      &lt;li&gt;promoção e experimentação de tecnologias abertas e livres&lt;/li&gt;
+      &lt;li&gt;foco no cidadão e na sociedade&lt;/li&gt;
+      &lt;li&gt;incentivar
+        &lt;ul&gt;
+          &lt;li&gt;inovação&lt;/li&gt;
+          &lt;li&gt;apoio ao empreendedorismo inovador&lt;/li&gt;
+          &lt;li&gt;ecossistema tecnológico&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;políticas públicas orientadas por dados e evidências&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;práticas e métodos
+    &lt;ul&gt;
+      &lt;li&gt;desenvolvimento e prototipação de softwares&lt;/li&gt;
+      &lt;li&gt;métodos ágeis&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;participação e potencial criativo
+    &lt;ul&gt;
+      &lt;li&gt;servidores, estagiários e colaboradores&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;difusão de conhecimento
+    &lt;ul&gt;
+      &lt;li&gt;modernização e disseminação de práticas inovadoras&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F263" t="n">
+        <v>0</v>
+      </c>
+      <c r="G263" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>268</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Governança, Gestão de Riscos, Controle e Auditoria</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;governança, gestão de riscos, controle e auditoria
+    &lt;ul&gt;
+      &lt;li&gt;pilares essenciais&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Governança
+    &lt;ul&gt;
+      &lt;li&gt;autoridade competente deve implementar&lt;/li&gt;
+      &lt;li&gt;mecanismos devem assegurar
+        &lt;ul&gt;
+          &lt;li&gt;acompanhamento de resultados&lt;/li&gt;
+          &lt;li&gt;soluções de desempenho organizacional&lt;/li&gt;
+          &lt;li&gt;decisões fundamentadas em evidências&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Gestão de riscos e controle interno
+    &lt;ul&gt;
+      &lt;li&gt;estruturados, monitorados e aperfeiçoados&lt;/li&gt;
+      &lt;li&gt;integrados ao planejamento estratégico&lt;/li&gt;
+      &lt;li&gt;controles proporcionais aos riscos&lt;/li&gt;
+      &lt;li&gt;resultados devem apoiar
+        &lt;ul&gt;
+          &lt;li&gt;melhoria contínua&lt;/li&gt;
+          &lt;li&gt;fortalecimento da tomada de decisão&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;norteados pela proteção das liberdades civis&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Auditoria interna
+    &lt;ul&gt;
+      &lt;li&gt;agregar valor e melhorar operações&lt;/li&gt;
+      &lt;li&gt;abordagem sistemática e disciplinada&lt;/li&gt;
+      &lt;li&gt;realização independente
+        &lt;ul&gt;
+          &lt;li&gt;avaliação e consultoria&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;planejamento baseado em riscos&lt;/li&gt;
+      &lt;li&gt;apoio na prevenção e investigação de fraudes&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F264" t="n">
+        <v>0</v>
+      </c>
+      <c r="G264" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>269</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Diretrizes da Lei 14.129/2021</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Diretrizes Gerais (Princípios e Orientações)
+    &lt;ul&gt;
+      &lt;li&gt;respeito a normas existentes
+        &lt;ul&gt;
+          &lt;li&gt;LAI, LGPD e Código Tributário&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;desburocratização e modernização
+        &lt;ul&gt;
+          &lt;li&gt;serviços simples e acessíveis&lt;/li&gt;
+          &lt;li&gt;disponíveis em dispositivos móveis&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;plataforma única
+        &lt;ul&gt;
+          &lt;li&gt;acesso centralizado&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;transparência e monitoramento
+        &lt;ul&gt;
+          &lt;li&gt;controle e fiscalização social&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;linguagem clara e compreensível
+        &lt;ul&gt;
+          &lt;li&gt;dever de prestar contas à população&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;proteção de dados pessoais
+        &lt;ul&gt;
+          &lt;li&gt;diretriz obrigatória observando a LGPD&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;interoperabilidade e abertura de dados&lt;/li&gt;
+      &lt;li&gt;acessibilidade
+        &lt;ul&gt;
+          &lt;li&gt;pessoas com deficiência&lt;/li&gt;
+          &lt;li&gt;tratamento adequado aos idosos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;ações educativas
+        &lt;ul&gt;
+          &lt;li&gt;qualificação de servidores e inclusão digital&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;apoio técnico a outros entes federados&lt;/li&gt;
+      &lt;li&gt;assinaturas eletrônicas
+        &lt;ul&gt;
+          &lt;li&gt;estímulo ao uso nas interações&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;governo como plataforma
+        &lt;ul&gt;
+          &lt;li&gt;uso de dados para políticas e novos negócios&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;padrões e formatos abertos e livres
+        &lt;ul&gt;
+          &lt;li&gt;prioridade conforme o Marco Civil da Internet&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Diretrizes para Laboratórios de Inovação
+    &lt;ul&gt;
+      &lt;li&gt;colaboração institucional e com a sociedade&lt;/li&gt;
+      &lt;li&gt;promoção de tecnologias abertas e livres&lt;/li&gt;
+      &lt;li&gt;foco no cidadão e na sociedade&lt;/li&gt;
+      &lt;li&gt;incentivo à inovação e empreendedorismo inovador&lt;/li&gt;
+      &lt;li&gt;políticas públicas orientadas por dados e evidências&lt;/li&gt;
+      &lt;li&gt;participação de servidores e colaboradores&lt;/li&gt;
+      &lt;li&gt;difusão de conhecimento e modernização&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F265" t="n">
+        <v>0</v>
+      </c>
+      <c r="G265" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>270</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Análise de Investimentos</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Taxa Interna de Retorno Modificada (TIRM)</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;transporte de fluxos &lt;ul&gt; &lt;li&gt;negativos para Valor Presente &lt;ul&gt; &lt;li&gt;Taxa de Financiamento&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;positivos para Valor Futuro &lt;ul&gt; &lt;li&gt;Taxa de Reinvestimento&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;transformação do fluxo &lt;ul&gt; &lt;li&gt;torna o fluxo convencional&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;possibilidade de trabalhar com duas taxas diferentes&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F266" t="n">
+        <v>0</v>
+      </c>
+      <c r="G266" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: alguns flashcards criados - NRs
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G305"/>
+  <dimension ref="A1:G315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13277,6 +13277,1245 @@
         <v>0</v>
       </c>
     </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>313</v>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>NR 10</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Segurança em Eletricidade&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Medidas de controle e sistemas preventivos
+        &lt;ul&gt;
+          &lt;li&gt;Geração, transmissão, distribuição e consumo&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Intervenções em instalações
+        &lt;ul&gt;
+          &lt;li&gt;Análise de risco&lt;/li&gt;
+          &lt;li&gt;Esquemas unifilares atualizados&lt;/li&gt;
+          &lt;li&gt;Prontuário de Instalações Elétricas
+            &lt;ul&gt;
+              &lt;li&gt;Carga instalada superior a 75 kW&lt;/li&gt;
+              &lt;li&gt;Conteúdo mínimo
+                &lt;ul&gt;
+                  &lt;li&gt;procedimentos e instruções técnicas&lt;/li&gt;
+                  &lt;li&gt;inspeções e medições&lt;/li&gt;
+                  &lt;li&gt;especificação de EPI/EPC e ferramentas&lt;/li&gt;
+                  &lt;li&gt;comprovação de qualificação e autorização&lt;/li&gt;
+                  &lt;li&gt;testes de isolação elétrica&lt;/li&gt;
+                  &lt;li&gt;certificações em áreas classificadas&lt;/li&gt;
+                  &lt;li&gt;relatório técnico atualizado&lt;/li&gt;
+                &lt;/ul&gt;
+              &lt;/li&gt;
+              &lt;li&gt;Manutenção por profissional habilitado&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Medidas de Proteção
+        &lt;ul&gt;
+          &lt;li&gt;Coletiva (Prioritária)
+            &lt;ul&gt;
+              &lt;li&gt;Desenergização&lt;/li&gt;
+              &lt;li&gt;Tensão de segurança&lt;/li&gt;
+              &lt;li&gt;Medidas alternativas
+                &lt;ul&gt;
+                  &lt;li&gt;isolação, barreiras, sinalização e bloqueios&lt;/li&gt;
+                &lt;/ul&gt;
+              &lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;Individual
+            &lt;ul&gt;
+              &lt;li&gt;EPIs específicos&lt;/li&gt;
+              &lt;li&gt;Proibição de adornos pessoais&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Segurança em Projetos
+        &lt;ul&gt;
+          &lt;li&gt;Dispositivos de desligamento&lt;/li&gt;
+          &lt;li&gt;Espaço seguro e influências externas&lt;/li&gt;
+          &lt;li&gt;Aterramento temporário e definitivo&lt;/li&gt;
+          &lt;li&gt;Memorial descritivo&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Instalações Desenergizadas
+        &lt;ul&gt;
+          &lt;li&gt;Sequência para liberação
+            &lt;ol&gt;
+              &lt;li&gt;seccionamento&lt;/li&gt;
+              &lt;li&gt;impedimento de reenergização&lt;/li&gt;
+              &lt;li&gt;constatação da ausência de tensão&lt;/li&gt;
+              &lt;li&gt;aterramento temporário com equipotencialização&lt;/li&gt;
+              &lt;li&gt;proteção de elementos energizados&lt;/li&gt;
+              &lt;li&gt;sinalização de impedimento&lt;/li&gt;
+            &lt;/ol&gt;
+          &lt;/li&gt;
+          &lt;li&gt;Sequência para reenergização
+            &lt;ol&gt;
+              &lt;li&gt;retirada de ferramentas e equipamentos&lt;/li&gt;
+              &lt;li&gt;retirada de trabalhadores não envolvidos&lt;/li&gt;
+              &lt;li&gt;remoção do aterramento e proteções&lt;/li&gt;
+              &lt;li&gt;remoção da sinalização&lt;/li&gt;
+              &lt;li&gt;destravamento e religação&lt;/li&gt;
+            &lt;/ol&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Trabalhadores
+        &lt;ul&gt;
+          &lt;li&gt;Classificação
+            &lt;ul&gt;
+              &lt;li&gt;Qualificado (curso oficial)&lt;/li&gt;
+              &lt;li&gt;Habilitado (registro em conselho)&lt;/li&gt;
+              &lt;li&gt;Capacitado (sob supervisão)&lt;/li&gt;
+              &lt;li&gt;Autorizado (anuência formal)&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;Treinamento
+            &lt;ul&gt;
+              &lt;li&gt;Básico (40h)&lt;/li&gt;
+              &lt;li&gt;Complementar SEP/Alta Tensão (40h)&lt;/li&gt;
+              &lt;li&gt;Reciclagem bienal&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;Exame de saúde compatível&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Emergência e Sinalização
+        &lt;ul&gt;
+          &lt;li&gt;Plano de emergência e métodos de resgate&lt;/li&gt;
+          &lt;li&gt;Treinamento em primeiros socorros e combate a incêndio&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F306" t="n">
+        <v>0</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>314</v>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>NR 11</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Equipamentos de movimentação&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;resistência e segurança
+        &lt;ul&gt;
+          &lt;li&gt;indicação de carga máxima visível&lt;/li&gt;
+          &lt;li&gt;inspeção permanente
+            &lt;ul&gt;
+              &lt;li&gt;cabos, cordas, correntes e ganchos&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;operadores de equipamentos motorizados
+        &lt;ul&gt;
+          &lt;li&gt;treinamento específico&lt;/li&gt;
+          &lt;li&gt;cartão de identificação visível
+            &lt;ul&gt;
+              &lt;li&gt;validade: 1 ano&lt;/li&gt;
+              &lt;li&gt;revalidação mediante exame de saúde&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;segurança ambiental
+        &lt;ul&gt;
+          &lt;li&gt;sinal de advertência sonora (buzina)&lt;/li&gt;
+          &lt;li&gt;controle de gases tóxicos em locais fechados&lt;/li&gt;
+          &lt;li&gt;proibição de motores a combustão interna sem neutralizadores&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Transporte de sacas&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;transporte manual
+        &lt;ul&gt;
+          &lt;li&gt;distância máxima: 60m&lt;/li&gt;
+          &lt;li&gt;auxílio de ajudante em veículos&lt;/li&gt;
+          &lt;li&gt;vedado
+            &lt;ul&gt;
+              &lt;li&gt;uso de pranchas sobre vãos &gt; 1,00m&lt;/li&gt;
+              &lt;li&gt;pisos escorregadios ou molhados&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;empilhamento
+        &lt;ul&gt;
+          &lt;li&gt;limitado à resistência do piso e estabilidade&lt;/li&gt;
+          &lt;li&gt;processo manual exige escada de madeira
+            &lt;ul&gt;
+              &lt;li&gt;largura mínima: 1,00m&lt;/li&gt;
+              &lt;li&gt;patamar final: 1,00m x 1,00m&lt;/li&gt;
+              &lt;li&gt;corrimão lateral a 1,00m de altura&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Armazenamento de materiais&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;capacidade de carga do piso&lt;/li&gt;
+      &lt;li&gt;proibição de obstrução
+        &lt;ul&gt;
+          &lt;li&gt;portas e saídas de emergência&lt;/li&gt;
+          &lt;li&gt;equipamentos contra incêndio&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;afastamento de estruturas laterais
+        &lt;ul&gt;
+          &lt;li&gt;distância mínima: 0,50m&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Chapas de rochas ornamentais (Anexo I)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;inspeção e manutenção
+        &lt;ul&gt;
+          &lt;li&gt;registro em meio físico ou eletrônico&lt;/li&gt;
+          &lt;li&gt;relatório anual com ART&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;proteções e dispositivos
+        &lt;ul&gt;
+          &lt;li&gt;fueiros com sistema de trava&lt;/li&gt;
+          &lt;li&gt;ventosas
+            &lt;ul&gt;
+              &lt;li&gt;dispositivo contra ricocheteamento de mangueira&lt;/li&gt;
+              &lt;li&gt;alarme sonoro e visual para pressão&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;cavaletes
+            &lt;ul&gt;
+              &lt;li&gt;altura mínima: 1,50m&lt;/li&gt;
+              &lt;li&gt;afastamento das paredes: 0,50m&lt;/li&gt;
+              &lt;li&gt;sinalização de 0,80m entre laterais&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;operação segura
+        &lt;ul&gt;
+          &lt;li&gt;proibida permanência de pessoas entre chapas&lt;/li&gt;
+          &lt;li&gt;proibida retirada de um único lado do carro&lt;/li&gt;
+          &lt;li&gt;interrupção de circulação durante a movimentação&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;capacitação
+        &lt;ol&gt;
+          &lt;li&gt;Módulo I: Saúde e Segurança (16h)&lt;/li&gt;
+          &lt;li&gt;Módulo II: Conteúdo do Anexo I (4h)&lt;/li&gt;
+          &lt;li&gt;Módulo III: Ponte Rolante (16h)&lt;/li&gt;
+        &lt;/ol&gt;
+        &lt;ul&gt;
+          &lt;li&gt;orientação em serviço: 30 dias&lt;/li&gt;
+          &lt;li&gt;reciclagem: trienal (16h)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F307" t="n">
+        <v>0</v>
+      </c>
+      <c r="G307" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>315</v>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>NR 12</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Princípios Gerais&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;resguardar a saúde e integridade física&lt;/li&gt;
+      &lt;li&gt;fases abrangidas: projeto, utilização, fabricação e comercialização&lt;/li&gt;
+      &lt;li&gt;ordem de prioridade das medidas
+        &lt;ol&gt;
+          &lt;li&gt;proteção coletiva&lt;/li&gt;
+          &lt;li&gt;administrativas ou organização do trabalho&lt;/li&gt;
+          &lt;li&gt;proteção individual&lt;/li&gt;
+        &lt;/ol&gt;
+      &lt;/li&gt;
+      &lt;li&gt;responsabilidades do trabalhador
+        &lt;ul&gt;
+          &lt;li&gt;cumprir procedimentos operacionais&lt;/li&gt;
+          &lt;li&gt;não alterar proteções&lt;/li&gt;
+          &lt;li&gt;comunicar danos em dispositivos de segurança&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Arranjo Físico e Instalações&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;áreas de circulação demarcadas e desobstruídas&lt;/li&gt;
+      &lt;li&gt;distância mínima segura entre máquinas&lt;/li&gt;
+      &lt;li&gt;ferramentas organizadas em locais específicos&lt;/li&gt;
+      &lt;li&gt;estabilidade de máquinas estacionárias e móveis
+        &lt;ul&gt;
+          &lt;li&gt;rodízios com travas (no mínimo duas)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Instalações e Dispositivos Elétricos&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;prevenção de choques, incêndio e explosão&lt;/li&gt;
+      &lt;li&gt;aterramento obrigatório de carcaças e invólucros&lt;/li&gt;
+      &lt;li&gt;condutores com resistência mecânica e proteção contra calor/lubrificantes&lt;/li&gt;
+      &lt;li&gt;quadros de comando
+        &lt;ul&gt;
+          &lt;li&gt;porta mantida fechada&lt;/li&gt;
+          &lt;li&gt;sinalização de perigo&lt;/li&gt;
+          &lt;li&gt;identificação de circuitos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Proibições
+        &lt;ul&gt;
+          &lt;li&gt;chave geral como dispositivo de partida/parada&lt;/li&gt;
+          &lt;li&gt;chaves tipo faca&lt;/li&gt;
+          &lt;li&gt;partes energizadas expostas&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Sistemas de Segurança&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;proteção de zonas de perigo
+        &lt;ul&gt;
+          &lt;li&gt;Proteção Fixa (removível apenas com ferramentas)&lt;/li&gt;
+          &lt;li&gt;Proteção Móvel (intertravada com a estrutura)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Requisitos
+        &lt;ul&gt;
+          &lt;li&gt;categoria de segurança conforme análise de risco&lt;/li&gt;
+          &lt;li&gt;dificultar burla&lt;/li&gt;
+          &lt;li&gt;paralisação de movimentos em caso de falha&lt;/li&gt;
+          &lt;li&gt;monitoramento automático&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Dispositivos de Acionamento Bimanual
+        &lt;ul&gt;
+          &lt;li&gt;atuação síncrona (retardo máximo de 0,5 s)&lt;/li&gt;
+          &lt;li&gt;sinal de saída cessa ao desacionar qualquer controle&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Parada de Emergência&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;acesso fácil e visualização clara&lt;/li&gt;
+      &lt;li&gt;prevalece sobre todos os comandos&lt;/li&gt;
+      &lt;li&gt;retenção do acionador até desacionamento manual&lt;/li&gt;
+      &lt;li&gt;exige rearme (reset) manual após correção do evento&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Manutenção e Intervenções&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;registro em livro ou sistema informatizado&lt;/li&gt;
+      &lt;li&gt;Procedimentos LOTO (Lockout/Tagout)
+        &lt;ul&gt;
+          &lt;li&gt;isolamento e descarga de energia&lt;/li&gt;
+          &lt;li&gt;bloqueio mecânico e elétrico na posição "desligado"&lt;/li&gt;
+          &lt;li&gt;sinalização com cartão ou etiqueta&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Capacitação&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;realizada antes do início da função e sem ônus&lt;/li&gt;
+      &lt;li&gt;conteúdo programático teórico e prático&lt;/li&gt;
+      &lt;li&gt;reciclagem obrigatória em modificações significativas&lt;/li&gt;
+      &lt;li&gt;operadores de máquinas autopropelidas devem portar identificação com foto&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Sinalização e Manuais&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;inscrições em língua portuguesa e legíveis&lt;/li&gt;
+      &lt;li&gt;informações indeléveis (razão social, CNPJ, modelo, peso)&lt;/li&gt;
+      &lt;li&gt;manual deve permanecer disponível no local de trabalho&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>0</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>316</v>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>NR 13</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Gestão da integridade estrutural
+    &lt;ul&gt;
+      &lt;li&gt;objetiva garantir a segurança e saúde&lt;/li&gt;
+      &lt;li&gt;responsabilidade do empregador&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Equipamentos abrangidos
+    &lt;ul&gt;
+      &lt;li&gt;caldeiras (&gt; 60 kPa)&lt;/li&gt;
+      &lt;li&gt;vasos de pressão
+        &lt;ul&gt;
+          &lt;li&gt;produto P.V &gt; 8 ou&lt;/li&gt;
+          &lt;li&gt;fluidos classe A&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;tubulações (fluidos classe A ou B)&lt;/li&gt;
+      &lt;li&gt;tanques metálicos (&gt; 20.000 L e Ø &gt; 3m)&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Condições de risco grave e iminente
+    &lt;ul&gt;
+      &lt;li&gt;operação sem dispositivos de segurança&lt;/li&gt;
+      &lt;li&gt;atraso na inspeção de caldeiras&lt;/li&gt;
+      &lt;li&gt;falta de controle do nível de água&lt;/li&gt;
+      &lt;li&gt;inaptidão atestada em relatório&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Profissional Legalmente Habilitado (PLH)
+    &lt;ul&gt;
+      &lt;li&gt;engenheiro com competência legal&lt;/li&gt;
+      &lt;li&gt;responsável técnico por inspeções e projetos&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Caldeiras
+    &lt;ul&gt;
+      &lt;li&gt;Categorias
+        &lt;ul&gt;
+          &lt;li&gt;A (pressão ≥ 1.960 kPa)&lt;/li&gt;
+          &lt;li&gt;B (60 kPa &lt; pressão &lt; 1.960 kPa)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Itens obrigatórios
+        &lt;ul&gt;
+          &lt;li&gt;válvula de segurança&lt;/li&gt;
+          &lt;li&gt;instrumento de pressão&lt;/li&gt;
+          &lt;li&gt;sistema de alimentação independente&lt;/li&gt;
+          &lt;li&gt;controle automático de nível&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Inspeção periódica
+        &lt;ul&gt;
+          &lt;li&gt;Prazos padrão
+            &lt;ul&gt;
+              &lt;li&gt;12 meses (Cat A e B)&lt;/li&gt;
+              &lt;li&gt;24 meses (Cat A com teste de válvulas)&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;Prazos com SPIE
+            &lt;ul&gt;
+              &lt;li&gt;até 30 meses (Cat A)&lt;/li&gt;
+              &lt;li&gt;até 48 meses (Cat A com SIS)&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Vasos de Pressão
+    &lt;ul&gt;
+      &lt;li&gt;Categorização
+        &lt;ul&gt;
+          &lt;li&gt;Classe de fluido (A, B, C, D)&lt;/li&gt;
+          &lt;li&gt;Potencial de risco (Grupo 1 a 5)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Inspeção periódica
+        &lt;ul&gt;
+          &lt;li&gt;conforme tabela de prazos (1 a 10 anos)&lt;/li&gt;
+          &lt;li&gt;ampliável com inspeção baseada em risco&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Documentação obrigatória
+    &lt;ul&gt;
+      &lt;li&gt;prontuário atualizado&lt;/li&gt;
+      &lt;li&gt;registro de segurança (livro ou sistema)&lt;/li&gt;
+      &lt;li&gt;projeto de instalação e alteração&lt;/li&gt;
+      &lt;li&gt;relatórios de inspeção&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Capacitação
+    &lt;ul&gt;
+      &lt;li&gt;Operador de caldeira
+        &lt;ul&gt;
+          &lt;li&gt;pré-requisito: ensino médio&lt;/li&gt;
+          &lt;li&gt;curso (40h) e estágio supervisionado
+            &lt;ul&gt;
+              &lt;li&gt;Cat A (80h)&lt;/li&gt;
+              &lt;li&gt;Cat B (60h)&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Unidades de processo
+        &lt;ul&gt;
+          &lt;li&gt;treinamento de segurança (40h)&lt;/li&gt;
+          &lt;li&gt;estágio (300h)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F309" t="n">
+        <v>0</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>317</v>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>NR 14</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;operação com segurança
+    &lt;ul&gt;
+      &lt;li&gt;construção sólida
+        &lt;ul&gt;
+          &lt;li&gt;revestimento refratário&lt;/li&gt;
+          &lt;li&gt;calor radiante dentro dos limites&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;instalação
+        &lt;ul&gt;
+          &lt;li&gt;normas técnicas oficiais&lt;/li&gt;
+          &lt;li&gt;segurança e conforto&lt;/li&gt;
+          &lt;li&gt;evitar
+            &lt;ul&gt;
+              &lt;li&gt;acúmulo de gases nocivos e&lt;/li&gt;
+              &lt;li&gt;altas temperaturas&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;escadas e plataformas
+            &lt;ul&gt;
+              &lt;li&gt;acesso e execução segura&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;combustíveis gasosos ou líquidos
+        &lt;ul&gt;
+          &lt;li&gt;sistemas de proteção contra
+            &lt;ul&gt;
+              &lt;li&gt;explosão&lt;/li&gt;
+              &lt;li&gt;retrocesso da chama&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;chaminé
+        &lt;ul&gt;
+          &lt;li&gt;saída dos gases de combustão&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>0</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>318</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>NR 15</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Agente Físico: Ruído (Anexo 1)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Classificação: Risco físico (cor verde)&lt;/li&gt;
+      &lt;li&gt;Limites de Tolerância:
+        &lt;ul&gt;
+          &lt;li&gt;85 dB(A) &amp;rarr; 8 horas&lt;/li&gt;
+          &lt;li&gt;90 dB(A) &amp;rarr; 4 horas&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Cálculo de Dose:
+        &lt;ul&gt;
+          &lt;li&gt;Fórmula: (Exposição 1 / Limite 1) + (Exposição 2 / Limite 2)&lt;/li&gt;
+          &lt;li&gt;Se resultado &amp;gt; 1 &amp;rarr; Condição Insalubre&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Insalubridade vs. Periculosidade&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Ruído gera &lt;strong&gt;Insalubridade&lt;/strong&gt; (danos graduais), nunca periculosidade (risco imediato).&lt;/li&gt;
+      &lt;li&gt;Adicional de Insalubridade por Ruído: 20% (Grau Médio).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Eliminação do Risco&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;O EPI (abafador) tenta neutralizar o risco, mas a cessação do adicional depende de &lt;strong&gt;avaliação pericial&lt;/strong&gt;.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>0</v>
+      </c>
+      <c r="G311" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>319</v>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>NR 16</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Adicional de Periculosidade&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;valor: 30%&lt;/li&gt;
+      &lt;li&gt;incidência: salário base
+        &lt;ul&gt;
+          &lt;li&gt;sem acréscimos de prêmios ou gratificações&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;direito de opção pelo adicional de insalubridade&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Caracterização Jurídica&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;responsabilidade do empregador&lt;/li&gt;
+      &lt;li&gt;laudo técnico obrigatório
+        &lt;ul&gt;
+          &lt;li&gt;Médico do Trabalho ou Engenheiro de Segurança&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;delimitação física das áreas de risco&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Explosivos (Anexo I)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;atividades abrangidas
+        &lt;ul&gt;
+          &lt;li&gt;armazenamento e transporte&lt;/li&gt;
+          &lt;li&gt;escorva e carregamento&lt;/li&gt;
+          &lt;li&gt;detonação e verificação de falhas&lt;/li&gt;
+          &lt;li&gt;queima de materiais deteriorados&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;área de risco definida por tabelas de distância&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Inflamáveis (Anexo II)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;limites de exclusão para transporte
+        &lt;ul&gt;
+          &lt;li&gt;líquidos: até 200 litros&lt;/li&gt;
+          &lt;li&gt;gases liquefeitos: até 135 quilos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;tanques de consumo próprio não computados
+        &lt;ul&gt;
+          &lt;li&gt;originais de fábrica e suplementares certificados&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;líquido combustível: ponto de fulgor &amp;gt; 60°C e &amp;le; 93°C&lt;/li&gt;
+      &lt;li&gt;operações em postos de serviço (abastecimento)&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Segurança Pessoal ou Patrimonial (Anexo III)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;exposição a roubos ou violência física&lt;/li&gt;
+      &lt;li&gt;atividades profissionais
+        &lt;ul&gt;
+          &lt;li&gt;vigilância patrimonial e de eventos&lt;/li&gt;
+          &lt;li&gt;transporte de valores e escolta armada&lt;/li&gt;
+          &lt;li&gt;telemonitoramento&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Energia Elétrica (Anexo IV)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Alta Tensão (AT)&lt;/li&gt;
+      &lt;li&gt;Sistema Elétrico de Potência (SEP)&lt;/li&gt;
+      &lt;li&gt;Baixa Tensão
+        &lt;ul&gt;
+          &lt;li&gt;em caso de descumprimento das medidas de proteção da NR 10&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;exclusão: trabalho em extra-baixa tensão ou desenergizado&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Motocicleta (Anexo V)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;deslocamento em vias públicas&lt;/li&gt;
+      &lt;li&gt;exclusões
+        &lt;ul&gt;
+          &lt;li&gt;trajeto residência-trabalho&lt;/li&gt;
+          &lt;li&gt;vias privadas ou estradas lindeiras&lt;/li&gt;
+          &lt;li&gt;uso eventual ou por tempo reduzido&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Agentes de Trânsito (Anexo VI)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;risco de colisões e atropelamentos&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Radiações Ionizantes&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;atividades em minas, reatores e laboratórios&lt;/li&gt;
+      &lt;li&gt;exclusão: áreas com Raio X móvel para diagnóstico médico&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F312" t="n">
+        <v>0</v>
+      </c>
+      <c r="G312" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>320</v>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>NR 17</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Adaptação às características psicofisiológicas&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;conforto, segurança e saúde&lt;/li&gt;
+      &lt;li&gt;desempenho eficiente&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Avaliação das situações de trabalho&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Avaliação ergonômica preliminar (obrigatória)
+        &lt;ul&gt;
+          &lt;li&gt;identificar perigos e planejar prevenção&lt;/li&gt;
+          &lt;li&gt;registrada e integrada ao PGR&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Análise Ergonômica do Trabalho - AET (específica)
+        &lt;ul&gt;
+          &lt;li&gt;situações complexas ou falha de medidas&lt;/li&gt;
+          &lt;li&gt;sugerida pelo PCMSO ou acidentes&lt;/li&gt;
+          &lt;li&gt;relatório mantido por 20 anos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Isenção de AET (salvo exceções)
+        &lt;ul&gt;
+          &lt;li&gt;MEI, ME e EPP (graus de risco 1 e 2)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Organização do trabalho&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;considerar: normas, ritmo e aspectos cognitivos&lt;/li&gt;
+      &lt;li&gt;evitar sobrecarga muscular e posturas nocivas&lt;/li&gt;
+      &lt;li&gt;medidas de prevenção
+        &lt;ul&gt;
+          &lt;li&gt;pausas (tempo de trabalho efetivo)&lt;/li&gt;
+          &lt;li&gt;alternância de atividades&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;saída garantida para necessidades fisiológicas&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Manuseio de cargas&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;peso não pode comprometer a saúde&lt;/li&gt;
+      &lt;li&gt;redução para mulheres e menores&lt;/li&gt;
+      &lt;li&gt;alcance horizontal máximo: 60 cm&lt;/li&gt;
+      &lt;li&gt;medidas técnicas facilitadoras&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Mobiliário e Equipamentos&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;regulagens adaptáveis à antropometria&lt;/li&gt;
+      &lt;li&gt;alternância entre pé e sentado&lt;/li&gt;
+      &lt;li&gt;assentos: altura ajustável, encosto lombar e borda arredondada&lt;/li&gt;
+      &lt;li&gt;terminais de vídeo: ajuste de tela e proteção contra reflexos&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Conforto Ambiental&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Iluminação (NHO 11)
+        &lt;ul&gt;
+          &lt;li&gt;evitar ofuscamento e sombras&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Ambientes de solicitação intelectual
+        &lt;ul&gt;
+          &lt;li&gt;Ruído: até 65 dB(A)&lt;/li&gt;
+          &lt;li&gt;Temperatura: entre 18 e 25 &amp;deg;C (climatizados)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Teleatendimento (Anexo II)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;jornada máxima: 6h diárias (36h semanais)&lt;/li&gt;
+      &lt;li&gt;pausas obrigatórias
+        &lt;ul&gt;
+          &lt;li&gt;2 períodos de 10 min&lt;/li&gt;
+          &lt;li&gt;intervalo de refeição: 20 min&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;headsets individuais e higienizados&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F313" t="n">
+        <v>0</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>321</v>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>NR 18</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Indústria da construção&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;implementação de medidas de controle e sistemas preventivos&lt;/li&gt;
+      &lt;li&gt;abrange demolição, reparo, pintura, limpeza e manutenção&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;PGR (Programa de Gerenciamento de Riscos)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;obrigatória elaboração por PLH
+        &lt;ul&gt;
+          &lt;li&gt;exceção para obras até 7m e com 10 trabalhadores&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;deve conter projetos
+        &lt;ul&gt;
+          &lt;li&gt;áreas de vivência&lt;/li&gt;
+          &lt;li&gt;instalações elétricas temporárias&lt;/li&gt;
+          &lt;li&gt;sistemas de proteção coletiva e SPIQ&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;atualizado conforme a etapa da obra&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Áreas de vivência&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;condições de segurança, conforto e privacidade&lt;/li&gt;
+      &lt;li&gt;instalações sanitárias
+        &lt;ul&gt;
+          &lt;li&gt;1 conjunto (lavatório, bacia e mictório) para cada 20&lt;/li&gt;
+          &lt;li&gt;1 chuveiro para cada 10&lt;/li&gt;
+          &lt;li&gt;deslocamento máximo: 150m&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;água potável e filtrada
+        &lt;ul&gt;
+          &lt;li&gt;1 bebedouro para cada 25&lt;/li&gt;
+          &lt;li&gt;distância máxima horizontal: 100m&lt;/li&gt;
+          &lt;li&gt;distância máxima vertical: 15m&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Escavação e fundação&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;escavação com profundidade superior a 1,25m
+        &lt;ul&gt;
+          &lt;li&gt;exige projeto e liberação de PLH&lt;/li&gt;
+          &lt;li&gt;protegida com taludes ou escoramentos&lt;/li&gt;
+          &lt;li&gt;faixa de proteção de 1m livre de cargas na borda&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;tubulão escavado manualmente
+        &lt;ul&gt;
+          &lt;li&gt;profundidade máxima: 15m&lt;/li&gt;
+          &lt;li&gt;diâmetro mínimo: 0,9m&lt;/li&gt;
+          &lt;li&gt;obrigatoriamente encamisado em toda extensão&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Proteção contra quedas&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;obrigatória instalação onde houver risco&lt;/li&gt;
+      &lt;li&gt;proteção de periferia
+        &lt;ul&gt;
+          &lt;li&gt;anteparos rígidos com 1,2m de altura ou&lt;/li&gt;
+          &lt;li&gt;sistema de guarda-corpo e rodapé
+            &lt;ul&gt;
+              &lt;li&gt;travessão superior: 1,2m&lt;/li&gt;
+              &lt;li&gt;travessão intermediário: 0,7m&lt;/li&gt;
+              &lt;li&gt;rodapé: 0,15m&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Máquinas e Equipamentos&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;conformidade com NR 12&lt;/li&gt;
+      &lt;li&gt;serra circular projetada por PLH
+        &lt;ul&gt;
+          &lt;li&gt;estrutura metálica estável e coifa de proteção&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;máquinas autopropelidas acima de 4.500 kg
+        &lt;ul&gt;
+          &lt;li&gt;cabine climatizada&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Equipamentos de guindar&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;utilização conforme plano de carga&lt;/li&gt;
+      &lt;li&gt;dispositivos obrigatórios
+        &lt;ul&gt;
+          &lt;li&gt;limitador de carga e altura&lt;/li&gt;
+          &lt;li&gt;alarme sonoro&lt;/li&gt;
+          &lt;li&gt;anemômetro para indicar velocidade do vento&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Andaimes&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;projeto por PLH e fabricação por empresa habilitada&lt;/li&gt;
+      &lt;li&gt;montagem e desmontagem com uso de SPIQ&lt;/li&gt;
+      &lt;li&gt;torres de andaimes
+        &lt;ul&gt;
+          &lt;li&gt;altura máxima: 4 vezes a menor dimensão da base&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>0</v>
+      </c>
+      <c r="G314" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>322</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>NR 19</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Disposições Gerais&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;definição: substância que sofre decomposição rápida com calor e pressão&lt;/li&gt;
+      &lt;li&gt;conformidade obrigatória com o Exército Brasileiro (DFPC)&lt;/li&gt;
+      &lt;li&gt;proibida a fabricação em perímetro urbano&lt;/li&gt;
+      &lt;li&gt;PGR deve prever riscos específicos de incêndio e explosão&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Fabricação&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;exige Certificado de Conformidade do Exército&lt;/li&gt;
+      &lt;li&gt;monitoramento eletrônico permanente em áreas perigosas&lt;/li&gt;
+      &lt;li&gt;restrições de pessoal
+        &lt;ul&gt;
+          &lt;li&gt;máximo de 4 trabalhadores em locais de encartuchamento&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;infraestrutura física
+        &lt;ul&gt;
+          &lt;li&gt;paredes e tetos incombustíveis&lt;/li&gt;
+          &lt;li&gt;pisos antiestáticos e aterramento de equipamentos&lt;/li&gt;
+          &lt;li&gt;ventilação adequada&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;proibições no manuseio
+        &lt;ul&gt;
+          &lt;li&gt;ferramentas que gerem centelha ou calor por atrito&lt;/li&gt;
+          &lt;li&gt;calçados com pregos ou peças metálicas externas&lt;/li&gt;
+          &lt;li&gt;fumo ou prática de fogo&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;matérias-primas no local
+        &lt;ul&gt;
+          &lt;li&gt;quantidade máxima para 4 horas de trabalho&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Armazenamento&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;depósitos e paióis
+        &lt;ul&gt;
+          &lt;li&gt;paredes duplas com intervalo de 0,50 m (paióis permanentes)&lt;/li&gt;
+          &lt;li&gt;materiais incombustíveis e maus condutores de calor&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;gestão do espaço
+        &lt;ul&gt;
+          &lt;li&gt;ocupação máxima de 60% da área&lt;/li&gt;
+          &lt;li&gt;distância mínima de 0,70 m entre o teto e o empilhamento&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;segregação e compatibilidade
+        &lt;ul&gt;
+          &lt;li&gt;proibido armazenar explosivos com iniciadores ou pólvoras&lt;/li&gt;
+          &lt;li&gt;seguir grupos de incompatibilidade (Anexo III)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;distâncias mínimas
+        &lt;ul&gt;
+          &lt;li&gt;respeitar Tabela de Quantidades-Distâncias (Anexo II)&lt;/li&gt;
+          &lt;li&gt;distâncias podem ser reduzidas à metade em depósitos barricados&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Transporte&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;conformidade com agências reguladoras (ANTT, ANTAQ, ANAC)&lt;/li&gt;
+      &lt;li&gt;requisitos do veículo
+        &lt;ul&gt;
+          &lt;li&gt;carroceria fechada (tipo baú) ou contêiner&lt;/li&gt;
+          &lt;li&gt;sistema de rastreamento em tempo real (GPS)&lt;/li&gt;
+          &lt;li&gt;botão de pânico e bloqueio remoto de portas&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;segurança na operação
+        &lt;ul&gt;
+          &lt;li&gt;sinalização de "Explosivo" visível&lt;/li&gt;
+          &lt;li&gt;supervisão por trabalhador capacitado&lt;/li&gt;
+          &lt;li&gt;proteção contra umidade e raios solares&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Fogos de Artifício (Anexo I)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;vestimentas de algodão ou material antiestático&lt;/li&gt;
+      &lt;li&gt;manipulação de pólvora branca exige lâmina d'água de 0,10 m&lt;/li&gt;
+      &lt;li&gt;proibida a remuneração por produtividade&lt;/li&gt;
+      &lt;li&gt;proibida a mão de obra de menores de 18 anos&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>0</v>
+      </c>
+      <c r="G315" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: alguns flashcards criados - NR 24
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G315"/>
+  <dimension ref="A1:G319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14516,6 +14516,478 @@
         <v>0</v>
       </c>
     </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>323</v>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>NR 20</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Gestão de inflamáveis e combustíveis&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;extração, produção, armazenamento e transferência&lt;/li&gt;
+      &lt;li&gt;manuseio e manipulação&lt;/li&gt;
+      &lt;li&gt;abrange etapas desde o projeto até a desativação&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Definições técnicas&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;líquidos inflamáveis: ponto de fulgor &amp;le; 60&amp;deg;C&lt;/li&gt;
+      &lt;li&gt;líquidos combustíveis: ponto de fulgor &amp;gt; 60&amp;deg;C e &amp;le; 93&amp;deg;C&lt;/li&gt;
+      &lt;li&gt;gases inflamáveis: inflamam a 20&amp;deg;C e 101,3 kPa&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Classificação das instalações&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Classe I
+        &lt;ul&gt;
+          &lt;li&gt;postos de serviço&lt;/li&gt;
+          &lt;li&gt;gases: &amp;gt; 2t até 60t&lt;/li&gt;
+          &lt;li&gt;líquidos: &amp;gt; 10 m&amp;sup3; até 5.000 m&amp;sup3;&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Classe II
+        &lt;ul&gt;
+          &lt;li&gt;engarrafadoras e transporte dutoviário&lt;/li&gt;
+          &lt;li&gt;gases: &amp;gt; 60t até 600t&lt;/li&gt;
+          &lt;li&gt;líquidos: &amp;gt; 5.000 m&amp;sup3; até 50.000 m&amp;sup3;&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Classe III
+        &lt;ul&gt;
+          &lt;li&gt;refinarias, petroquímicas e usinas de etanol&lt;/li&gt;
+          &lt;li&gt;gases: &amp;gt; 600t&lt;/li&gt;
+          &lt;li&gt;líquidos: &amp;gt; 50.000 m&amp;sup3;&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Documentação e Projetos&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Prontuário da Instalação
+        &lt;ul&gt;
+          &lt;li&gt;projeto e plano de inspeção/manutenção&lt;/li&gt;
+          &lt;li&gt;análise de riscos e plano de emergência&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Análise de Riscos
+        &lt;ul&gt;
+          &lt;li&gt;Classe I: APP/APR (Análise Preliminar)&lt;/li&gt;
+          &lt;li&gt;Classe II e III: metodologias definidas por profissional habilitado&lt;/li&gt;
+          &lt;li&gt;revisão periódica ou em caso de modificações&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Segurança Operacional&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;procedimentos escritos para todas as fases
+        &lt;ul&gt;
+          &lt;li&gt;pré-operação, operação normal e emergência&lt;/li&gt;
+          &lt;li&gt;parada e pós-emergência&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;controle de fontes de ignição
+        &lt;ul&gt;
+          &lt;li&gt;aterramento e controle de eletricidade estática&lt;/li&gt;
+          &lt;li&gt;permissão de trabalho para atividades a quente&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Capacitação (Cursos)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Iniciação: trabalhadores que apenas adentram a área&lt;/li&gt;
+      &lt;li&gt;Básico, Intermediário, Avançado I e II
+        &lt;ul&gt;
+          &lt;li&gt;definidos pela classe da instalação e função&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Atualização periódica
+        &lt;ul&gt;
+          &lt;li&gt;bienal ou trienal conforme a carga horária&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Emergência&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Plano de Resposta a Emergências (PRE)&lt;/li&gt;
+      &lt;li&gt;exercícios simulados anuais obrigatórios&lt;/li&gt;
+      &lt;li&gt;comunicação de ocorrências em até 2 dias úteis&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>0</v>
+      </c>
+      <c r="G316" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>324</v>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>NR 21</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Proteção do trabalhador&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;abrigos contra intempéries&lt;/li&gt;
+      &lt;li&gt;medidas contra
+        &lt;ul&gt;
+          &lt;li&gt;insolação excessiva e calor&lt;/li&gt;
+          &lt;li&gt;frio e umidade&lt;/li&gt;
+          &lt;li&gt;ventos inconvenientes&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;profilaxia de endemias
+        &lt;ul&gt;
+          &lt;li&gt;em regiões pantanosas ou alagadiças&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Alojamento e moradia&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;condições sanitárias adequadas&lt;/li&gt;
+      &lt;li&gt;moradia familiar
+        &lt;ul&gt;
+          &lt;li&gt;vedada a modalidade coletiva&lt;/li&gt;
+          &lt;li&gt;capacidade dimensionada&lt;/li&gt;
+          &lt;li&gt;ventilação e luz direta&lt;/li&gt;
+          &lt;li&gt;estrutural
+            &lt;ul&gt;
+              &lt;li&gt;paredes caiadas&lt;/li&gt;
+              &lt;li&gt;pisos impermeáveis&lt;/li&gt;
+              &lt;li&gt;cobertura impermeável e não combustível&lt;/li&gt;
+              &lt;li&gt;portas e janelas com dispositivos de fechamento&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;compartimentos mínimos
+            &lt;ul&gt;
+              &lt;li&gt;dormitório&lt;/li&gt;
+              &lt;li&gt;cozinha&lt;/li&gt;
+              &lt;li&gt;compartimento sanitário&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;localização
+        &lt;ul&gt;
+          &lt;li&gt;local arejado e livre de vegetação&lt;/li&gt;
+          &lt;li&gt;afastamento mínimo de 50m de
+            &lt;ul&gt;
+              &lt;li&gt;depósitos de feno ou estercos&lt;/li&gt;
+              &lt;li&gt;currais, estábulos e pocilgas&lt;/li&gt;
+              &lt;li&gt;viveiros de criação&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Saneamento e Higiene&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;poço de água protegido&lt;/li&gt;
+      &lt;li&gt;fossas negras
+        &lt;ul&gt;
+          &lt;li&gt;distância do poço: 15m&lt;/li&gt;
+          &lt;li&gt;distância da casa: 10m&lt;/li&gt;
+          &lt;li&gt;posicionada à jusante do poço&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;instalações sanitárias
+        &lt;ul&gt;
+          &lt;li&gt;ventilação abundante&lt;/li&gt;
+          &lt;li&gt;proteção contra pragas e animais&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F317" t="n">
+        <v>0</v>
+      </c>
+      <c r="G317" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>325</v>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>NR 22</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Gestão e Responsabilidade&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;planejamento e desenvolvimento compatíveis com segurança&lt;/li&gt;
+      &lt;li&gt;supervisão técnica por profissional legalmente habilitado (PLH)
+        &lt;ul&gt;
+          &lt;li&gt;registro obrigatório de intervenções e ocorrências&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;interrupção de atividades em risco grave e iminente&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Gerenciamento de Riscos (GRO/PGR)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;identificação de perigos específicos
+        &lt;ul&gt;
+          &lt;li&gt;atmosferas explosivas e deficiência de oxigênio&lt;/li&gt;
+          &lt;li&gt;estabilidade de maciços e ventilação mecânica&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;ações integradas entre contratante e contratada&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Organização e Equipes&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;equipes mínimas de dois trabalhadores para atividades críticas
+        &lt;ul&gt;
+          &lt;li&gt;abatimento de choco e contenção de maciço&lt;/li&gt;
+          &lt;li&gt;perfuração e manuseio de explosivos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;exceção: atividades mecanizadas com análise de risco&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Circulação e Transporte&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Plano de Trânsito obrigatório&lt;/li&gt;
+      &lt;li&gt;transporte de trabalhadores
+        &lt;ul&gt;
+          &lt;li&gt;obrigatório para trajetos superiores a 1.000 m&lt;/li&gt;
+          &lt;li&gt;veículos projetados ou adaptados com segurança&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;vias de trânsito a céu aberto
+        &lt;ul&gt;
+          &lt;li&gt;largura: 2x a do maior veículo (pista simples) ou 3x (pista dupla)&lt;/li&gt;
+          &lt;li&gt;construção de leiras (altura = 1/2 do pneu)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;transporte vertical
+        &lt;ul&gt;
+          &lt;li&gt;dispositivos de intertravamento e frenagem de segurança&lt;/li&gt;
+          &lt;li&gt;comunicação permanente com o operador&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Equipamentos e Máquinas&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;transportadores contínuos
+        &lt;ul&gt;
+          &lt;li&gt;parada de emergência e sensores de segurança&lt;/li&gt;
+          &lt;li&gt;sinal sonoro 20 segundos antes da partida&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;máquinas autopropelidas
+        &lt;ul&gt;
+          &lt;li&gt;cabine climatizada para massa superior a 4.500 kg&lt;/li&gt;
+          &lt;li&gt;proteção contra queda de objetos e raios solares&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Mineração Subterrânea (Subsolo)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Ventilação Mecânica
+        &lt;ul&gt;
+          &lt;li&gt;suprir oxigênio (mínimo 19% em volume)&lt;/li&gt;
+          &lt;li&gt;diluir gases inflamáveis e poeiras&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;monitoramento de Metano
+        &lt;ul&gt;
+          &lt;li&gt;suspensão de atividades: &gt; 1%&lt;/li&gt;
+          &lt;li&gt;proibição de desmonte: &gt; 0,8%&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;câmaras de refúgio
+        &lt;ul&gt;
+          &lt;li&gt;distância máxima das frentes: 750 m&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Estabilidade e Maciços&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;monitoramento geomecânico e hidrogeológico&lt;/li&gt;
+      &lt;li&gt;abatimento imediato de chocos&lt;/li&gt;
+      &lt;li&gt;isolamento de áreas com blocos instáveis&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Explosivos e Desmonte&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Plano de Fogo elaborado por PLH&lt;/li&gt;
+      &lt;li&gt;atividades supervisionadas por Blaster&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Segurança em Barragens e Depósitos&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Plano de Ação de Emergência (PAEBM)&lt;/li&gt;
+      &lt;li&gt;restrição na Zona de Autossalvamento&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Condições Sanitárias&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;instalações sanitárias nas frentes de trabalho
+        &lt;ul&gt;
+          &lt;li&gt;distância máxima: 250 m&lt;/li&gt;
+          &lt;li&gt;proporção: 1 bacia/lavatório para cada 20 trabalhadores&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F318" t="n">
+        <v>0</v>
+      </c>
+      <c r="G318" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>326</v>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>NR 23</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Quinta-feira, 16 de abril de 2026, 17:52:43 (Fuso horário local).
+---
+### Resumo com lista em cascata
+· **Medidas de prevenção contra incêndios**
+    o estabelecidas para ambientes de trabalho
+    o conformidade com
+        § legislação estadual
+        § normas técnicas oficiais (complementar)
+· **Informações aos trabalhadores**
+    o utilização de equipamentos de combate
+    o procedimentos de resposta e evacuação
+    o funcionamento de dispositivos de alarme
+· **Saídas e vias de passagem**
+    o número suficiente para abandono rápido
+    o requisitos de segurança
+        § sinalização indicando a direção da saída
+        § manutenção permanente de desobstrução
+        § proibição de trancamento durante a jornada
+        § permissão de dispositivos de fácil abertura interna
+---
+### Estrutura em HTML
+```html
+&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Medidas de prevenção contra incêndios&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;estabelecidas para ambientes de trabalho&lt;/li&gt;
+      &lt;li&gt;conformidade com
+        &lt;ul&gt;
+          &lt;li&gt;legislação estadual&lt;/li&gt;
+          &lt;li&gt;normas técnicas oficiais (complementar)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Informações aos trabalhadores&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;utilização de equipamentos de combate&lt;/li&gt;
+      &lt;li&gt;procedimentos de resposta e evacuação&lt;/li&gt;
+      &lt;li&gt;funcionamento de dispositivos de alarme&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Saídas e vias de passagem&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;número suficiente para abandono rápido&lt;/li&gt;
+      &lt;li&gt;requisitos de segurança
+        &lt;ul&gt;
+          &lt;li&gt;sinalização indicando a direção da saída&lt;/li&gt;
+          &lt;li&gt;manutenção permanente de desobstrução&lt;/li&gt;
+          &lt;li&gt;proibição de trancamento durante a jornada&lt;/li&gt;
+          &lt;li&gt;permissão de dispositivos de fácil abertura interna&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;
+```</t>
+        </is>
+      </c>
+      <c r="F319" t="n">
+        <v>0</v>
+      </c>
+      <c r="G319" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: flashcards de correção de simulado criados
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G334"/>
+  <dimension ref="A1:G347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8863,11 +8863,35 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>&lt;ol&gt;
-	&lt;li&gt;Pré-Desenvolvimento &lt;ol&gt; &lt;li&gt;Planejamento do Projeto &lt;ul&gt; &lt;li&gt;são realizadas &lt;ul&gt; &lt;li&gt;brainstorming&lt;/li&gt; &lt;li&gt;visitas a feiras técnicas&lt;/li&gt; &lt;li&gt;análise de produtos da concorrência&lt;/li&gt; &lt;li&gt;pesquisa de mercado&lt;/li&gt; &lt;li&gt;elaboração das especificações do projeto&lt;/li&gt; &lt;li&gt;dentre outros&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ol&gt;&lt;/li&gt;
-	&lt;li&gt;Desenvolvimento &lt;ol&gt; &lt;li&gt;Projeto Informacional&lt;/li&gt; &lt;li&gt;Projeto Conceitual&lt;/li&gt; &lt;li&gt;Projeto Detalhado&lt;/li&gt; &lt;li&gt;Preparação da Produção&lt;/li&gt; &lt;li&gt;Lançamento do Produto&lt;/li&gt; &lt;/ol&gt;&lt;/li&gt;
-	&lt;li&gt;Pós-Desenvolvimento &lt;ol&gt; &lt;li&gt;Acompanhar Produto/Processo&lt;/li&gt; &lt;li&gt;Descontinuar Produto&lt;/li&gt; &lt;/ol&gt;&lt;/li&gt;
-&lt;/ol&gt;</t>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;I. PRÉ-DESENVOLVIMENTO&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Planejamento Estratégico (Portfólio)&lt;/li&gt;
+      &lt;li&gt;Planejamento do Projeto (Briefing e Equipe)&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;II. DESENVOLVIMENTO (Foco Técnico)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Informacional:&lt;/strong&gt; Tradução de requisitos em especificações.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Conceitual:&lt;/strong&gt; Geração de &lt;u&gt;Princípios de Solução&lt;/u&gt; (Abstração).&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Detalhado - Configuração:&lt;/strong&gt; Definição de &lt;u&gt;Arranjo Físico&lt;/u&gt; e Arquitetura.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Detalhado - Precisão:&lt;/strong&gt; Definição de &lt;u&gt;Tolerâncias&lt;/u&gt; e Ajustes (Paramétrico).&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Preparação da Produção:&lt;/strong&gt; Ferramentais e Lote Piloto.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Lançamento:&lt;/strong&gt; Vendas e Suporte.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;III. PÓS-DESENVOLVIMENTO&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Acompanhamento (Pós-venda) e Descontinuidade.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;SISTEMA DE GATES (Sinalização)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;span style="color:red;"&gt;●&lt;/span&gt; &lt;strong&gt;Vermelho (Gate):&lt;/strong&gt; Decisão Gerencial/Negócio (Go / No-Go).&lt;/li&gt;
+      &lt;li&gt;&lt;span style="color:blue;"&gt;●&lt;/span&gt; &lt;strong&gt;Azul (Revisão):&lt;/strong&gt; Verificação Técnica/Qualidade.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F227" t="n">
@@ -11187,8 +11211,10 @@
       </c>
     </row>
     <row r="276">
-      <c r="A276" t="n">
-        <v>284</v>
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>284</t>
+        </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
@@ -11197,46 +11223,39 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Gestão da Qualidade</t>
+          <t>Gestão do Conhecimento</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Tipos de Benchmarking</t>
+          <t>Benchmarking</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-  &lt;li&gt;&lt;strong&gt;Interno&lt;/strong&gt;
-    &lt;ul&gt;
-      &lt;li&gt;comparação entre unidades da mesma empresa&lt;/li&gt;
-      &lt;li&gt;foco em disseminar internamente o que já funciona&lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;&lt;strong&gt;Competitivo&lt;/strong&gt;
-    &lt;ul&gt;
-      &lt;li&gt;alvo: concorrentes diretos&lt;/li&gt;
-      &lt;li&gt;foco em &lt;strong&gt;desempenho&lt;/strong&gt; (indicadores/números)&lt;/li&gt;
-      &lt;li&gt;alta barreira de acesso e riscos legais&lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;&lt;strong&gt;Funcional&lt;/strong&gt;
-    &lt;ul&gt;
-      &lt;li&gt;alvo: empresas de setores diferentes com funções similares&lt;/li&gt;
-      &lt;li&gt;foco em &lt;strong&gt;práticas&lt;/strong&gt; (processos) e não apenas resultados
-        &lt;ul&gt;
-          &lt;li&gt;&lt;strong&gt;escolha dos parceiros&lt;/strong&gt; (colaboração)&lt;/li&gt;
-          &lt;li&gt;&lt;strong&gt;estudo detalhado do próprio processo&lt;/strong&gt;&lt;/li&gt;
-          &lt;li&gt;&lt;strong&gt;preparo da visita&lt;/strong&gt; técnica&lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;&lt;strong&gt;Genérico&lt;/strong&gt;
-    &lt;ul&gt;
-      &lt;li&gt;processos idênticos em áreas totalmente distintas&lt;/li&gt;
-      &lt;li&gt;busca por inovação disruptiva&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Conceito de Benchmarking&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Processo de aprendizado e adaptação de melhores práticas de mercado.&lt;/li&gt;
+      &lt;li&gt;Não é uma simples "cópia", mas uma análise de desempenho e adaptação à realidade local.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Categorias Principais&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Interno:&lt;/strong&gt; Comparação entre unidades da mesma organização.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Competitivo:&lt;/strong&gt; Foco em concorrentes diretos.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Funcional/Genérico:&lt;/strong&gt; Foco em processos excelentes, independente do setor de atuação.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Vantagens do Benchmarking Multissetorial&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Maior facilidade na troca de informações (não há conflito de interesses).&lt;/li&gt;
+      &lt;li&gt;Possibilidade de saltos de produtividade ao adotar soluções de indústrias mais avançadas em certas áreas.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Dica para a Prova:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Palavras como "exclusivamente", "fundamentalmente" ou "apenas no mesmo setor" costumam tornar itens de benchmarking &lt;strong&gt;errados&lt;/strong&gt;.&lt;/li&gt;
     &lt;/ul&gt;
   &lt;/li&gt;
 &lt;/ul&gt;</t>
@@ -15075,7 +15094,7 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Engenharia de Produto</t>
+          <t>Engenharia do Trabalho</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
@@ -16775,6 +16794,738 @@
         <v>0</v>
       </c>
     </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>344</v>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>ações de Gestão Ambiental Organizacional</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Gestão de Resíduos&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Segregação na fonte geradora&lt;/li&gt;
+      &lt;li&gt;Implementação de logística reversa&lt;/li&gt;
+      &lt;li&gt;Destinação para co-processamento ou reciclagem&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Eficiência Energética e Hídrica&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Sistemas de reuso de água industrial&lt;/li&gt;
+      &lt;li&gt;Uso de fontes de energia renováveis (solar, eólica)&lt;/li&gt;
+      &lt;li&gt;Substituição de equipamentos obsoletos por modelos de alta eficiência&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Estratégias de Operação&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Aplicação de Produção Mais Limpa (P+L)&lt;/li&gt;
+      &lt;li&gt;Análise do Ciclo de Vida do produto (ACV)&lt;/li&gt;
+      &lt;li&gt;Controle de emissões atmosféricas e efluentes&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Políticas Organizacionais&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Treinamento e capacitação em educação ambiental&lt;/li&gt;
+      &lt;li&gt;Gestão de transporte coletivo para redução de emissões&lt;/li&gt;
+      &lt;li&gt;Seleção de fornecedores com critérios de sustentabilidade (Compras Verdes)&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Compliance e Melhoria Contínua&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Auditorias internas de conformidade legal&lt;/li&gt;
+      &lt;li&gt;Monitoramento de indicadores de desempenho ambiental (KPIs)&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F335" t="n">
+        <v>0</v>
+      </c>
+      <c r="G335" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>345</v>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>principais termos técnicos de tipos e mudanças nas estruturas organizacionais</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Processos de Reestruturação&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Downsizing:&lt;/strong&gt; Redução do quadro de funcionários para corte de custos.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Rightsizing:&lt;/strong&gt; Redesign estratégico para o tamanho ideal da operação.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Delayering (Achatamento):&lt;/strong&gt; Eliminação de níveis hierárquicos intermediários.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Dinâmicas de Autoridade&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Span of Control (Amplitude):&lt;/strong&gt; Quantidade de pessoas sob o comando de um líder.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Unity of Command (Unidade de Comando):&lt;/strong&gt; Princípio de ter apenas um superior direto.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Empowerment:&lt;/strong&gt; Delegação de autoridade para a base (ligado à descentralização).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Modelos de Estrutura&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Functional (Funcional):&lt;/strong&gt; Foco na especialização técnica de cada setor.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Divisional (Divisional):&lt;/strong&gt; Foco em resultados por unidades (produto/mercado).&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Matrix (Matricial):&lt;/strong&gt; Estrutura híbrida com reporte duplo (funcional e projeto).&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Flat (Achatada):&lt;/strong&gt; Pouca hierarquia e grande autonomia dos colaboradores.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F336" t="n">
+        <v>0</v>
+      </c>
+      <c r="G336" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>346</v>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Mentalidade de Risco e Prevenção</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Mentalidade de Risco como Base da Prevenção&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Abordagem Proativa:&lt;/strong&gt; Identificar perigos potenciais para agir antes da ocorrência da não conformidade.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Integração ao Processo:&lt;/strong&gt; A prevenção deixa de ser um evento isolado e torna-se parte natural do fluxo de trabalho.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Riscos na Reestruturação Organizacional&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Downsizing:&lt;/strong&gt; O risco é a perda de talentos; a prevenção é o planejamento sucessório.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Delayering:&lt;/strong&gt; O risco é o vácuo de liderança; a prevenção é a automação de relatórios de controle.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Gestão de Autoridade e Riscos&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Empowerment:&lt;/strong&gt; Previne a lentidão burocrática, mas exige controle de risco sobre a competência técnica da base.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Span of Control:&lt;/strong&gt; Uma amplitude muito larga sem suporte tecnológico gera risco de falha humana por sobrecarga.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Estruturas e Controles Preventivos&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Matrix (Matricial):&lt;/strong&gt; Exige protocolos de resolução de conflitos para prevenir a quebra da Unidade de Comando.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Flat (Achatada):&lt;/strong&gt; Requer alta maturidade da equipe para prevenir a falta de direção estratégica.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F337" t="n">
+        <v>0</v>
+      </c>
+      <c r="G337" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>347</v>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>ARL (Average Run Length)</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Curva OC (Operating Characteristic)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Definição:&lt;/strong&gt; Gráfico que relaciona a magnitude de um desvio (k) com a probabilidade de não detectá-lo (&amp;beta;).&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Leitura:&lt;/strong&gt; Se o processo se desloca em 1&amp;sigma; (k=1) e o gráfico aponta 0,7 no eixo Y, isso significa que há 70% de chance de NÃO perceber o erro na primeira amostra.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;ARL (Average Run Length)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Conceito:&lt;/strong&gt; Número médio de amostras até o ponto sair dos limites de controle.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Fórmula Vital:&lt;/strong&gt; $ARL = \frac{1}{1 - \beta}$&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Exemplo da Questão:&lt;/strong&gt; Se &amp;beta; = 0,7, então $ARL = \frac{1}{0,3} = 3,33$.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Dica para Petrobras/Cebraspe:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Se o ARL for alto, o gráfico é ruim para detectar aquele desvio específico.&lt;/li&gt;
+      &lt;li&gt;Sempre verifique se a curva no gráfico representa &amp;beta; (prob. de aceitar o erro) ou $1-\beta$ (poder de detecção). A curva OC padrão sempre plota o &amp;beta; (começa em 1 no k=0 e cai conforme k aumenta).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F338" t="n">
+        <v>0</v>
+      </c>
+      <c r="G338" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>348</v>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Gestão da tecnologia</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceito de Gestão da Tecnologia&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Aplicação prática de métodos científicos para resolução de problemas.&lt;/li&gt;
+      &lt;li&gt;Integração entre ciência, engenharia e administração.&lt;/li&gt;
+      &lt;li&gt;Foco na criação de valor e alcance de metas estratégicas.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Principais Objetivos&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Geração de &lt;strong&gt;Vantagem Competitiva&lt;/strong&gt; sustentável.&lt;/li&gt;
+      &lt;li&gt;Otimização do Ciclo de Vida da Tecnologia (Curva S).&lt;/li&gt;
+      &lt;li&gt;Redução de riscos associados à adoção de novas tecnologias.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Tipos de Inovação&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Incremental:&lt;/strong&gt; Melhorias contínuas em processos existentes.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Radical:&lt;/strong&gt; Ruptura com o modelo atual e criação de novos padrões.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Transferência Tecnológica:&lt;/strong&gt; Aplicação comercial de pesquisas científicas.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Dica para Petrobras/Cebraspe:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;A GT não é um fim em si mesma, mas um &lt;strong&gt;meio&lt;/strong&gt; para a organização ser mais eficiente e competitiva.&lt;/li&gt;
+      &lt;li&gt;Fique atento ao termo &lt;i&gt;"Método Científico"&lt;/i&gt;: se a questão associar gestão tecnológica a empirismo puro ou sorte, geralmente estará incorreta.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F339" t="n">
+        <v>0</v>
+      </c>
+      <c r="G339" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>349</v>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>QFD - Modelo de 4 Matrizes</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceito do QFD (Quality Function Deployment)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Ferramenta para traduzir a "Voz do Cliente" em especificações técnicas.&lt;/li&gt;
+      &lt;li&gt;Reduz mudanças de projeto de última hora e aumenta a satisfação.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;O Modelo de 4 Matrizes (Sequência Lógica)&lt;/strong&gt;
+    &lt;ol&gt;
+      &lt;li&gt;&lt;strong&gt;Matriz 1: Planejamento do Produto (House of Quality)&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;Foco: Requisitos do Cliente vs. Requisitos de Projeto (Engenharia).&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Matriz 2: Desdobramento de Partes&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;Foco: Requisitos de Projeto vs. Características dos Componentes.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Matriz 3: Planejamento do Processo&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;Foco: Características dos Componentes vs. Operações de Produção.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Matriz 4: Planejamento da Produção&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;Foco: Operações de Produção vs. Controles de Qualidade/Instruções.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ol&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Componentes da Matriz 1 (HOQ)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;O quê:&lt;/strong&gt; Necessidades do cliente.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Como:&lt;/strong&gt; Atributos técnicos do produto.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Matriz de Relações:&lt;/strong&gt; Impacto do "Como" no "O quê".&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Telhado (Roof):&lt;/strong&gt; Correlação entre os requisitos técnicos (conflitos ou sinergias).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F340" t="n">
+        <v>0</v>
+      </c>
+      <c r="G340" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>350</v>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Sistemas de Codificação de Materiais</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Numeração Arbitrária (Sequencial)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Atribuição de números por ordem de entrada (1, 2, 3...).&lt;/li&gt;
+      &lt;li&gt;Não possui relação com as características físicas do item.&lt;/li&gt;
+      &lt;li&gt;Dificulta a comunicação técnica e o agrupamento de materiais similares.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Codificação por Grupos e Classes (Sistema Decimal)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;O código é estruturado de forma lógica e hierárquica.&lt;/li&gt;
+      &lt;li&gt;Cada bloco de números representa uma categoria (ex: Grupo -&gt; Classe -&gt; Item).&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Facilita a comunicação interna&lt;/strong&gt;, pois o código "fala" o que o material é.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Dica para Concursos:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Se a questão associar &lt;u&gt;Arbitrário&lt;/u&gt; a &lt;u&gt;Facilidade de Comunicação&lt;/u&gt; ou &lt;u&gt;Lógica de Classes&lt;/u&gt;, o item estará &lt;strong&gt;ERRADO&lt;/strong&gt;.&lt;/li&gt;
+      &lt;li&gt;O sistema arbitrário é simples de implementar, mas pobre em informação.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F341" t="n">
+        <v>0</v>
+      </c>
+      <c r="G341" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="n">
+        <v>351</v>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>BSC (Perspectivas)</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Perspectiva Financeira (Resultados Diretos)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Foco no valor para o acionista (ROI, Lucro, EBITDA).&lt;/li&gt;
+      &lt;li&gt;Representa o objetivo final da estratégia (Efeito).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Perspectiva do Cliente (Mercado)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Foco na satisfação e retenção de clientes.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Perspectiva de Processos Internos (Eficiência)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Foco na excelência das atividades operacionais.&lt;/li&gt;
+      &lt;li&gt;Inclui indicadores como &lt;strong&gt;Custo por Pedido&lt;/strong&gt;.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Perspectiva de Aprendizado e Crescimento (Infraestrutura)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Foco em pessoas, sistemas e cultura organizacional.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;NOTA DE ATENÇÃO:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Regra:&lt;/strong&gt; Apenas índices que medem o desempenho financeiro &lt;u&gt;diretamente&lt;/u&gt; entram na Perspectiva Financeira.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Cuidado:&lt;/strong&gt; Evite classificar indicadores de "meio" (como custos operacionais ou taxas de conversão) como financeiros, mesmo que eles impactem o lucro &lt;u&gt;indiretamente&lt;/u&gt;.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F342" t="n">
+        <v>0</v>
+      </c>
+      <c r="G342" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="n">
+        <v>352</v>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Gestão de Investimentos e Risco</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>modelo CAPM (Capital Asset Pricing Model)</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceito CAPM (Capital Asset Pricing Model)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Modelo que determina o retorno esperado de um investimento com base no risco sistêmico.&lt;/li&gt;
+      &lt;li&gt;Fórmula: $E[R] = R_f + \beta \cdot (R_m - R_f)$.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Cálculo para Carteiras (Portfólio)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;O Beta da carteira é a média ponderada dos Betas individuais.&lt;/li&gt;
+      &lt;li&gt;$\beta_{carteira} = (\% \text{Ativo A} \cdot \beta_A) + (\% \text{Ativo B} \cdot \beta_B)$.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Premissas Importantes&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Taxa Livre de Risco ($R_f$):&lt;/strong&gt; Retorno de ativos sem risco de crédito.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Beta ($\beta$):&lt;/strong&gt; Se &gt; 1, o ativo é mais volátil que o mercado; se &lt; 1, é mais defensivo.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Prêmio de Risco:&lt;/strong&gt; A diferença $(R_m - R_f)$ representa a compensação por correr risco de mercado.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Dica para Concursos:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Cuidado para não confundir "Retorno de Mercado" ($R_m$) com "Prêmio de Risco" ($R_m - R_f$). A questão já deu a diferença (o prêmio) de 10%, facilitando o cálculo.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>0</v>
+      </c>
+      <c r="G343" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="n">
+        <v>353</v>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Gestão da Manutenção e Confiabilidade</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Relação entre MTTF e R(t)</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;MTTF de Sistemas (Tempo Esperado)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Definição Matemática:&lt;/strong&gt; O MTTF é a área sob a curva de confiabilidade $R(t)$.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Sistema em Série:&lt;/strong&gt; $MTTF_{serie} = \frac{1}{\sum \lambda_i}$ (Soma as taxas de falha).&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Sistema em Paralelo (Ativos Idênticos):&lt;/strong&gt; 
+        &lt;ul&gt;
+          &lt;li&gt;Fórmula: $MTTF = \frac{1}{\lambda} \cdot (1 + \frac{1}{2} + \frac{1}{3} + ... + \frac{1}{n})$.&lt;/li&gt;
+          &lt;li&gt;Exemplo n=3: $\frac{1}{\lambda} \cdot \frac{11}{6}$.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Dica de Prova:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Se a questão der a função $F(t) = 1 - e^{-t}$ e pedir o tempo esperado de um sistema &lt;strong&gt;paralelo&lt;/strong&gt; de 3 unidades, a resposta sempre será $11/6$ anos (se $\lambda = 1$).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F344" t="n">
+        <v>0</v>
+      </c>
+      <c r="G344" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="n">
+        <v>354</v>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Verbos</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Presente Histórico e Paralelismo Temporal</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceitos de Verbo para o Cebraspe&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Pretérito Perfeito do Subjuntivo (Tenha Prevalecido):&lt;/strong&gt; Expressa um fato passado concluído em relação a um momento presente.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Presente do Indicativo (É):&lt;/strong&gt; Utilizado aqui para expressar uma definição conceitual e permanente (Presente Atemporal).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Desconstruindo a Pegadinha&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Presente Histórico:&lt;/strong&gt; &lt;u&gt;Não ocorre&lt;/u&gt; neste texto. Ele serve para "trazer o passado para o presente" em narrações, o que não é o caso de um manual técnico.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Paralelismo Temporal:&lt;/strong&gt; Não exige que todos os verbos estejam no mesmo tempo, mas sim que a relação entre eles seja lógica. No texto, a relação é: "Embora algo tenha ocorrido (passado), o fato é (presente)...".&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Dica de Ouro:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Sempre que a banca afirmar que um verbo é "Presente Histórico", verifique se o texto está contando uma história antiga. Se for um texto dissertativo/informativo como este, quase nunca será presente histórico.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F345" t="n">
+        <v>0</v>
+      </c>
+      <c r="G345" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>355</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Iterpretação x Inferência textual</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Compreensão (Literal)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Comandos:&lt;/strong&gt; "Segundo o texto...", "De acordo com o texto...", "O autor afirma que...", "Na linha X, o texto diz...".&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Foco:&lt;/strong&gt; Informação explícita. A resposta está &lt;u&gt;escrita&lt;/u&gt; (mesmo que com outras palavras).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Inferência / Depreensão (Lógica)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Comandos:&lt;/strong&gt; "Infere-se...", "Depreende-se...", "Conclui-se...", "O texto permite concluir que...".&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Foco:&lt;/strong&gt; Informação implícita. É o que &lt;u&gt;nasce&lt;/u&gt; do papel através da lógica do autor.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Extrapolação (ERRO de Interpretação)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Identificação:&lt;/strong&gt; Itens que inserem causas, consequências ou opiniões que &lt;u&gt;não estão&lt;/u&gt; no texto.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Alerta:&lt;/strong&gt; Cuidado com o "bom senso" ou conhecimentos externos que o autor não mencionou.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;O "Pulo do Gato":&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Se o comando é &lt;i&gt;"Segundo o texto"&lt;/i&gt; e a alternativa exige uma conclusão lógica (inferência), o item costuma estar &lt;strong&gt;Errado&lt;/strong&gt; por não ser literal.&lt;/li&gt;
+      &lt;li&gt;Se o comando é &lt;i&gt;"Infere-se"&lt;/i&gt; e a alternativa traz um fato externo, o item é &lt;strong&gt;Extrapolação&lt;/strong&gt;.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>0</v>
+      </c>
+      <c r="G346" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="n">
+        <v>356</v>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Dados</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>DAMA-DMBOK</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Governança de Dados (DAMA-DMBOK)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Foco:&lt;/strong&gt; Autoridade, Planejamento e Controle sobre os ativos de dados.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Responsabilidades:&lt;/strong&gt; Definir políticas, normas, métricas e fiscalizar a conformidade.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Não faz:&lt;/strong&gt; Não realiza a execução técnica direta das atividades operacionais.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Gerenciamento de Dados&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Foco:&lt;/strong&gt; Operacionalização e &lt;u&gt;execução direta&lt;/u&gt; das tarefas.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Responsabilidades:&lt;/strong&gt; Implementar as políticas de qualidade, segurança e arquitetura no ambiente técnico.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Dica de Ouro para a Prova:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Governança:&lt;/strong&gt; "Garante" que as coisas sejam feitas conforme a lei (Fiscal).&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Gerenciamento:&lt;/strong&gt; "Faz" as coisas acontecerem (Executor).&lt;/li&gt;
+      &lt;li&gt;Leu "Execução Direta" vinculada à Governança? O item está &lt;strong&gt;ERRADO&lt;/strong&gt;.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>0</v>
+      </c>
+      <c r="G347" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: flashcards de correção de simulado criados - todos
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G347"/>
+  <dimension ref="A1:G350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17526,6 +17526,182 @@
         <v>0</v>
       </c>
     </row>
+    <row r="348">
+      <c r="A348" t="n">
+        <v>357</v>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Mecanismos de Coesão Textual</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Paralelismo</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Paralelismo Sintático&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Substantivo com Substantivo:&lt;/strong&gt; "Temos fé &lt;u&gt;na&lt;/u&gt; vitória e &lt;u&gt;na&lt;/u&gt; aprovação."&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Verbo com Verbo:&lt;/strong&gt; "É necessário &lt;u&gt;estudar&lt;/u&gt; teoria e &lt;u&gt;praticar&lt;/u&gt; exercícios."&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Cuidado:&lt;/strong&gt; Omissão de preposição no segundo termo quebra o paralelismo (Ex: "Gosto de café e chocolate" está OK, mas "Gosto &lt;u&gt;do&lt;/u&gt; café e chocolate" é erro, deve ser "&lt;u&gt;do&lt;/u&gt; café e &lt;u&gt;do&lt;/u&gt; chocolate").&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Paralelismo Semântico&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Manutenção da lógica e do campo de ideias.&lt;/li&gt;
+      &lt;li&gt;Evita o "efeito lista de supermercado" com itens que não se conversam.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Impacto nas Reescritas (Cebraspe)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Muitas reescritas que parecem corretas falham porque trocam um substantivo simples por uma oração (Ex: "...buscando &lt;u&gt;agilidade&lt;/u&gt; e &lt;u&gt;que os processos sejam rápidos&lt;/u&gt;"). Isso quebra a simetria.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>0</v>
+      </c>
+      <c r="G348" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>358</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Inflação Acumulada</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceito de Inflação Acumulada&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Representa o aumento real de preços em uma sequência de períodos.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Regra de Ouro:&lt;/strong&gt; Taxas de inflação (ou juros) &lt;u&gt;nunca se somam&lt;/u&gt; aritmeticamente; elas são capitalizadas (multiplicadas).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Fórmula de Cálculo&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Para taxas $i_1, i_2, ..., i_n$, a fórmula é: $I_{acc} = [(1 + i_1) \cdot (1 + i_2) \cdot ... \cdot (1 + i_n)] - 1$.&lt;/li&gt;
+      &lt;li&gt;Exemplo: Inflação de 10% e 10% no mês seguinte vira $(1,10 \cdot 1,10) - 1 = 21\%$.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Deflação e Variações Negativas&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Se houver queda de preços (ex: -2%), o fator de multiplicação será menor que 1 (ex: $1 - 0,02 = 0,98$).&lt;/li&gt;
+      &lt;li&gt;O processo de multiplicação entre os períodos permanece idêntico.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Média da Inflação&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Para achar a inflação média periódica a partir da acumulada, utiliza-se a &lt;strong&gt;Média Geométrica&lt;/strong&gt; (raiz enésima do fator total).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Dica para Petrobras/ANSA:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;A banca adora colocar a soma simples nas alternativas para te induzir ao erro. Sempre transforme em fator ($1 + i$) antes de operar.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F349" t="n">
+        <v>0</v>
+      </c>
+      <c r="G349" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>359</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Proteção contra vírus</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Aplicativos Antivírus</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;1ª Geração (Assinatura / Escaneamento Simples)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Foco em identificar o que já é conhecido.&lt;/li&gt;
+      &lt;li&gt;Técnica: Comparação de &lt;u&gt;assinaturas&lt;/u&gt; (strings de bits específicas).&lt;/li&gt;
+      &lt;li&gt;Limitação: Inútil contra vírus novos ou modificados.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;2ª Geração (Proativa / Escaneamento Avançado)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Foco em prever ameaças novas (Zero-Day).&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Técnica Principal: Heurística&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;Não busca o código exato, mas &lt;u&gt;padrões e regras de similaridade&lt;/u&gt;.&lt;/li&gt;
+          &lt;li&gt;Identifica variações de famílias de vírus conhecidos.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Outras Técnicas desta Geração:&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;&lt;strong&gt;Análise Comportamental:&lt;/strong&gt; Bloqueia ações suspeitas durante a execução.&lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Sandboxing:&lt;/strong&gt; Emulação em ambiente isolado.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Diferença de Ouro para a Prova:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Se a questão diz que o antivírus detecta vírus &lt;u&gt;por semelhança&lt;/u&gt; ou &lt;u&gt;por padrões de código&lt;/u&gt;, ela está falando de &lt;strong&gt;HEURÍSTICA&lt;/strong&gt; (2ª Geração).&lt;/li&gt;
+      &lt;li&gt;Se diz que detecta pela &lt;u&gt;ação&lt;/u&gt; do arquivo no sistema, está falando de &lt;strong&gt;COMPORTAMENTO&lt;/strong&gt;.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F350" t="n">
+        <v>0</v>
+      </c>
+      <c r="G350" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: final do dia 17/04
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -5567,7 +5567,7 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G135" t="n">
         <v>1</v>
@@ -5842,7 +5842,7 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G142" t="n">
         <v>1</v>
@@ -5886,7 +5886,7 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G143" t="n">
         <v>1</v>
@@ -5960,7 +5960,7 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G145" t="n">
         <v>1</v>
@@ -5999,7 +5999,7 @@
         <v>0</v>
       </c>
       <c r="G146" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147">
@@ -7483,7 +7483,7 @@
         <v>1</v>
       </c>
       <c r="G188" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="189">
@@ -7545,7 +7545,7 @@
         <v>0</v>
       </c>
       <c r="G190" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="191">
@@ -7576,7 +7576,7 @@
         <v>0</v>
       </c>
       <c r="G191" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="192">
@@ -7731,7 +7731,7 @@
         <v>0</v>
       </c>
       <c r="G196" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="197">
@@ -7907,7 +7907,7 @@
         <v>0</v>
       </c>
       <c r="G199" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="200">
@@ -7985,7 +7985,7 @@
         <v>0</v>
       </c>
       <c r="G201" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="202">
@@ -8588,7 +8588,7 @@
         <v>0</v>
       </c>
       <c r="G218" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="219">
@@ -8625,7 +8625,7 @@
         <v>0</v>
       </c>
       <c r="G219" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="220">
@@ -8901,7 +8901,7 @@
         <v>0</v>
       </c>
       <c r="G226" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="227">
@@ -8971,7 +8971,7 @@
         <v>0</v>
       </c>
       <c r="G228" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="229">
@@ -9330,7 +9330,7 @@
         <v>0</v>
       </c>
       <c r="G238" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="239">
@@ -10184,7 +10184,7 @@
         <v>0</v>
       </c>
       <c r="G254" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="255">
@@ -16972,7 +16972,7 @@
         <v>0</v>
       </c>
       <c r="G335" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="336">

</xml_diff>

<commit_message>
:up: conteudo front colocado tb no back
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -8971,7 +8971,7 @@
         <v>0</v>
       </c>
       <c r="G228" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="229">
@@ -16972,7 +16972,7 @@
         <v>0</v>
       </c>
       <c r="G335" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="336">

</xml_diff>

<commit_message>
:release: fómulas matemáticas agora podem ser lidas
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -1199,12 +1199,14 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>37</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1234,12 +1236,14 @@
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
-        <v>40</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1253,7 +1257,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>etapas do FMEA</t>
+          <t>etapas do FMEA (Análise de Modo e Efeitos de Falha)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1274,7 +1278,7 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -1316,8 +1320,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
-        <v>42</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1331,7 +1337,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>3 fases da FTA</t>
+          <t>3 fases da FTA (Fault Tree Analysis) - Análise da Árvore de Falhas</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1347,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
@@ -3267,31 +3273,15 @@
       <c r="E72" t="inlineStr">
         <is>
           <t>&lt;ol&gt;
-	&lt;li&gt;Socialização
-&lt;ul&gt;
-	&lt;li&gt;tácito → tácito&lt;/li&gt;
-&lt;/ul&gt;
-&lt;/li&gt;
-	&lt;li&gt;Externalização
-&lt;ul&gt;
-	&lt;li&gt;tácito → explícito&lt;/li&gt;
-&lt;/ul&gt;
-&lt;/li&gt;
-	&lt;li&gt;Combinação
-&lt;ul&gt;
-	&lt;li&gt;explícito → explícito
-&lt;ul&gt;
-	&lt;li&gt;explícito → tácito&lt;/li&gt;
-&lt;/ul&gt;
-&lt;/li&gt;
-&lt;/ul&gt;
-&lt;/li&gt;
-	&lt;li&gt;Internalização&lt;/li&gt;
+	&lt;li&gt;Socialização &lt;ul&gt; &lt;li&gt;tácito → tácito&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Externalização &lt;ul&gt; &lt;li&gt;tácito → explícito&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Combinação &lt;ul&gt; &lt;li&gt;explícito → explícito&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Internalização &lt;ul&gt; &lt;li&gt;explícito → tácito&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 &lt;/ol&gt;</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G72" t="n">
         <v>1</v>
@@ -8334,8 +8324,10 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" t="n">
-        <v>276</v>
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -8354,7 +8346,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tácito &lt;ul&gt; &lt;li&gt;reside nas pessoas&lt;/li&gt; &lt;li&gt;é subjetivo, pessoal, difícil de formalizar&lt;/li&gt; &lt;li&gt;dimensão técnica &lt;ul&gt; &lt;li&gt;&lt;i&gt;know-how&lt;/i&gt;&lt;/li&gt; &lt;li&gt;habilidades motoras&lt;/li&gt; &lt;li&gt;perceptivas difíceis de verbalizar&lt;/li&gt; &lt;/ul&gt; &lt;/li&gt; &lt;li&gt;dimensão cognitiva &lt;ul&gt; &lt;li&gt;modelos mentais&lt;/li&gt; &lt;li&gt;crenças&lt;/li&gt; &lt;li&gt;crenças&lt;/li&gt; &lt;li&gt;percepções&lt;/li&gt; &lt;li&gt;intuições&lt;/li&gt; &lt;/ul&gt; &lt;/li&gt; &lt;/ul&gt;
+          <t xml:space="preserve">Tácito &lt;ul&gt; &lt;li&gt;reside nas pessoas&lt;/li&gt; &lt;li&gt;é subjetivo, pessoal, difícil de formalizar&lt;/li&gt; &lt;li&gt;dimensão técnica &lt;ul&gt; &lt;li&gt;&lt;i&gt;know-how&lt;/i&gt;&lt;/li&gt; &lt;li&gt;habilidades motoras&lt;/li&gt; &lt;li&gt;perceptivas difíceis de verbalizar&lt;/li&gt; &lt;/ul&gt; &lt;/li&gt; &lt;li&gt;dimensão cognitiva &lt;ul&gt; &lt;li&gt;modelos mentais&lt;/li&gt; &lt;li&gt;crenças&lt;/li&gt; &lt;li&gt;valores&lt;/li&gt; &lt;li&gt;percepções&lt;/li&gt; &lt;li&gt;intuições&lt;/li&gt; &lt;/ul&gt; &lt;/li&gt; &lt;/ul&gt;
 Explícito &lt;ul&gt; &lt;li&gt;pode ser formalizado&lt;/li&gt; &lt;li&gt;é documentado, codificado e sistematizado em procedimentos, manuais, relatórios, sistemas de informação, bancos de dados&lt;/li&gt; &lt;li&gt;mais fácil de ser transferido entre pessoas, de ser replicado e armazenado&lt;/li&gt; &lt;/ul&gt;
 </t>
         </is>
@@ -8363,7 +8355,7 @@
         <v>0</v>
       </c>
       <c r="G194" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="195">

</xml_diff>

<commit_message>
:up: função de criar parágrafos aplicadas também em textos e enunciados da seção praticar/simuado
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -5066,7 +5066,7 @@
         <v>0</v>
       </c>
       <c r="G115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="116">
@@ -7103,7 +7103,7 @@
         <v>0</v>
       </c>
       <c r="G168" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="169">
@@ -10684,7 +10684,7 @@
         <v>0</v>
       </c>
       <c r="G219" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="220">

</xml_diff>

<commit_message>
:up: algumas questões respondidas - CG
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -4082,7 +4082,7 @@
         <v>0</v>
       </c>
       <c r="G86" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="87">
@@ -4122,7 +4122,7 @@
         <v>0</v>
       </c>
       <c r="G87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88">
@@ -4158,7 +4158,7 @@
         <v>0</v>
       </c>
       <c r="G88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="89">
@@ -4192,7 +4192,7 @@
         <v>1</v>
       </c>
       <c r="G89" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90">
@@ -4226,7 +4226,7 @@
         <v>0</v>
       </c>
       <c r="G90" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="91">
@@ -4939,7 +4939,7 @@
         <v>1</v>
       </c>
       <c r="G111" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="112">
@@ -4970,7 +4970,7 @@
         <v>0</v>
       </c>
       <c r="G112" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113">
@@ -5001,7 +5001,7 @@
         <v>0</v>
       </c>
       <c r="G113" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="114">
@@ -5032,7 +5032,7 @@
         <v>0</v>
       </c>
       <c r="G114" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115">
@@ -5070,8 +5070,10 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="n">
-        <v>194</v>
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>194</t>
+        </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -5090,14 +5092,14 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Muitos investidores, credores por empréstimos e outros credores</t>
+          <t>Muitos investidores, credores por empréstimos e outros credores, existentes e potenciais, não podem exigir que as entidades que reportam forneçam informações diretamente a eles, devendo se basear em relatórios financeiros para fins gerais para muitas das informações financeiras de que necessitam. Consequentemente, eles são os principais usuários aos quais se destinam relatórios financeiros para fins gerais.</t>
         </is>
       </c>
       <c r="F116" t="n">
         <v>0</v>
       </c>
       <c r="G116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117">
@@ -7059,7 +7061,7 @@
         <v>1</v>
       </c>
       <c r="G167" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="168">
@@ -7161,7 +7163,7 @@
         <v>0</v>
       </c>
       <c r="G169" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="170">
@@ -7218,7 +7220,7 @@
         <v>0</v>
       </c>
       <c r="G170" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="171">
@@ -7326,7 +7328,7 @@
         <v>0</v>
       </c>
       <c r="G171" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="172">
@@ -10489,7 +10491,7 @@
         <v>0</v>
       </c>
       <c r="G215" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="216">
@@ -10541,7 +10543,7 @@
         <v>0</v>
       </c>
       <c r="G216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217">
@@ -10587,7 +10589,7 @@
         <v>0</v>
       </c>
       <c r="G217" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="218">
@@ -10638,7 +10640,7 @@
         <v>0</v>
       </c>
       <c r="G218" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="219">
@@ -10736,7 +10738,7 @@
         <v>0</v>
       </c>
       <c r="G220" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="221">

</xml_diff>

<commit_message>
:up: alguns cards criados - RL
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G300"/>
+  <dimension ref="A1:G308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1155,7 +1155,7 @@
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" t="n">
         <v>5</v>
@@ -1275,16 +1275,60 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>etapas da Análise de Modo e Efeitos de Falha (FMEA - Failure Mode and Effect Analysis)</t>
+          <t>Análise de Modo e Efeitos de Falha (FMEA - Failure Mode and Effect Analysis)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>&lt;ol&gt;
-	&lt;li&gt;Definição e Identificação &lt;ol&gt; &lt;li&gt;Função do equipament&lt;/li&gt; &lt;li&gt;Falha funcional&lt;/li&gt; &lt;li&gt;Componente&lt;/li&gt; &lt;li&gt;Modo (s) de falha potencial&lt;/li&gt; &lt;li&gt;Efeito (s) potencial (is) da falha&lt;/li&gt; &lt;li&gt;Causa (s) potencial (is) de falha&lt;/li&gt; &lt;li&gt;Controles atuais&lt;/li&gt; &lt;li&gt;Frequência do processo atual&lt;/li&gt; &lt;/ol&gt;&lt;/li&gt;
-	&lt;li&gt;quantificação do risco de cada modo de falha &lt;ul&gt; &lt;li&gt;usando um número de prioridade de risco (NPR) &lt;ul&gt; &lt;li&gt;NPR = SEV x OCC x DET &lt;ul&gt; &lt;li&gt;Gravidade ou Severidade (SEV)&lt;/li&gt; &lt;li&gt;Probabilidade de ocorrência (OCC)&lt;/li&gt; &lt;li&gt;Probabilidade de detecção (DET)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;minimizar o risco &lt;ul&gt; &lt;li&gt;priorização pelo NPR &lt;ul&gt; &lt;li&gt;20% principais&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;Implementando Soluções&lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Conceito:&lt;/strong&gt; Proativo, quantitativo e focado em impedir a falha.&lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Relação com o RCFA:&lt;/strong&gt; Serve de base para o RCFA; se uma falha prevista ocorre, o RCFA investiga se a causa real era a prevista.&lt;/li&gt;
+    &lt;li&gt;Definição e Identificação 
+        &lt;ol&gt; 
+            &lt;li&gt;Função do equipament&lt;/li&gt; 
+            &lt;li&gt;Falha funcional&lt;/li&gt; 
+            &lt;li&gt;Componente&lt;/li&gt; 
+            &lt;li&gt;Modo (s) de falha potencial&lt;/li&gt; 
+            &lt;li&gt;Efeito (s) potencial (is) da falha&lt;/li&gt; 
+            &lt;li&gt;Causa (s) potencial (is) de falha&lt;/li&gt; 
+            &lt;li&gt;Controles atuais&lt;/li&gt; 
+            &lt;li&gt;Frequência do processo atual&lt;/li&gt; 
+        &lt;/ol&gt;
+    &lt;/li&gt;
+    &lt;li&gt;quantificação do risco de cada modo de falha 
+        &lt;ul&gt; 
+            &lt;li&gt;usando um número de prioridade de risco (NPR) 
+                &lt;ul&gt; 
+                    &lt;li&gt;
+                        &lt;math xmlns="http://www.w3.org/1998/Math/MathML"&gt;
+                            &lt;mi&gt;NPR&lt;/mi&gt;
+                            &lt;mo&gt;=&lt;/mo&gt;
+                            &lt;mi&gt;SEV&lt;/mi&gt;
+                            &lt;mo&gt;&amp;#x00D7;&lt;/mo&gt;
+                            &lt;mi&gt;OCC&lt;/mi&gt;
+                            &lt;mo&gt;&amp;#x00D7;&lt;/mo&gt;
+                            &lt;mi&gt;DET&lt;/mi&gt;
+                        &lt;/math&gt;
+                        &lt;ul&gt; 
+                            &lt;li&gt;Gravidade ou Severidade (SEV)&lt;/li&gt; 
+                            &lt;li&gt;Probabilidade de ocorrência (OCC)&lt;/li&gt; 
+                            &lt;li&gt;Probabilidade de detecção (DET)&lt;/li&gt; 
+                        &lt;/ul&gt;
+                    &lt;/li&gt; 
+                &lt;/ul&gt;
+            &lt;/li&gt; 
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;minimizar o risco 
+        &lt;ul&gt; 
+            &lt;li&gt;priorização pelo NPR 
+                &lt;ul&gt; 
+                    &lt;li&gt;20% principais&lt;/li&gt; 
+                &lt;/ul&gt;
+            &lt;/li&gt; 
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;Implementando Soluções&lt;/li&gt;
 &lt;/ol&gt;</t>
         </is>
       </c>
@@ -1292,7 +1336,7 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21">
@@ -1313,18 +1357,20 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Etapas do processo da análise da causa raiz da falha (RCFA - Root Cause FailureAnalisys)</t>
+          <t>análise da causa raiz da falha (RCFA - Root Cause FailureAnalisys)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>&lt;ol&gt;
-	&lt;li&gt;Identificação dos sintomas&lt;/li&gt;
-	&lt;li&gt;Avaliação das causas endereçáveis&lt;/li&gt;
-	&lt;li&gt;Coletando e analisando dados&lt;/li&gt;
-	&lt;li&gt;Isolando e testando variáveis&lt;/li&gt;
-	&lt;li&gt;Identificando a (s) causa (s)&lt;/li&gt;
-	&lt;li&gt;Criação e implementação de um plano de ação&lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Conceito:&lt;/strong&gt; Reativo, qualitativo e focado em corrigir a falha (causa raiz).&lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Relação com o FMEA:&lt;/strong&gt; Pode ser considerado uma simplificação da FMEA. Os achados da RCFA devem atualizar as causas potenciais do FMEA.&lt;/li&gt;
+    &lt;li&gt;Identificação dos sintomas&lt;/li&gt;
+    &lt;li&gt;Avaliação das causas endereçáveis&lt;/li&gt;
+    &lt;li&gt;Coletando e analisando dados&lt;/li&gt;
+    &lt;li&gt;Isolando e testando variáveis&lt;/li&gt;
+    &lt;li&gt;Identificando a (s) causa (s)&lt;/li&gt;
+    &lt;li&gt;Criação e implementação de um plano de ação&lt;/li&gt;
 &lt;/ol&gt;</t>
         </is>
       </c>
@@ -1332,7 +1378,7 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
@@ -1369,7 +1415,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
@@ -1426,7 +1472,7 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -4082,7 +4128,7 @@
         <v>0</v>
       </c>
       <c r="G86" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="87">
@@ -4122,7 +4168,7 @@
         <v>0</v>
       </c>
       <c r="G87" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="88">
@@ -4158,12 +4204,14 @@
         <v>0</v>
       </c>
       <c r="G88" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="n">
-        <v>164</v>
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>164</t>
+        </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -4183,7 +4231,7 @@
       <c r="E89" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;Atos contábeis ou Atos Administrativos &lt;ul&gt; &lt;li&gt;não provocam alterações do patrimônio&lt;/li&gt; &lt;li&gt;ou apenas irão alterar o Patrimônio no futuro&lt;/li&gt; &lt;li&gt;Ex.: &lt;ul&gt; &lt;li&gt;admissão de empregados&lt;/li&gt; &lt;li&gt;assinatura de um contrato de compra&lt;/li&gt; &lt;li&gt;venda&lt;/li&gt; &lt;li&gt;o aval de um título de crédito&lt;/li&gt; &lt;li&gt;uma fiança prestada em favor de terceiros&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;Lei 6.404/76: Art. 176. (...) § 4º As demonstrações serão complementadas&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Atos contábeis ou Atos Administrativos &lt;ul&gt; &lt;li&gt;não provocam alterações do patrimônio&lt;/li&gt; &lt;li&gt;ou apenas irão alterar o Patrimônio no futuro&lt;/li&gt; &lt;li&gt;Ex.: &lt;ul&gt; &lt;li&gt;admissão de empregados&lt;/li&gt; &lt;li&gt;assinatura de um contrato de compra&lt;/li&gt; &lt;li&gt;venda&lt;/li&gt; &lt;li&gt;o aval de um título de crédito&lt;/li&gt; &lt;li&gt;uma fiança prestada em favor de terceiros&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;Lei 6.404/76: Art. 176. (...) § 4º  As demonstrações serão complementadas por notas explicativas e outros quadros analíticos ou demonstrações contábeis necessários para esclarecimento da situação patrimonial e dos resultados do exercício.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 	&lt;li&gt;Fatos contábeis ou Fatos Administrativos &lt;ul&gt; &lt;li&gt;provocam variações no patrimônio da entidade&lt;/li&gt; &lt;li&gt;são contabilizados através &lt;ul&gt; &lt;li&gt;das contas patrimoniais (ativo, passivo, patrimônio líquido)&lt;/li&gt; &lt;li&gt;e/ou das contas de resultado (receitas e despesas)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
@@ -4192,7 +4240,7 @@
         <v>1</v>
       </c>
       <c r="G89" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="90">
@@ -4226,7 +4274,7 @@
         <v>0</v>
       </c>
       <c r="G90" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="91">
@@ -4261,7 +4309,7 @@
         <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -4297,7 +4345,7 @@
         <v>0</v>
       </c>
       <c r="G92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -4331,7 +4379,7 @@
         <v>0</v>
       </c>
       <c r="G93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -4366,7 +4414,7 @@
         <v>0</v>
       </c>
       <c r="G94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
@@ -4397,7 +4445,7 @@
         <v>0</v>
       </c>
       <c r="G95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -4428,7 +4476,7 @@
         <v>0</v>
       </c>
       <c r="G96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97">
@@ -4459,7 +4507,7 @@
         <v>0</v>
       </c>
       <c r="G97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -4493,7 +4541,7 @@
         <v>0</v>
       </c>
       <c r="G98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -4528,7 +4576,7 @@
         <v>0</v>
       </c>
       <c r="G99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100">
@@ -4563,7 +4611,7 @@
         <v>0</v>
       </c>
       <c r="G100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -4598,7 +4646,7 @@
         <v>0</v>
       </c>
       <c r="G101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102">
@@ -4629,7 +4677,7 @@
         <v>0</v>
       </c>
       <c r="G102" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103">
@@ -4660,7 +4708,7 @@
         <v>0</v>
       </c>
       <c r="G103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -4695,7 +4743,7 @@
         <v>0</v>
       </c>
       <c r="G104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -4726,7 +4774,7 @@
         <v>0</v>
       </c>
       <c r="G105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -4766,7 +4814,7 @@
         <v>0</v>
       </c>
       <c r="G106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -4797,7 +4845,7 @@
         <v>1</v>
       </c>
       <c r="G107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -4832,7 +4880,7 @@
         <v>0</v>
       </c>
       <c r="G108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109">
@@ -4861,7 +4909,7 @@
           <t>&lt;ul&gt;
 	&lt;li&gt;Equivalência contrapositiva &lt;ul&gt; &lt;li&gt;p→q ≡ ~q→~p&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 	&lt;li&gt;Transformação da condicional em disjunção inclusiva &lt;ul&gt; &lt;li&gt;p→q ≡ ~p∨q&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;Transformação disjunção inclusiva em condicional &lt;ul&gt; &lt;li&gt;p∨q ≡ ~p→q&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;Transformação disjunção inclusiva em condicional &lt;ul&gt; &lt;li&gt;~p→q ≡ p∨q&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -4869,7 +4917,7 @@
         <v>0</v>
       </c>
       <c r="G109" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110">
@@ -4903,7 +4951,7 @@
         <v>1</v>
       </c>
       <c r="G110" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111">
@@ -4931,7 +4979,7 @@
         <is>
           <t>&lt;ul&gt;
 	&lt;li&gt;caráter científico  (1º Congresso Brasileiro de Contabilidade/1924)&lt;ul&gt; &lt;li&gt;ciência que estuda e pratica as funções de orientação, de controle e de registro dos atos e fatos de uma administração econômica&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;doutrina  (IPECAFI)&lt;ul&gt; &lt;li&gt;objetivamente, um sistema de informação&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;objetivamente, um sistema de informação e avaliação destinado a prover seus usuários com demonstrações e análises de natureza econômica, financeira, física e de produtividade, com relação à entidade objeto de contabilização&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -4939,7 +4987,7 @@
         <v>1</v>
       </c>
       <c r="G111" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="112">
@@ -4970,7 +5018,7 @@
         <v>0</v>
       </c>
       <c r="G112" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="113">
@@ -4998,7 +5046,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G113" t="n">
         <v>3</v>
@@ -5032,7 +5080,7 @@
         <v>0</v>
       </c>
       <c r="G114" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="115">
@@ -5066,7 +5114,7 @@
         <v>0</v>
       </c>
       <c r="G115" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116">
@@ -5099,7 +5147,7 @@
         <v>0</v>
       </c>
       <c r="G116" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="117">
@@ -5199,7 +5247,7 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G119" t="n">
         <v>3</v>
@@ -5235,7 +5283,7 @@
         <v>0</v>
       </c>
       <c r="G120" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="121">
@@ -5268,7 +5316,7 @@
         <v>0</v>
       </c>
       <c r="G121" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="122">
@@ -5301,7 +5349,7 @@
         <v>0</v>
       </c>
       <c r="G122" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123">
@@ -5334,7 +5382,7 @@
         <v>1</v>
       </c>
       <c r="G123" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="124">
@@ -5367,7 +5415,7 @@
         <v>0</v>
       </c>
       <c r="G124" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="125">
@@ -5400,7 +5448,7 @@
         <v>0</v>
       </c>
       <c r="G125" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="126">
@@ -5427,97 +5475,56 @@
       <c r="E126" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-  &lt;li&gt;operação padrão digital
-    &lt;ul&gt;
-      &lt;li&gt;gestão de políticas e processos&lt;/li&gt;
-      &lt;li&gt;documentos com validade legal
-        &lt;ul&gt;
-          &lt;li&gt;assinados eletronicamente&lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;atos processuais
-    &lt;ul&gt;
-      &lt;li&gt;meio digital
-        &lt;ul&gt;
-          &lt;li&gt;exceções
-            &lt;ul&gt;
-              &lt;li&gt;solicitação do usuário&lt;/li&gt;
-              &lt;li&gt;inviabilidade técnica ou indisponibilidade&lt;/li&gt;
-              &lt;li&gt;risco à celeridade&lt;/li&gt;
-            &lt;/ul&gt;
-          &lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-      &lt;li&gt;validade
-        &lt;ul&gt;
-          &lt;li&gt;preservados parâmetros de segurança&lt;/li&gt;
-          &lt;li&gt;não se aplica ao anonimato&lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-      &lt;li&gt;contagem de prazo
-        &lt;ul&gt;
-          &lt;li&gt;dia e hora do recebimento&lt;/li&gt;
-          &lt;li&gt;tempestivos até as 23h59 do último dia
-            &lt;ul&gt;
-              &lt;li&gt;horário de Brasília&lt;/li&gt;
-            &lt;/ul&gt;
-          &lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;acesso e arquivamento
-    &lt;ul&gt;
-      &lt;li&gt;sistemas informatizados ou cópias&lt;/li&gt;
-      &lt;li&gt;classificação conforme a LAI&lt;/li&gt;
-      &lt;li&gt;assegurar preservação e acesso
-        &lt;ul&gt;
-          &lt;li&gt;normas da instituição arquivística pública responsável (ex: Arq. Nacional)&lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;prestação digital de serviços
-    &lt;ul&gt;
-      &lt;li&gt;tecnologias acessíveis à população
-&lt;ul&gt;
-	&lt;li&gt;incluindo
-&lt;ul&gt;
-	&lt;li&gt;baixa renda&lt;/li&gt;
-	&lt;li&gt;áreas rurais ou isoladas&lt;/li&gt;
-&lt;/ul&gt;
-&lt;/li&gt;
-&lt;/ul&gt;
-&lt;/li&gt;
-      &lt;li&gt;atendimento presencial
-        &lt;ul&gt;
-          &lt;li&gt;permanece como direito&lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-      &lt;li&gt;preferência pelo autosserviço&lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;Estratégia de Governo Digital
-    &lt;ul&gt;
-      &lt;li&gt;atuação integrada e cooperativa&lt;/li&gt;
-      &lt;li&gt;entes federados podem elaborar a própria
-        &lt;ul&gt;
-          &lt;li&gt;alinhada à nacional&lt;/li&gt;
-&lt;li style="color: #e74c3c;"&gt;Independe de delegação formal ou Lei Complementar (Autonomia)&lt;/li&gt;
-        &lt;/ul&gt;
-      &lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-&lt;/ul&gt;</t>
+	&lt;li&gt;&lt;strong&gt;Digitalização (Arts. 5º - 13)&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Soluções Digitais para:
+				&lt;ul&gt;
+					&lt;li&gt;gestão de políticas (finalísticas e administrativas)&lt;/li&gt;
+					&lt;li&gt;trâmite de processos administrativos eletrônicos&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Documentos e Atos Processuais:
+				&lt;ul&gt;
+					&lt;li&gt;emissão (atestados, certidões, diplomas) assinados eletronicamente&lt;/li&gt;
+					&lt;li&gt;validade: mediante assinatura eletrônica (autenticidade, integridade, segurança)&lt;/li&gt;
+					&lt;li&gt;originais: documentos nato-digitais assinados eletronicamente&lt;/li&gt;
+					&lt;li&gt;tempestividade: até 23h59 (&lt;strong&gt;horário de Brasília&lt;/strong&gt;) com recibo de protocolo&lt;/li&gt;
+					&lt;li&gt;realização: regra em meio eletrônico (exceções: solicitação, inviabilidade ou risco à celeridade)&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Acesso e Arquivamento:
+				&lt;ul&gt;
+					&lt;li&gt;vistas: sistema ou cópia (preferencialmente eletrônica)&lt;/li&gt;
+					&lt;li&gt;sigilo: classificação conforme a LAI&lt;/li&gt;
+					&lt;li&gt;guarda: conforme legislação e normas arquivísticas nacionais&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;strong&gt;Governo Digital (Arts. 14 - 16)&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Prestação Digital de Serviços:
+				&lt;ul&gt;
+					&lt;li&gt;acesso: tecnologias de amplo alcance (baixa renda/áreas isoladas)&lt;/li&gt;
+					&lt;li&gt;atendimento: direito ao presencial; preferência pelo &lt;strong&gt;autosserviço&lt;/strong&gt;&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Estratégias:
+				&lt;ul&gt;
+					&lt;li&gt;Nacional: integrada e cooperativa&lt;/li&gt;
+					&lt;li&gt;Entes Federados: autonomia para editar estratégia própria (compatível com a federal)&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F126" t="n">
         <v>0</v>
       </c>
       <c r="G126" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="127">
@@ -5547,7 +5554,7 @@
 	&lt;li&gt;Criadas pelo Poder Executivo federal&lt;/li&gt;
 	&lt;li&gt;Objetivo: &lt;ul&gt; &lt;li&gt;fortalecer o trabalho colaborativo&lt;/li&gt; &lt;li&gt;gerar, compartilhar e disseminar conhecimentos e experiências&lt;/li&gt; &lt;li&gt;identificar e avaliar novas tecnologias&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 	&lt;li&gt;Papeis &lt;ul&gt; &lt;li&gt;formular propostas relacionadas a padrões, políticas, guias e manuais&lt;/li&gt; &lt;li&gt;promover discussões sobre desafios e possibilidades de ação&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
-	&lt;li&gt;A participação é aberta a todos os órgãos e entidades&lt;/li&gt;
+	&lt;li&gt;A participação é aberta a todos os órgãos e entidades da administração pública&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -5555,7 +5562,7 @@
         <v>0</v>
       </c>
       <c r="G127" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="128">
@@ -5584,8 +5591,6 @@
           <t>&lt;ul&gt;
 	&lt;li&gt;Base Nacional de Serviços Públicos&lt;/li&gt;
 	&lt;li&gt;Plataformas de Governo Digital&lt;/li&gt;
-	&lt;li&gt;Prestação Digital dos Serviços Públicos&lt;/li&gt;
-	&lt;li&gt;Direitos dos Usuários da Prestação Digital de Serviços Públicos&lt;/li&gt;
 	&lt;li&gt;Cartas de Serviços ao Usuário (Lei nº 13.460/2017)&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
@@ -5594,7 +5599,7 @@
         <v>0</v>
       </c>
       <c r="G128" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="129">
@@ -5633,7 +5638,7 @@
         <v>0</v>
       </c>
       <c r="G129" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="130">
@@ -5668,7 +5673,7 @@
         <v>0</v>
       </c>
       <c r="G130" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="131">
@@ -5702,7 +5707,7 @@
         <v>0</v>
       </c>
       <c r="G131" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="132">
@@ -5735,7 +5740,7 @@
         <v>0</v>
       </c>
       <c r="G132" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="133">
@@ -6972,7 +6977,7 @@
         <v>0</v>
       </c>
       <c r="G165" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="166">
@@ -7030,7 +7035,7 @@
         <v>0</v>
       </c>
       <c r="G166" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="167">
@@ -7061,7 +7066,7 @@
         <v>1</v>
       </c>
       <c r="G167" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="168">
@@ -7105,7 +7110,7 @@
         <v>0</v>
       </c>
       <c r="G168" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="169">
@@ -7163,7 +7168,7 @@
         <v>0</v>
       </c>
       <c r="G169" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="170">
@@ -7220,7 +7225,7 @@
         <v>0</v>
       </c>
       <c r="G170" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="171">
@@ -7328,7 +7333,7 @@
         <v>0</v>
       </c>
       <c r="G171" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="172">
@@ -7402,7 +7407,7 @@
         <v>0</v>
       </c>
       <c r="G172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173">
@@ -7482,7 +7487,7 @@
         <v>0</v>
       </c>
       <c r="G173" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174">
@@ -7658,7 +7663,7 @@
         <v>0</v>
       </c>
       <c r="G176" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="177">
@@ -7725,7 +7730,7 @@
         <v>0</v>
       </c>
       <c r="G177" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="178">
@@ -7809,7 +7814,7 @@
         <v>0</v>
       </c>
       <c r="G178" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="179">
@@ -7887,7 +7892,7 @@
         <v>0</v>
       </c>
       <c r="G179" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="180">
@@ -7991,12 +7996,14 @@
         <v>0</v>
       </c>
       <c r="G180" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="n">
-        <v>270</v>
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>270</t>
+        </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -8019,14 +8026,17 @@
 	&lt;li&gt;transporte de fluxos &lt;ul&gt; &lt;li&gt;negativos para Valor Presente &lt;ul&gt; &lt;li&gt;Taxa de Financiamento&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;li&gt;positivos para Valor Futuro &lt;ul&gt; &lt;li&gt;Taxa de Reinvestimento&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 	&lt;li&gt;transformação do fluxo &lt;ul&gt; &lt;li&gt;torna o fluxo convencional&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 	&lt;li&gt;possibilidade de trabalhar com duas taxas diferentes&lt;/li&gt;
-&lt;/ul&gt;</t>
+    &lt;li&gt;Taxa de Financiamento &lt;ul&gt; &lt;li&gt;utilizada para descapitalizar saídas de caixa (fluxos negativos)&lt;/li&gt; &lt;li&gt;desnecessária se houver apenas um fluxo negativo na data zero (t=0)&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+    &lt;li&gt;Taxa de Reinvestimento &lt;ul&gt; &lt;li&gt;utilizada para capitalizar as receitas (fluxos positivos)&lt;/li&gt; &lt;li&gt;essencial para o cálculo da TIRM, mesmo em fluxos convencionais&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+    &lt;li&gt;Dependência da TIRM (Caso Específico) &lt;ul&gt; &lt;li&gt;se negativo apenas na data zero: depende apenas dos fluxos e da Taxa de Reinvestimento&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+    &lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F181" t="n">
         <v>0</v>
       </c>
       <c r="G181" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="182">
@@ -8084,7 +8094,7 @@
         <v>2</v>
       </c>
       <c r="G182" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="183">
@@ -8117,7 +8127,7 @@
         <v>1</v>
       </c>
       <c r="G183" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="184">
@@ -10491,7 +10501,7 @@
         <v>0</v>
       </c>
       <c r="G215" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="216">
@@ -10543,7 +10553,7 @@
         <v>0</v>
       </c>
       <c r="G216" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="217">
@@ -10589,7 +10599,7 @@
         <v>0</v>
       </c>
       <c r="G217" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="218">
@@ -10640,7 +10650,7 @@
         <v>0</v>
       </c>
       <c r="G218" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="219">
@@ -10686,7 +10696,7 @@
         <v>0</v>
       </c>
       <c r="G219" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="220">
@@ -10738,7 +10748,7 @@
         <v>0</v>
       </c>
       <c r="G220" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="221">
@@ -15074,7 +15084,7 @@
         <v>1</v>
       </c>
       <c r="G264" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="265">
@@ -15423,7 +15433,7 @@
         <v>0</v>
       </c>
       <c r="G270" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="271">
@@ -15484,7 +15494,7 @@
         <v>0</v>
       </c>
       <c r="G271" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="272">
@@ -15850,7 +15860,7 @@
         <v>0</v>
       </c>
       <c r="G278" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="279">
@@ -15961,7 +15971,7 @@
         <v>0</v>
       </c>
       <c r="G280" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="281">
@@ -17011,6 +17021,473 @@
         <v>0</v>
       </c>
     </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>395</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Formas de Indeterminação do Sujeito</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>&lt;ol&gt;
+  &lt;li&gt;&lt;strong&gt;Verbo na 3ª Pessoa do Plural&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Requisito: O sujeito não deve ter sido mencionado anteriormente no contexto.&lt;/li&gt;
+      &lt;li&gt;Exemplo: "Disseram que a prova da Petrobras será difícil."&lt;/li&gt;
+      &lt;li&gt;Nota de Inspeção: Se o contexto permitir identificar o agente (ex: "Os diretores chegaram. Disseram..."), o sujeito deixa de ser indeterminado e passa a ser Sujeito Oculto/Desinencial.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Verbo na 3ª Pessoa do Singular + Partícula "SE" (IIS)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Requisito: O verbo deve ser Intransitivo (V.I.), Transitivo Indireto (V.T.I.) ou de Ligação (V.L.).&lt;/li&gt;
+      &lt;li&gt;Configuração: O "SE" atua como Índice de Indeterminação do Sujeito.&lt;/li&gt;
+      &lt;li&gt;Exemplo (VTI): "Precisa-se de novos engenheiros de produção."&lt;/li&gt;
+      &lt;li&gt;Exemplo (VI): "Vive-se bem em Piranhas."&lt;/li&gt;
+      &lt;li&gt;Alerta de Erro (Cebraspe): Se o verbo for Transitivo Direto (VTD), o "SE" vira Partícula Passivadora e o sujeito será o termo que sofre a ação (Sujeito Paciente).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Verbo no Infinitivo Impessoal&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Requisito: O verbo não se refere a uma pessoa específica, expressando a ação de forma genérica.&lt;/li&gt;
+      &lt;li&gt;Exemplo: "Era proibido fumar naquela área da usina."&lt;/li&gt;
+      &lt;li&gt;Exemplo: "Estudar é necessário para a aprovação."&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ol&gt;</t>
+        </is>
+      </c>
+      <c r="F301" t="n">
+        <v>0</v>
+      </c>
+      <c r="G301" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>396</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Funções Sintáticas</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Circunstâncias Adverbiais</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>&lt;ol&gt;
+  &lt;li&gt;&lt;strong&gt;Causal&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Função: Indica o motivo da oração principal.&lt;/li&gt;
+      &lt;li&gt;Conjunções: porque, visto que, como (no início da frase), uma vez que, já que.&lt;/li&gt;
+      &lt;li&gt;Exemplo: "A produção parou &lt;em&gt;porque&lt;/em&gt; a máquina quebrou."&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Comparativa&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Função: Estabelece comparação com a principal.&lt;/li&gt;
+      &lt;li&gt;Conjunções: como, tal qual, tanto quanto, (mais/menos) que.&lt;/li&gt;
+      &lt;li&gt;Exemplo: "O sistema opera &lt;em&gt;como&lt;/em&gt; um relógio."&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Concessiva (O terror do Cebraspe)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Função: Indica um fato contrário, mas que não impede a ação principal (ideia de oposição/contraste).&lt;/li&gt;
+      &lt;li&gt;Conjunções: embora, conquanto, ainda que, mesmo que, posto que, apesar de que.&lt;/li&gt;
+      &lt;li&gt;Exemplo: "O engenheiro foi contratado, &lt;em&gt;embora&lt;/em&gt; não tivesse experiência no setor."&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Condicional&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Função: Indica uma condição para que o fato ocorra.&lt;/li&gt;
+      &lt;li&gt;Conjunções: se, caso, contanto que, desde que, a menos que.&lt;/li&gt;
+      &lt;li&gt;Exemplo: "O custo será reduzido &lt;em&gt;se&lt;/em&gt; a automação for aplicada."&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Conformativa&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Função: Indica acordo ou conformidade.&lt;/li&gt;
+      &lt;li&gt;Conjunções: conforme, segundo, consoante, como.&lt;/li&gt;
+      &lt;li&gt;Exemplo: "A nota fiscal foi emitida &lt;em&gt;conforme&lt;/em&gt; Martins e Dutra orientaram."&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Consecutiva&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Função: Indica a consequência de um fato mencionado na principal.&lt;/li&gt;
+      &lt;li&gt;Conjunções: de sorte que, de modo que, (tão/tal/tanto) que.&lt;/li&gt;
+      &lt;li&gt;Exemplo: "Estudou tanto &lt;em&gt;que&lt;/em&gt; passou em primeiro lugar."&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Final&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Função: Indica o objetivo ou a finalidade.&lt;/li&gt;
+      &lt;li&gt;Conjunções: para que, a fim de que, porque (com valor de para que).&lt;/li&gt;
+      &lt;li&gt;Exemplo: "Treinamos a equipe &lt;em&gt;para que&lt;/em&gt; o erro não se repita."&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Temporal&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Função: Indica o tempo em que ocorre a ação.&lt;/li&gt;
+      &lt;li&gt;Conjunções: quando, logo que, assim que, enquanto, mal.&lt;/li&gt;
+      &lt;li&gt;Exemplo: "A auditoria começou &lt;em&gt;assim que&lt;/em&gt; o relatório ficou pronto."&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Proporcional&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Função: Indica um fato que ocorre simultaneamente e na mesma proporção.&lt;/li&gt;
+      &lt;li&gt;Conjunções: à medida que, à proporção que, quanto mais... mais.&lt;/li&gt;
+      &lt;li&gt;Exemplo: "O risco aumenta &lt;em&gt;à medida que&lt;/em&gt; o controle diminui."&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ol&gt;</t>
+        </is>
+      </c>
+      <c r="F302" t="n">
+        <v>0</v>
+      </c>
+      <c r="G302" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>397</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Princípio do Custo Afundado (Sunk Cost)</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Princípio de custo irrelevante &lt;ul&gt; &lt;li&gt;gastos passados, já incorridos e irrecuperáveis, não devem afetar escolhas futuras.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F303" t="n">
+        <v>0</v>
+      </c>
+      <c r="G303" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>398</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129-2021</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Direitos dos Usuários da Prestação Digital de Serviços Públicos</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+    &lt;li&gt;&lt;strong&gt;Direitos dos Usuários (Art. 27 - Lei 14.129)&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;&lt;strong&gt;Gratuidade&lt;/strong&gt; no acesso às Plataformas de Governo Digital.&lt;/li&gt;
+            &lt;li&gt;Atendimento conforme a &lt;strong&gt;Carta de Serviços ao Usuário&lt;/strong&gt; (fidelidade ao prometido).&lt;/li&gt;
+            &lt;li&gt;&lt;strong&gt;Padronização&lt;/strong&gt; de formulários, guias e documentos (físicos e digitais).&lt;/li&gt;
+            &lt;li&gt;Recebimento de &lt;strong&gt;protocolo (físico ou digital)&lt;/strong&gt; de TODAS as solicitações.&lt;/li&gt;
+            &lt;li&gt;Indicação de &lt;strong&gt;canal preferencial&lt;/strong&gt; para receber notificações e avisos.&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Leis Complementares citadas:&lt;/strong&gt;
+        &lt;ul&gt;
+            &lt;li&gt;Lei 13.460/2017 (Participação e Proteção do Usuário).&lt;/li&gt;
+            &lt;li&gt;Lei 13.709/2018 (LGPD).&lt;/li&gt;
+        &lt;/ul&gt;
+    &lt;/li&gt;
+    &lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F304" t="n">
+        <v>0</v>
+      </c>
+      <c r="G304" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>399</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Equivalências e Negações Lógicas</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Conectivo "Ou" Implícito</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;&lt;strong&gt;Regra da Vírgula Disjuntiva&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Ocorre em enumerações onde o último conectivo da lista é "ou".&lt;/li&gt;
+			&lt;li&gt;As vírgulas anteriores assumem automaticamente o valor lógico de disjunção ($\lor$).&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;strong&gt;Critério de Identificação&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;O fechamento da sentença determina a função das vírgulas:
+				&lt;ul&gt;
+					&lt;li&gt;Se termina em "ou": todas as vírgulas anteriores operam como "ou".&lt;/li&gt;
+					&lt;li&gt;Finalidade: evitar a repetição excessiva do conectivo no texto.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F305" t="n">
+        <v>0</v>
+      </c>
+      <c r="G305" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>400</v>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Lógica de Argumentação</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Lógica de Argumentação</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;&lt;strong&gt;Estrutura e Validade&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Definição: Conjunto de Premissas ($P_1, P_2, ...$) $\to$ Conclusão ($C$).&lt;/li&gt;
+			&lt;li&gt;Argumento Válido: A verdade das premissas **obriga** a verdade da conclusão.
+				&lt;ul&gt;
+					&lt;li&gt;$(P_1 \land P_2 \land ...) \to C$ é uma Tautologia.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Argumento Inválido (Falácia/Sofisma): É possível ter premissas (V) e conclusão (F).&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;strong&gt;Técnica de Validação (Método das Premissas Verdadeiras)&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Passo 1: Assuma que a Conclusão é &lt;strong&gt;Falsa&lt;/strong&gt;.&lt;/li&gt;
+			&lt;li&gt;Passo 2: Tente tornar todas as Premissas &lt;strong&gt;Verdadeiras&lt;/strong&gt;.&lt;/li&gt;
+			&lt;li&gt;Análise do Resultado:
+				&lt;ul&gt;
+					&lt;li&gt;Conseguiu (Sem contradição) $\to$ &lt;strong&gt;Inválido&lt;/strong&gt;.&lt;/li&gt;
+					&lt;li&gt;Houve contradição (Premissa forçada a ser F) $\to$ &lt;strong&gt;Válido&lt;/strong&gt;.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;strong&gt;Regras de Inferência Rápidas&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Modus Ponens: $(p \to q) \land p \implies q$.&lt;/li&gt;
+			&lt;li&gt;Modus Tollens: $(p \to q) \land \neg q \implies \neg p$.&lt;/li&gt;
+			&lt;li&gt;Silogismo Hipotético: $(p \to q) \land (q \to r) \implies (p \to r)$.&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F306" t="n">
+        <v>0</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Diagramas Lógicos</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Negação de Proposições Quantificadas</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Relações:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Nenhum $\equiv \sim \exists$ (Negação de "Algum")&lt;/li&gt;
+      &lt;li&gt;Algum $\equiv \exists$&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;hr&gt;
+  &lt;li&gt;$\sim \forall \equiv \exists$
+    &lt;ul&gt;
+      &lt;li&gt;Para negar "Todo gato mia", basta "Algum gato não mia"&lt;/li&gt;
+      &lt;li&gt;Para negar "Nenhuma cobra voa", basta "Alguma cobra voa"&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;$\sim \exists \equiv \forall$
+    &lt;ul&gt;
+      &lt;li&gt;Para negar "Algum médico é rico", basta "Nenhum médico é rico"&lt;/li&gt;
+      &lt;li&gt;Para negar "Existe aluno que não estuda", basta "Todo aluno estuda"&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F307" t="n">
+        <v>0</v>
+      </c>
+      <c r="G307" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>402</v>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Lógica de Primeira Ordem</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Lógica de Primeira Ordem (LPO)</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceitos Iniciais&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Variável ($x$):&lt;/strong&gt; Objeto que assume valores do Universo de Discurso.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Predicado ($P(x)$):&lt;/strong&gt; Propriedade atribuída à variável.
+        &lt;ul&gt;
+          &lt;li&gt;Ex: $I(x) = x$ é ímpar.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Quantificadores&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Universal ($\forall$):&lt;/strong&gt; "Todo", "Qualquer", "Cada".&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Existencial ($\exists$):&lt;/strong&gt; "Algum", "Existe", "Pelo menos um".&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Tradução de Proposições Categóricas&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Todo A é B:&lt;/strong&gt; $(\forall x)(A(x) \rightarrow B(x))$
+        &lt;ul&gt;
+          &lt;li&gt;Lógica: "Se é A, então é B".&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Algum A é B:&lt;/strong&gt; $(\exists x)(A(x) \land B(x))$
+        &lt;ul&gt;
+          &lt;li&gt;Lógica: "Existe x que é A e B ao mesmo tempo".&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Nenhum A é B:&lt;/strong&gt; $(\forall x)(A(x) \rightarrow \neg B(x))$ ou $\neg (\exists x)(A(x) \land B(x))$
+        &lt;ul&gt;
+          &lt;li&gt;Lógica: "Se é A, então não é B" ou "Não existe A que seja B".&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Algum A não é B:&lt;/strong&gt; $(\exists x)(A(x) \land \neg B(x))$
+        &lt;ul&gt;
+          &lt;li&gt;Lógica: "Existe x que é A e não é B".&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>0</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: last f Pc
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G308"/>
+  <dimension ref="A1:G335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -682,7 +682,7 @@
         <v>4</v>
       </c>
       <c r="G5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -741,7 +741,7 @@
         <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -1135,17 +1135,27 @@
     &lt;ul&gt;
       &lt;li&gt;&lt;strong&gt;Preventiva:&lt;/strong&gt; Atuação baseada em &lt;u&gt;intervalos fixos&lt;/u&gt; (Tempo, Ciclos, Km).
         &lt;ul&gt;
+&lt;li&gt;&lt;strong&gt;Subdivisões (Cesgranrio):&lt;/strong&gt; Por tempo e Preditiva.&lt;/li&gt;
           &lt;li&gt;&lt;strong&gt;Gatilho:&lt;/strong&gt; Calendário ou horímetro. A troca ocorre mesmo se o item estiver em perfeitas condições. No gráfico, os intervalos são constantes ($\Delta t$).&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Na Curva P-F:&lt;/strong&gt; Atua no intervalo onde a falha se torna mais evidente e percebida por inspeções ou sinais claros, antes da parada total.&lt;/li&gt;
         &lt;/ul&gt;
       &lt;/li&gt;
       &lt;li&gt;&lt;strong&gt;Preditiva:&lt;/strong&gt; Atuação baseada no &lt;u&gt;estado real&lt;/u&gt; via monitoramento de variáveis (Vibração, Temperatura, Termografia).
         &lt;ul&gt;
           &lt;li&gt;&lt;strong&gt;Gatilho:&lt;/strong&gt; Quando a variável monitorada atinge um limite de alerta. O intervalo entre intervenções é variável.&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Na Curva P-F:&lt;/strong&gt; Início da falha potencial (Ponto P). Utiliza sensores e monitoramento para detectar anomalias antes de haver sinais visíveis ou falha funcional.&lt;/li&gt;
         &lt;/ul&gt;
       &lt;/li&gt;
       &lt;li&gt;&lt;strong&gt;Corretiva Planejada:&lt;/strong&gt; Estratégia de "rodar até falhar", mas com logística e recursos já prontos para a troca imediata após o limite de desempenho.&lt;/li&gt;
       &lt;li&gt;&lt;strong&gt;Detectiva:&lt;/strong&gt; Focada em sistemas de proteção (ex: alarmes, geradores de reserva). Busca identificar "falhas ocultas" que só seriam percebidas em uma emergência.&lt;/li&gt;
-      &lt;li&gt;&lt;strong&gt;Prescritiva:&lt;/strong&gt; Evolução da preditiva que utiliza análise de dados para sugerir "o que fazer" para evitar a falha, agindo na causa raiz operacional.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Prescritiva:&lt;/strong&gt;
+  &lt;ul&gt;
+    &lt;li&gt;Evolução da preditiva.&lt;/li&gt;
+    &lt;li&gt;Sugere ações via IA/Dados.&lt;/li&gt;
+    &lt;li&gt;Causa raiz operacional.&lt;/li&gt;
+    &lt;li&gt;Tendência (Indústria 4.0).&lt;/li&gt;
+    &lt;/ul&gt;
+&lt;/li&gt;
     &lt;/ul&gt;
   &lt;/li&gt;
 &lt;/ul&gt;</t>
@@ -1155,12 +1165,14 @@
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
-        <v>25</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1182,10 +1194,24 @@
           <t>&lt;ul&gt;
   &lt;li&gt;&lt;strong&gt;Filosofia e Objetivos&lt;/strong&gt;
     &lt;ul&gt;
-      &lt;li&gt;&lt;strong&gt;Conceito:&lt;/strong&gt; Gestão integrada focada na eficácia global dos equipamentos (OEE), com envolvimento de todos os níveis (do operador à alta gestão).&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Conceito:&lt;/strong&gt; Gestão baseada na &lt;strong&gt;parceria com o operador&lt;/strong&gt; e envolvimento de todos os níveis para maximizar o OEE.&lt;/li&gt;
       &lt;li&gt;&lt;strong&gt;Metas Principais:&lt;/strong&gt; Zero Quebras, Zero Defeitos, Zero Acidentes e Redução de Custos.&lt;/li&gt;
     &lt;/ul&gt;
   &lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Estratégia Quebra Zero (Nakajima / FGV)&lt;/strong&gt;
+    &lt;ul&gt;
+        &lt;li&gt;&lt;strong&gt;Conceito:&lt;/strong&gt; Garantir que a máquina não pare durante o período programado para operar.&lt;/li&gt;
+        &lt;li&gt;&lt;strong&gt;As 5 Medidas Fundamentais:&lt;/strong&gt;
+            &lt;ol&gt;
+                &lt;li&gt;&lt;strong&gt;Condições Básicas:&lt;/strong&gt; Limpeza, asseio e ordem (5S) estruturam a operação.&lt;/li&gt;
+                &lt;li&gt;&lt;strong&gt;Condições de Operação:&lt;/strong&gt; Obedecer aos limites técnicos.&lt;/li&gt;
+                &lt;li&gt;&lt;strong&gt;Recuperação da Deterioração:&lt;/strong&gt; Tratar o desgaste antes da quebra.&lt;/li&gt;
+                &lt;li&gt;&lt;strong&gt;Sanar Falhas de Projeto:&lt;/strong&gt; Usar diagnósticos e previsão de vida média para redesenhar pontos fracos.&lt;/li&gt;
+                &lt;li&gt;&lt;strong&gt;Habilidades Técnicas:&lt;/strong&gt; Capacitar operadores e mantenedores.&lt;/li&gt;
+            &lt;/ol&gt;
+        &lt;/li&gt;
+    &lt;/ul&gt;
+&lt;/li&gt;
   &lt;li&gt;&lt;strong&gt;Os 8 Pilares da TPM&lt;/strong&gt;
     &lt;ul&gt;
       &lt;li&gt;1. Manutenção Autônoma (Operador cuida da máquina).&lt;/li&gt;
@@ -1217,7 +1243,7 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19">
@@ -1251,10 +1277,10 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G19" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
@@ -1281,7 +1307,7 @@
       <c r="E20" t="inlineStr">
         <is>
           <t>&lt;ol&gt;
-    &lt;li&gt;&lt;strong&gt;Conceito:&lt;/strong&gt; Proativo, quantitativo e focado em impedir a falha.&lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Conceito:&lt;/strong&gt; Proativo, qualitativa e focado em impedir a falha (Raciocínio Indutivo / Bottom-Up).&lt;/li&gt;
     &lt;li&gt;&lt;strong&gt;Relação com o RCFA:&lt;/strong&gt; Serve de base para o RCFA; se uma falha prevista ocorre, o RCFA investiga se a causa real era a prevista.&lt;/li&gt;
     &lt;li&gt;Definição e Identificação 
         &lt;ol&gt; 
@@ -1336,7 +1362,7 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21">
@@ -1363,7 +1389,7 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>&lt;ol&gt;
-    &lt;li&gt;&lt;strong&gt;Conceito:&lt;/strong&gt; Reativo, qualitativo e focado em corrigir a falha (causa raiz).&lt;/li&gt;
+    &lt;li&gt;&lt;strong&gt;Conceito:&lt;/strong&gt; Reativo, qualitativo e focado em corrigir a causa raiz (Raciocínio Dedutivo / Top-Down).&lt;/li&gt;
     &lt;li&gt;&lt;strong&gt;Relação com o FMEA:&lt;/strong&gt; Pode ser considerado uma simplificação da FMEA. Os achados da RCFA devem atualizar as causas potenciais do FMEA.&lt;/li&gt;
     &lt;li&gt;Identificação dos sintomas&lt;/li&gt;
     &lt;li&gt;Avaliação das causas endereçáveis&lt;/li&gt;
@@ -1378,7 +1404,7 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22">
@@ -1415,7 +1441,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
@@ -1472,7 +1498,7 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
@@ -1878,7 +1904,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G34" t="n">
         <v>2</v>
@@ -2049,7 +2075,7 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40">
@@ -2120,7 +2146,7 @@
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
@@ -2189,7 +2215,7 @@
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
@@ -2306,7 +2332,7 @@
         <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47">
@@ -2750,10 +2776,10 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58">
@@ -3031,8 +3057,10 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="n">
-        <v>108</v>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -3051,14 +3079,16 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>P&lt;sub&gt;n&lt;/sub&gt;&lt;sup&gt;k&lt;sub&gt;1&lt;/sub&gt;,k&lt;sub&gt;2&lt;/sub&gt;,...k&lt;sub&gt;i&lt;/sub&gt;&lt;/sup&gt; = n!/(k&lt;sub&gt;1&lt;/sub&gt;! x k&lt;sub&gt;2&lt;/sub&gt;! x ... x k&lt;sub&gt;i&lt;/sub&gt;!)</t>
+          <t>&lt;li&gt;
+  $$P_{n}^{k_{1}, k_{2}, \dots, k_{i}} = \frac{n!}{k_{1}! \cdot k_{2}! \cdot \dots \cdot k_{i}!}$$
+&lt;/li&gt;</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -3089,7 +3119,7 @@
         <v>2</v>
       </c>
       <c r="G65" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="66">
@@ -3115,14 +3145,32 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>CR&lt;sup&gt;p&lt;/sup&gt;&lt;sub&gt;n&lt;/sub&gt; = P&lt;sup&gt;n-1,p&lt;/sup&gt;&lt;sub&gt;n-1+p&lt;/sub&gt; = C&lt;sup&gt;n+p-1&lt;/sup&gt;&lt;sub&gt;n&lt;/sub&gt; = [(n-1+p)!]/[(n-1)!xp!]</t>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Combinação com Repetição (ou Completa)&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Identidade e Relações:&lt;/strong&gt;
+        $$CR^{p}_{n} = P^{p, n-1}_{n+p-1} = C^{n+p-1}_{p} = \binom{n+p-1}{p}$$
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Fórmula Fatorial:&lt;/strong&gt;
+        $$\frac{(n+p-1)!}{p! \cdot (n-1)!}$$
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Variáveis:&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;&lt;strong&gt;$n$:&lt;/strong&gt; Número de tipos ou categorias disponíveis.&lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;$p$:&lt;/strong&gt; Número de elementos a serem escolhidos (vagas).&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Gatilho:&lt;/strong&gt; Problemas de "Soluções Inteiras Não Negativas" ou distribuição de objetos idênticos em caixas distintas.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67">
@@ -3193,7 +3241,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G68" t="n">
         <v>0</v>
@@ -3234,7 +3282,7 @@
         <v>5</v>
       </c>
       <c r="G69" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="70">
@@ -3272,7 +3320,7 @@
         <v>7</v>
       </c>
       <c r="G70" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71">
@@ -3329,7 +3377,7 @@
         <v>7</v>
       </c>
       <c r="G71" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="72">
@@ -3364,7 +3412,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G72" t="n">
         <v>1</v>
@@ -3449,7 +3497,7 @@
         <v>6</v>
       </c>
       <c r="G73" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="74">
@@ -3498,12 +3546,14 @@
         <v>4</v>
       </c>
       <c r="G74" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="n">
-        <v>124</v>
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -3523,7 +3573,20 @@
       <c r="E75" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;Comunidades de Prática (CoP)&lt;/li&gt;
+	&lt;li&gt;Comunidades de Prática (CoP)
+&lt;ul&gt;
+  &lt;li&gt;Grupos orgânicos e informais para troca de experiências e desafios reais (não é grupo formal de trabalho).&lt;/li&gt;
+  &lt;li&gt;Elementos fundamentais:
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Domínio:&lt;/strong&gt; Tema de interesse compartilhado.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Engajamento social:&lt;/strong&gt; Interação regular e construção de confiança.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Prática compartilhada:&lt;/strong&gt; Foco na realidade vivida e soluções testadas.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Objetivo: Capturar e difundir o conhecimento tácito (experiência individual).&lt;/li&gt;
+  &lt;li&gt;Premissa: Autenticidade e espontaneidade (não deve ser imposta ou controlada em excesso).&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
 	&lt;li&gt;Lições Aprendidas, Storytelling e Repositórios de Conhecimento &lt;ul&gt; &lt;li&gt;mentoring, coaching e aprendizagem organizacional&lt;/li&gt; &lt;li&gt;circuitos de aprendizagem&lt;/li&gt; &lt;li&gt;cinco disciplinas essenciais que precisam estar integradas para que uma organização aprenda de verdade&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
 	&lt;li&gt;Mapas de Conhecimento&lt;/li&gt;
 	&lt;li&gt;Bases de Conhecimento e Sistemas de Informação&lt;/li&gt;
@@ -3535,7 +3598,7 @@
         <v>0</v>
       </c>
       <c r="G75" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="76">
@@ -3599,7 +3662,7 @@
         <v>2</v>
       </c>
       <c r="G76" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="77">
@@ -3634,7 +3697,7 @@
         <v>1</v>
       </c>
       <c r="G77" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="78">
@@ -3673,7 +3736,7 @@
         <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="79">
@@ -3710,7 +3773,7 @@
         <v>2</v>
       </c>
       <c r="G79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="80">
@@ -3770,7 +3833,7 @@
         <v>6</v>
       </c>
       <c r="G80" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81">
@@ -3971,7 +4034,20 @@
   &lt;/li&gt;
   &lt;li&gt;&lt;strong&gt;Complemento Nominal (CN):&lt;/strong&gt; Completa nome (Adj/Adv/Subst. Abstrato). Sempre preposicionado e valor &lt;u&gt;passivo&lt;/u&gt;.&lt;/li&gt;
   &lt;li&gt;&lt;strong&gt;Agente da Passiva:&lt;/strong&gt; Executor da ação na Voz Passiva (preposição "por").&lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Predicativo do Sujeito:&lt;/strong&gt; Atributo, estado ou qualidade do sujeito. 
+    &lt;ul&gt;
+      &lt;li&gt;Gatilho: Aparece obrigatoriamente com Verbo de Ligação (VL) ou como núcleo nominal em predicados Verbo-Nominais.&lt;/li&gt;
+      &lt;li&gt;Exemplo: "O engenheiro de produção está &lt;em&gt;focado&lt;/em&gt;." (VL) / "Lucas trabalha &lt;em&gt;feliz&lt;/em&gt;." (V.I. + Pred. Sujeito).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
   &lt;li&gt;&lt;strong&gt;Predicativo do Objeto:&lt;/strong&gt; Característica atribuída ao objeto através do verbo.&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Diferencial CN vs. Adj Adn (O Teste do Alvo):&lt;/strong&gt;
+&lt;ul&gt;
+	&lt;li&gt;&lt;b&gt;CN&lt;/b&gt;: Sentido PASSIVO (é o alvo da ação). Ex: "Monitoramento &lt;u&gt;do estado&lt;/u&gt;" (O estado é monitorado).&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Adj Adn&lt;/b&gt;: Sentido ATIVO/POSSE. Ex: "Estado &lt;u&gt;do ativo&lt;/u&gt;" (O ativo possui um estado).&lt;/li&gt;
+	&lt;li&gt;Gatilho do Adjetivo: Se o termo se liga a um ADJETIVO, a função é &lt;b&gt;obrigatoriamente &lt;/b&gt;CN. &lt;ul&gt; &lt;li&gt;Ex: "Superior &lt;u&gt;ao calculado&lt;/u&gt;" (Superior = Adjetivo $\rightarrow$ termo seguinte = CN).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -4008,7 +4084,13 @@
           <t>&lt;ul&gt;
   &lt;li&gt;&lt;strong&gt;Adjunto Adnominal (AA):&lt;/strong&gt; Orbita o substantivo (Artigo, Adjetivo, Numeral, Pronome). Valor ativo.&lt;/li&gt;
   &lt;li&gt;&lt;strong&gt;Adjunto Adverbial:&lt;/strong&gt; Circunstância (Tempo, Lugar, Modo). Modifica Verbo, Adjetivo ou Advérbio.&lt;/li&gt;
-  &lt;li&gt;&lt;strong&gt;Aposto e Vocativo:&lt;/strong&gt; Aposto explica/resume; Vocativo interpela/chama (termo independente).&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Aposto e Vocativo:&lt;/strong&gt; Aposto explica/resume; Vocativo interpela/chama (termo independente).
+&lt;ul&gt;
+	&lt;li&gt;&lt;b&gt;Aposto Especificativo (A Es):&lt;/b&gt; Substantivo Próprio que especifica um Substantivo Comum sem vírgula. &lt;ul&gt; &lt;li&gt;Ex: "Biomas &lt;u&gt;amazônia e cerrado&lt;/u&gt;" (Substantivo + Substantivo).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Adjunto Adnominal (Adj Adn):&lt;/b&gt; Adjetivo que caracteriza o nome. &lt;ul&gt; &lt;li&gt;Ex: "Bioma &lt;u&gt;brasileiro&lt;/u&gt;" (Substantivo + Adjetivo).&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Regra da Vírgula (Faculdade):&lt;/b&gt; &lt;ul&gt; &lt;li&gt;Adjunto Adverbial deslocado de &lt;b&gt;até 3 palavras&lt;/b&gt; $\rightarrow$ Vírgula Facultativa.&lt;/li&gt; &lt;li&gt;Adjunto Adverbial deslocado de &lt;b&gt;4 palavras ou mais&lt;/b&gt; $\rightarrow$ Vírgula Obrigatória.&lt;/li&gt; &lt;li&gt;&lt;b&gt;Atenção:&lt;/b&gt; No Aposto Explicativo, a vírgula é &lt;b&gt;SEMPRE &lt;/b&gt;obrigatória, independente do tamanho.&lt;/li&gt; &lt;/ul&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -4020,8 +4102,10 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="n">
-        <v>160</v>
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -4063,7 +4147,12 @@
 					&lt;li&gt;Objetivas Diretas&lt;/li&gt;
 					&lt;li&gt;Objetivas Indiretas&lt;/li&gt;
 					&lt;li&gt;Completivas Nominais&lt;/li&gt;
-					&lt;li&gt;Predicativas&lt;/li&gt;
+					&lt;li&gt;Predicativas
+    &lt;ul&gt;
+        &lt;li&gt;&lt;strong&gt;Estrutura:&lt;/strong&gt; SS + VL + CSI.&lt;/li&gt;
+        &lt;li&gt;&lt;strong&gt;Diferencial:&lt;/strong&gt; Vem sempre após Verbo de Ligação. Ex: "O ponto é &lt;em&gt;que a intervenção ocorre&lt;/em&gt;."&lt;/li&gt;
+    &lt;/ul&gt;
+&lt;/li&gt;
 					&lt;li&gt;Apositivas&lt;/li&gt;
 				&lt;/ul&gt;
 			&lt;/li&gt;
@@ -4917,7 +5006,7 @@
         <v>0</v>
       </c>
       <c r="G109" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="110">
@@ -4951,7 +5040,7 @@
         <v>1</v>
       </c>
       <c r="G110" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="111">
@@ -5247,7 +5336,7 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G119" t="n">
         <v>3</v>
@@ -5283,7 +5372,7 @@
         <v>0</v>
       </c>
       <c r="G120" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="121">
@@ -5316,7 +5405,7 @@
         <v>0</v>
       </c>
       <c r="G121" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="122">
@@ -5349,7 +5438,7 @@
         <v>0</v>
       </c>
       <c r="G122" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="123">
@@ -5382,7 +5471,7 @@
         <v>1</v>
       </c>
       <c r="G123" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124">
@@ -5415,7 +5504,7 @@
         <v>0</v>
       </c>
       <c r="G124" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="125">
@@ -5445,7 +5534,7 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G125" t="n">
         <v>6</v>
@@ -5499,6 +5588,13 @@
 					&lt;li&gt;guarda: conforme legislação e normas arquivísticas nacionais&lt;/li&gt;
 				&lt;/ul&gt;
 			&lt;/li&gt;
+&lt;li&gt;Melhoria e Testes (Art. 13):
+				&lt;ul&gt;
+					&lt;li&gt;Órgãos &lt;strong&gt;podem&lt;/strong&gt; realizar testes e pesquisas com usuários.&lt;/li&gt;
+					&lt;li&gt;Finalidade: Identificar falhas e melhorar a experiência de uso.&lt;/li&gt;
+					&lt;li&gt;Regra: Deve observar estritamente a LGPD.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
 		&lt;/ul&gt;
 	&lt;/li&gt;
 	&lt;li&gt;&lt;strong&gt;Governo Digital (Arts. 14 - 16)&lt;/strong&gt;
@@ -5524,7 +5620,7 @@
         <v>0</v>
       </c>
       <c r="G126" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="127">
@@ -5562,7 +5658,7 @@
         <v>0</v>
       </c>
       <c r="G127" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="128">
@@ -5599,12 +5695,14 @@
         <v>0</v>
       </c>
       <c r="G128" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="n">
-        <v>212</v>
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -5631,6 +5729,7 @@
 	&lt;li&gt;Apoio a entes federados&lt;/li&gt;
 	&lt;li&gt;Uso de assinatura eletrônicas&lt;/li&gt;
 	&lt;li&gt;atendimento aos idosos&lt;/li&gt;
+&lt;li&gt;&lt;b&gt;Desburocratização e modernização&lt;/b&gt;&lt;/li&gt; &lt;li&gt;&lt;b&gt;Linguagem clara e compreensível&lt;/b&gt;&lt;/li&gt; &lt;li&gt;&lt;b&gt;Atuação integrada e interoperabilidade&lt;/b&gt;&lt;/li&gt; &lt;li&gt;&lt;b&gt;Presunção de boa-fé do usuário&lt;/b&gt;&lt;/li&gt; &lt;li&gt;&lt;b&gt;Acessibilidade (PcD e mobilidade reduzida)&lt;/b&gt;&lt;/li&gt; &lt;/ul&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -5638,7 +5737,7 @@
         <v>0</v>
       </c>
       <c r="G129" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="130">
@@ -5673,7 +5772,7 @@
         <v>0</v>
       </c>
       <c r="G130" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="131">
@@ -5707,7 +5806,7 @@
         <v>0</v>
       </c>
       <c r="G131" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="132">
@@ -5740,7 +5839,7 @@
         <v>0</v>
       </c>
       <c r="G132" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="133">
@@ -6444,6 +6543,13 @@
     &lt;ul&gt;
       &lt;li&gt;Único Banco de Dados Centralizado.&lt;/li&gt;
       &lt;li&gt;Relação com Tabelas.&lt;/li&gt;
+&lt;li&gt;Arquitetura Cliente/Servidor (Acesso restrito/controlado).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;li&gt;&lt;strong&gt;Infraestrutura e Compatibilidade&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Multiplataforma (Windows, Linux, UNIX).&lt;/li&gt;
+      &lt;li&gt;Superior aos sistemas legados (Integração e Internet).&lt;/li&gt;
     &lt;/ul&gt;
   &lt;/li&gt;
   &lt;li&gt;&lt;strong&gt;Objetivo Primordial&lt;/strong&gt;
@@ -6974,7 +7080,7 @@
         </is>
       </c>
       <c r="F165" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G165" t="n">
         <v>7</v>
@@ -7407,7 +7513,7 @@
         <v>0</v>
       </c>
       <c r="G172" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="173">
@@ -7487,7 +7593,7 @@
         <v>0</v>
       </c>
       <c r="G173" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="174">
@@ -7663,7 +7769,7 @@
         <v>0</v>
       </c>
       <c r="G176" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="177">
@@ -7707,13 +7813,18 @@
   &lt;li&gt;ente público pode utilizar ferramentas de outro ente&lt;/li&gt;
   &lt;li&gt;requisitos das ferramentas
     &lt;ul&gt;
-      &lt;li&gt;garantir segurança, transparência e confiabilidade&lt;/li&gt;
-      &lt;li&gt;comprovar autoria&lt;/li&gt;
-      &lt;li&gt;registrar emissão e recebimento&lt;/li&gt;
+      &lt;li&gt;garantir segurança, transparência e proteção de dados&lt;/li&gt;
+      &lt;li&gt;comprovar autoria e integridade&lt;/li&gt;
+      &lt;li&gt;registrar emissão e recebimento
+&lt;ul&gt;
+          &lt;li&gt;data e hora&lt;/li&gt;
+          &lt;li&gt;ainda que não de leitura&lt;/li&gt;
+        &lt;/ul&gt;
+&lt;/li&gt;
       &lt;li&gt;passíveis de auditoria&lt;/li&gt;
       &lt;li&gt;preservar dados
         &lt;ul&gt;
-          &lt;li&gt;mínimo de cinco anos&lt;/li&gt;
+          &lt;li&gt;$\ge 5$ anos&lt;/li&gt;
         &lt;/ul&gt;
       &lt;/li&gt;
     &lt;/ul&gt;
@@ -7730,12 +7841,14 @@
         <v>0</v>
       </c>
       <c r="G177" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="n">
-        <v>267</v>
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>267</t>
+        </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -7804,7 +7917,7 @@
   &lt;/li&gt;
   &lt;li&gt;difusão de conhecimento
     &lt;ul&gt;
-      &lt;li&gt;modernização e disseminação de práticas inovadoras&lt;/li&gt;
+      &lt;li&gt;modernização e disseminação de práticas inovadoras &lt;b&gt;no setor público&lt;/b&gt;&lt;/li&gt;
     &lt;/ul&gt;
   &lt;/li&gt;
 &lt;/ul&gt;</t>
@@ -7814,7 +7927,7 @@
         <v>0</v>
       </c>
       <c r="G178" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="179">
@@ -7848,12 +7961,19 @@
   &lt;/li&gt;
   &lt;li&gt;Governança
     &lt;ul&gt;
-      &lt;li&gt;autoridade competente deve implementar&lt;/li&gt;
-      &lt;li&gt;mecanismos devem assegurar
-        &lt;ul&gt;
-          &lt;li&gt;acompanhamento de resultados&lt;/li&gt;
-          &lt;li&gt;soluções de desempenho organizacional&lt;/li&gt;
-          &lt;li&gt;decisões fundamentadas em evidências&lt;/li&gt;
+      &lt;li&gt;autoridade competente deve implementar mecanismos, instâncias e práticas
+        &lt;ul&gt;
+          &lt;li&gt;devem assegurar no mínimo
+            &lt;ul&gt;
+              &lt;li&gt;acompanhamento de resultados&lt;/li&gt;
+              &lt;li&gt;soluções para melhoria do desempenho das organizações
+                &lt;ul&gt;
+                  &lt;li&gt;diretrizes e indicadores&lt;/li&gt;
+                &lt;/ul&gt;
+              &lt;/li&gt;
+              &lt;li&gt;decisões fundamentadas em evidências&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
         &lt;/ul&gt;
       &lt;/li&gt;
     &lt;/ul&gt;
@@ -7892,7 +8012,7 @@
         <v>0</v>
       </c>
       <c r="G179" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="180">
@@ -7996,7 +8116,7 @@
         <v>0</v>
       </c>
       <c r="G180" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="181">
@@ -8254,7 +8374,7 @@
         <v>0</v>
       </c>
       <c r="G185" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="186">
@@ -8333,7 +8453,7 @@
         <v>0</v>
       </c>
       <c r="G186" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="187">
@@ -8367,7 +8487,7 @@
         <v>0</v>
       </c>
       <c r="G187" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="188">
@@ -8533,7 +8653,7 @@
         <v>0</v>
       </c>
       <c r="G190" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="191">
@@ -8644,7 +8764,7 @@
         <v>0</v>
       </c>
       <c r="G192" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193">
@@ -8678,7 +8798,7 @@
         <v>0</v>
       </c>
       <c r="G193" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="194">
@@ -8794,7 +8914,7 @@
         <v>0</v>
       </c>
       <c r="G194" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195">
@@ -9624,7 +9744,7 @@
         <v>0</v>
       </c>
       <c r="G203" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="204">
@@ -9761,7 +9881,7 @@
         <v>0</v>
       </c>
       <c r="G205" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="206">
@@ -9884,7 +10004,7 @@
         <v>0</v>
       </c>
       <c r="G207" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="208">
@@ -10081,7 +10201,7 @@
         <v>0</v>
       </c>
       <c r="G210" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="211">
@@ -10272,7 +10392,7 @@
         <v>0</v>
       </c>
       <c r="G213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="214">
@@ -11044,7 +11164,7 @@
         <v>0</v>
       </c>
       <c r="G222" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="223">
@@ -12664,7 +12784,7 @@
         <v>0</v>
       </c>
       <c r="G236" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="237">
@@ -14081,7 +14201,7 @@
         <v>0</v>
       </c>
       <c r="G247" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="248">
@@ -14504,7 +14624,7 @@
         <v>0</v>
       </c>
       <c r="G254" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="255">
@@ -14633,7 +14753,7 @@
         <v>0</v>
       </c>
       <c r="G256" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="257">
@@ -15433,12 +15553,14 @@
         <v>0</v>
       </c>
       <c r="G270" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="271">
-      <c r="A271" t="n">
-        <v>365</v>
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>365</t>
+        </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
@@ -15469,6 +15591,7 @@
     &lt;ul&gt;
       &lt;li&gt;&lt;strong&gt;Sistemas em Série:&lt;/strong&gt; A falha de um item interrompe o sistema.
         &lt;ul&gt;
+&lt;li&gt;&lt;strong&gt;Todos&lt;/strong&gt; os componentes são essenciais para o sistema.&lt;/li&gt;
           &lt;li&gt;Confiabilidade: $R_s = R_1 \cdot R_2 \cdot ... \cdot R_n$&lt;/li&gt;
           &lt;li&gt;Taxa de Falha: $\lambda_{sist} = \sum \lambda_i$&lt;/li&gt;
         &lt;/ul&gt;
@@ -15494,7 +15617,7 @@
         <v>0</v>
       </c>
       <c r="G271" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="272">
@@ -15547,7 +15670,7 @@
         <v>0</v>
       </c>
       <c r="G272" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="273">
@@ -15641,7 +15764,7 @@
         <v>0</v>
       </c>
       <c r="G274" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="275">
@@ -15864,8 +15987,10 @@
       </c>
     </row>
     <row r="279">
-      <c r="A279" t="n">
-        <v>373</v>
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>373</t>
+        </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
@@ -15879,35 +16004,50 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Equivalente de Produção e Custeio por Processo</t>
+          <t>Custeio por Processo e Equivalente de Produção (EP)</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-  &lt;li&gt;&lt;strong&gt;Conceito de Equivalente de Produção (EP)&lt;/strong&gt;
-    &lt;ul&gt;
-      &lt;li&gt;É a tradução do estoque em processamento (WIP) em unidades acabadas.&lt;/li&gt;
-      &lt;li&gt;&lt;strong&gt;Fórmula:&lt;/strong&gt; $$EP = Qtd.\ Acabada + (Qtd.\ em\ Processo \cdot \%Acabamento)$$&lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;&lt;strong&gt;Lógica PEPS (FIFO) no Custeio por Processo&lt;/strong&gt;
-    &lt;ul&gt;
-      &lt;li&gt;O custo do período deve ser dividido apenas pelo &lt;u&gt;esforço realizado no período&lt;/u&gt;.&lt;/li&gt;
-      &lt;li&gt;&lt;strong&gt;Cálculo do EP (PEPS):&lt;/strong&gt;
-        &lt;ol&gt;
-          &lt;li&gt;Esforço para terminar o estoque inicial (Ex: se iniciou 75% pronto, falta 25%).&lt;/li&gt;
-          &lt;li&gt;Unidades iniciadas e terminadas no próprio mês.&lt;/li&gt;
-          &lt;li&gt;Esforço realizado no estoque final (Ex: 80 unidades a 75% = 60 EP).&lt;/li&gt;
-        &lt;/ol&gt;
-      &lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
-  &lt;li&gt;&lt;strong&gt;Regra de Ouro (CPA - Custo da Produção Acabada)&lt;/strong&gt;
-    &lt;ul&gt;
-      &lt;li&gt;O custo total das unidades que saíram da fábrica é a soma do custo que elas já traziam do mês anterior + o custo adicionado para finalizá-las no mês atual.&lt;/li&gt;
-    &lt;/ul&gt;
-  &lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Sistemas de Acumulação&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Contínuo (Processo): Uso de EP é obrigatório para avaliar o WIP (Work in Progress / Trabalho em Processo).&lt;/li&gt;
+			&lt;li&gt;Discreto (Ordens): Custos acumulados na OP (Ordem de Produção) sem necessidade de EP.&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Cálculo do EP Total&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Lógica: Soma das unidades prontas com a "fatia" equivalente das unidades incompletas.&lt;/li&gt;
+			&lt;li&gt;Fórmulas Compactas:
+				&lt;ul&gt;
+					&lt;li&gt;&lt;b&gt;CM (Custo Médio):&lt;/b&gt; $EP = UA + (UEP \cdot \%A)$&lt;/li&gt;
+					&lt;li&gt;&lt;b&gt;PEPS (Primeiro que Entra, Primeiro que Sai / FIFO - First-In, First-Out):&lt;/b&gt; $EP = (EI \cdot \%F) + IT + (EF \cdot \%A)$&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Legenda das Fórmulas:
+				&lt;ul&gt;
+					&lt;li&gt;$UA$: Unidades Acabadas; $UEP$: Unidades em Processo; $\%A$: Grau de Acabamento.&lt;/li&gt;
+					&lt;li&gt;$EI$: Estoque Inicial; $\%F$: Porcentagem que falta fazer; $IT$: Iniciadas e Terminadas; $EF$: Estoque Final.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Distribuição de Custos (Regra de Ouro)&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Custo Unitário ($CU$): $CU = \frac{CPP}{EP \text{ Total}}$
+				&lt;ul&gt;
+					&lt;li&gt;$CPP$: Custo de Produção do Período.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Destino dos Custos:
+				&lt;ul&gt;
+					&lt;li&gt;CPA (Custo da Produção Acabada): $UA \cdot CU$.&lt;/li&gt;
+					&lt;li&gt;CPPP (Custo da Produção de Produtos em Processo): $(UEP \cdot \%A) \cdot CU$.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
 &lt;/ul&gt;</t>
         </is>
       </c>
@@ -15915,7 +16055,7 @@
         <v>0</v>
       </c>
       <c r="G279" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="280">
@@ -15971,7 +16111,7 @@
         <v>0</v>
       </c>
       <c r="G280" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="281">
@@ -16248,7 +16388,7 @@
         <v>0</v>
       </c>
       <c r="G285" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="286">
@@ -16360,7 +16500,7 @@
         <v>0</v>
       </c>
       <c r="G287" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="288">
@@ -16828,7 +16968,7 @@
         <v>0</v>
       </c>
       <c r="G296" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="297">
@@ -16920,7 +17060,7 @@
         <v>0</v>
       </c>
       <c r="G298" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="299">
@@ -16957,7 +17097,7 @@
         <v>0</v>
       </c>
       <c r="G299" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="300">
@@ -17018,7 +17158,7 @@
         <v>0</v>
       </c>
       <c r="G300" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="301">
@@ -17250,7 +17390,7 @@
         <v>0</v>
       </c>
       <c r="G304" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="305">
@@ -17295,15 +17435,17 @@
         </is>
       </c>
       <c r="F305" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G305" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="306">
-      <c r="A306" t="n">
-        <v>400</v>
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
@@ -17323,30 +17465,34 @@
       <c r="E306" t="inlineStr">
         <is>
           <t>&lt;ul&gt;
-	&lt;li&gt;&lt;strong&gt;Estrutura e Validade&lt;/strong&gt;
+	&lt;li&gt;&lt;b&gt;Estrutura e Validade&lt;/b&gt;
 		&lt;ul&gt;
-			&lt;li&gt;Definição: Conjunto de Premissas ($P_1, P_2, ...$) $\to$ Conclusão ($C$).&lt;/li&gt;
-			&lt;li&gt;Argumento Válido: A verdade das premissas **obriga** a verdade da conclusão.
+			&lt;li&gt;Definição: Conjunto de Premissas ($P_1, P_2, \dots$) $\to$ Conclusão ($C$).&lt;/li&gt;
+			&lt;li&gt;Argumento:
 				&lt;ul&gt;
-					&lt;li&gt;$(P_1 \land P_2 \land ...) \to C$ é uma Tautologia.&lt;/li&gt;
-				&lt;/ul&gt;
-			&lt;/li&gt;
-			&lt;li&gt;Argumento Inválido (Falácia/Sofisma): É possível ter premissas (V) e conclusão (F).&lt;/li&gt;
-		&lt;/ul&gt;
-	&lt;/li&gt;
-	&lt;li&gt;&lt;strong&gt;Técnica de Validação (Método das Premissas Verdadeiras)&lt;/strong&gt;
-		&lt;ul&gt;
-			&lt;li&gt;Passo 1: Assuma que a Conclusão é &lt;strong&gt;Falsa&lt;/strong&gt;.&lt;/li&gt;
-			&lt;li&gt;Passo 2: Tente tornar todas as Premissas &lt;strong&gt;Verdadeiras&lt;/strong&gt;.&lt;/li&gt;
-			&lt;li&gt;Análise do Resultado:
-				&lt;ul&gt;
-					&lt;li&gt;Conseguiu (Sem contradição) $\to$ &lt;strong&gt;Inválido&lt;/strong&gt;.&lt;/li&gt;
-					&lt;li&gt;Houve contradição (Premissa forçada a ser F) $\to$ &lt;strong&gt;Válido&lt;/strong&gt;.&lt;/li&gt;
+					&lt;li&gt;Válido: A verdade das premissas &lt;b&gt;obriga&lt;/b&gt; a verdade da conclusão.
+						&lt;ul&gt;
+							&lt;li&gt;$(P_1 \land P_2 \land \dots) \to C$ é uma Tautologia.&lt;/li&gt;
+						&lt;/ul&gt;
+					&lt;/li&gt;
+					&lt;li&gt;Inválido (Falácia/Sofisma): É possível ter premissas (V) e conclusão (F).&lt;/li&gt;
 				&lt;/ul&gt;
 			&lt;/li&gt;
 		&lt;/ul&gt;
 	&lt;/li&gt;
-	&lt;li&gt;&lt;strong&gt;Regras de Inferência Rápidas&lt;/strong&gt;
+	&lt;li&gt;&lt;b&gt;Técnica de Validação (Método das Premissas Verdadeiras)&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Passo 1: Assuma que a Conclusão é &lt;b&gt;Falsa&lt;/b&gt;.&lt;/li&gt;
+			&lt;li&gt;Passo 2: Tente tornar todas as Premissas &lt;b&gt;Verdadeiras&lt;/b&gt;.&lt;/li&gt;
+			&lt;li&gt;Análise do Resultado:
+				&lt;ul&gt;
+					&lt;li&gt;Sucesso (Sem contradição) $\implies$ &lt;b&gt;Inválido&lt;/b&gt;.&lt;/li&gt;
+					&lt;li&gt;Contradição (Premissa forçada a ser F) $\implies$ &lt;b&gt;Válido&lt;/b&gt;.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Regras de Inferência Rápidas&lt;/b&gt;
 		&lt;ul&gt;
 			&lt;li&gt;Modus Ponens: $(p \to q) \land p \implies q$.&lt;/li&gt;
 			&lt;li&gt;Modus Tollens: $(p \to q) \land \neg q \implies \neg p$.&lt;/li&gt;
@@ -17360,7 +17506,7 @@
         <v>0</v>
       </c>
       <c r="G306" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="307">
@@ -17413,7 +17559,7 @@
         <v>0</v>
       </c>
       <c r="G307" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="308">
@@ -17485,6 +17631,1735 @@
         <v>0</v>
       </c>
       <c r="G308" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>403</v>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Regência Verbal e Nominal; e Crase</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Casos Obrigatórios e Específicos de Crase</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;Locuções Adverbiais Femininas (Modo, Tempo, Lugar)
+		&lt;ul&gt;
+			&lt;li&gt;Obrigatória para evitar ambiguidade.&lt;/li&gt;
+			&lt;li&gt;Ex: às cegas, à deriva, à noite, à direita, às vezes, à mão.&lt;/li&gt;
+			&lt;li&gt;Diferenciação: "Lavar a mão" (corpo) vs. "Lavar à mão" (modo).&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;Horas Exatas
+		&lt;ul&gt;
+			&lt;li&gt;Regra: Obrigatória em horas determinadas. Ex: "Às 10 horas".&lt;/li&gt;
+			&lt;li&gt;Exceção: Com preposição anterior (até, desde, para, após) &lt;strong&gt;não&lt;/strong&gt; ocorre crase.
+				&lt;ul&gt;
+					&lt;li&gt;Ex: "Desde as 8h", "Para as 14h".&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;Locuções Prepositivas e Conjuntivas
+		&lt;ul&gt;
+			&lt;li&gt;Prepositivas (a + fem. + de): à espera de, à procura de, à frente de.&lt;/li&gt;
+			&lt;li&gt;Conjuntivas (proporção): à medida que, à proporção que.&lt;/li&gt;
+			&lt;li&gt;&lt;strong&gt;Alerta Cebraspe:&lt;/strong&gt; Não existe "à medida em que".&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;Expressão "À moda de" (Mesmo com masculinas)
+		&lt;ul&gt;
+			&lt;li&gt;Ocorre quando a expressão está implícita.&lt;/li&gt;
+			&lt;li&gt;Ex: Gol à Pelé (à moda de Pelé).&lt;/li&gt;
+			&lt;li&gt;Ex: Bife à milanesa (à moda de Milão).&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F309" t="n">
+        <v>0</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>404</v>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>5S</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;&lt;strong&gt;Seiri (Utilização / Senso de Uso)&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Ação: Separar o necessário do desnecessário.&lt;/li&gt;
+			&lt;li&gt;Objetivo: Eliminar desperdícios, ferramentas obsoletas e materiais em excesso.&lt;/li&gt;
+			&lt;li&gt;Foco: Libertar espaço e reduzir custos de armazenamento.&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;strong&gt;Seiton (Ordenação / Senso de Organização)&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Ação: Definir um lugar específico para cada item necessário.&lt;/li&gt;
+			&lt;li&gt;Princípio: "Um lugar para cada coisa e cada coisa no seu lugar."&lt;/li&gt;
+			&lt;li&gt;Foco: Rapidez no acesso e redução de tempos de movimentação/procura.&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;strong&gt;Seiso (Limpeza / Senso de Limpeza)&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Ação: Eliminar a sujidade e as fontes de contaminação.&lt;/li&gt;
+			&lt;li&gt;&lt;strong&gt;Conexão TPM:&lt;/strong&gt; A limpeza deve ser encarada como uma forma de inspeção.&lt;/li&gt;
+			&lt;li&gt;Foco: Manutenção da integridade física e deteção precoce de falhas.&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;strong&gt;Seiketsu (Normalização / Senso de Saúde)&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Ação: Padronizar as práticas e manter a higiene física e mental.&lt;/li&gt;
+			&lt;li&gt;Objetivo: Criar regras e sinalizações para sustentar os três primeiros S.&lt;/li&gt;
+			&lt;li&gt;Foco: Segurança, bem-estar e preservação do ambiente de trabalho.&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;strong&gt;Shitsuke (Autodisciplina / Senso de Disciplina)&lt;/strong&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Ação: Tornar os procedimentos um hábito e uma responsabilidade partilhada.&lt;/li&gt;
+			&lt;li&gt;Objetivo: Sustentabilidade do programa a longo prazo sem necessidade de vigilância.&lt;/li&gt;
+			&lt;li&gt;Foco: Melhoria contínua (Kaizen) e mudança de cultura organizacional.&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>0</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>405</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Gestão da Manutenção e Confiabilidade</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>FMECA (Failure Mode, Effects and Criticality Analysis - Análise de Modos de Falha, Efeitos e Criticidade)</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Conceito:&lt;/b&gt; Técnica &lt;b&gt;qualitativa ou semi-quantitativa&lt;/b&gt; e indutiva (&lt;i&gt;bottom-up&lt;/i&gt; / de baixo para cima) que identifica a função de cada componente, seus potenciais modos de falha, efeitos e causas, realizando uma classificação baseada em graus de criticidade.&lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Objeto da Classificação (Ponto Vital):&lt;/b&gt; O FMECA é utilizado para classificar os &lt;b&gt;&lt;u&gt;modos e efeitos de falhas críticas&lt;/u&gt;&lt;/b&gt;. 
+    &lt;ul&gt;
+      &lt;li&gt;&lt;b&gt;Nota:&lt;/b&gt; Não classifica apenas "componentes críticos" de forma genérica, mas o binômio &lt;i&gt;Modo de Falha + Efeito&lt;/i&gt;.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;RPN (Risk Priority Number / Número de Prioridade de Risco):&lt;/b&gt; Índice usado para priorizar as ações de manutenção.
+    &lt;ul&gt;
+      &lt;li&gt;&lt;b&gt;Fórmula:&lt;/b&gt; $$RPN = S \times O \times D$$&lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;S (Severidade):&lt;/b&gt; Gravidade do efeito da falha no sistema/segurança.&lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;O (Ocorrência):&lt;/b&gt; Probabilidade ou frequência da causa da falha.&lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;D (Detecção):&lt;/b&gt; Eficácia dos controles em perceber a falha antes que ela gere o efeito.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Matriz de Criticidade:&lt;/b&gt; Diferencial em relação ao &lt;b&gt;FMEA&lt;/b&gt; (Failure Mode and Effects Analysis / Análise de Modos e Efeitos de Falha), pois cruza a &lt;u&gt;Probabilidade de Ocorrência&lt;/u&gt; com a &lt;u&gt;Severidade do Efeito&lt;/u&gt; para gerar um ranking visual de risco.&lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;RCM (Reliability-Centered Maintenance / Manutenção Centrada na Confiabilidade):&lt;/b&gt; Ferramenta essencial para decidir a estratégia de manutenção (preventiva, preditiva ou corretiva) com base na criticidade da falha definida no FMECA.&lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Aplicações:&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Identificação de &lt;b&gt;Pontos Únicos de Falha&lt;/b&gt; (Single Points of Failure / Ponto Único de Falha).&lt;/li&gt;
+      &lt;li&gt;Otimização de recursos focando no que realmente compromete a operação.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Norma de Referência:&lt;/b&gt; &lt;b&gt;MIL-STD-1629A&lt;/b&gt; (Padrão Militar para FMECA).&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>0</v>
+      </c>
+      <c r="G311" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>406</v>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Sistemas Legados</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Conceito:&lt;/strong&gt; Sistemas de informação antigos, tecnologias obsoletas ou métodos de processamento ultrapassados que continuam em uso por serem essenciais para a operação.&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Características Técnicas:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Dificuldade de integração com tecnologias modernas (ex: Internet/Web).&lt;/li&gt;
+      &lt;li&gt;Arquitetura geralmente monolítica ou baseada em mainframes.&lt;/li&gt;
+      &lt;li&gt;Dependência de hardware específico e software de manutenção escassa.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Problemas Operacionais:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Ilhas de Informação:&lt;/strong&gt; Dados fragmentados e isolados entre departamentos (contrário ao ERP).&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Redundância:&lt;/strong&gt; Mesma informação armazenada em múltiplos locais, gerando inconsistência.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Custo Elevado:&lt;/strong&gt; Manutenção cara devido à falta de profissionais especializados (ex: programadores COBOL - Common Business Oriented Language / Linguagem Comum Orientada a Negócios).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;ERP vs. Sistemas Legados:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;O ERP (Enterprise Resource Planning — Planeamento de Recursos Empresariais) substitui múltiplos sistemas legados por uma única base de dados centralizada.&lt;/li&gt;
+      &lt;li&gt;ERP é multi-plataforma e utiliza protocolos modernos; o legado é frequentemente restrito a uma única plataforma/SO (Sistema Operativo).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F312" t="n">
+        <v>0</v>
+      </c>
+      <c r="G312" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>407</v>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Gestão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Classificação da Informação (Lesca / Choo)</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Sem interesse&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Irrelevância.&lt;/li&gt;
+      &lt;li&gt;Ruído.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Potencial&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Utilidade futura.&lt;/li&gt;
+      &lt;li&gt;Dispensa de ação imediata.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Mínima&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Operacionalidade obrigatória.&lt;/li&gt;
+      &lt;li&gt;Funcionamento básico.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Crítica&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Estratégia essencial.&lt;/li&gt;
+      &lt;li&gt;Sucesso e diferenciação.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F313" t="n">
+        <v>0</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>408</v>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Probabilidade Condicional</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;&lt;b&gt;Definição&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Conceito: Probabilidade de um evento $A$ ocorrer, dado que um evento $B$ já ocorreu (restrição do espaço amostral).&lt;/li&gt;
+			&lt;li&gt;Notação: $P(A|B)$, lê-se "probabilidade de $A$ dado $B$".&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Fórmula Geral&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Cálculo: $P(A|B) = \frac{P(A \cap B)}{P(B)}$, onde $P(B) &gt; 0$.&lt;/li&gt;
+			&lt;li&gt;Interpretação dos termos:
+				&lt;ul&gt;
+					&lt;li&gt;$P(A \cap B)$: Interseção (ocorrência simultânea de $A$ e $B$).&lt;/li&gt;
+					&lt;li&gt;$P(B)$: Probabilidade do evento condicionante (o que já aconteceu).&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Teorema do Produto (Regra da Multiplicação)&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Derivação: $P(A \cap B) = P(B) \cdot P(A|B)$.&lt;/li&gt;
+			&lt;li&gt;Aplicação: Utilizada para calcular a probabilidade da interseção em eventos dependentes.&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Eventos Independentes&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Condição: A ocorrência de $B$ não altera a probabilidade de $A$.
+				&lt;ul&gt;
+					&lt;li&gt;$P(A|B) = P(A)$.&lt;/li&gt;
+					&lt;li&gt;$P(A \cap B) = P(A) \cdot P(B)$.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>0</v>
+      </c>
+      <c r="G314" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>409</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Igualdade de Conjuntos vs. Igualdade de Probabilidades (ICVP)</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;&lt;b&gt;Diferenciação Fundamental&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Igualdade de Conjuntos ($A = B$):
+				&lt;ul&gt;
+					&lt;li&gt;Condição: Possuem exatamente os mesmos elementos.&lt;/li&gt;
+					&lt;li&gt;Implicação: Se $A = B \implies P(A) = P(B)$.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Igualdade de Probabilidades ($P(A) = P(B)$):
+				&lt;ul&gt;
+					&lt;li&gt;Condição: Possuem a mesma medida numérica de chance.&lt;/li&gt;
+					&lt;li&gt;Aviso: &lt;b&gt;Não&lt;/b&gt; implica que os conjuntos sejam iguais ($A \neq B$ pode ocorrer).&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Armadilha de Equivalência Numérica&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Cenário: $P(B) = P(A^c)$ indica apenas que os valores são numericamente idênticos.&lt;/li&gt;
+			&lt;li&gt;Erro Lógico: Assumir que o conjunto $B$ &lt;b&gt;é&lt;/b&gt; o conjunto $A^c$.&lt;/li&gt;
+			&lt;li&gt;Fato: Dois conjuntos podem ter o mesmo "tamanho" (probabilidade) e estarem em locais completamente diferentes do Espaço Amostral (S).&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Exemplo Analógico (Dado de 6 faces)&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Evento $X$ (Sair face 1): $P(X) = 1/6$.&lt;/li&gt;
+			&lt;li&gt;Evento $Y$ (Sair face 6): $P(Y) = 1/6$.&lt;/li&gt;
+			&lt;li&gt;Conclusão: $P(X) = P(Y)$, mas o conjunto $\{1\} \neq \{6\}$. Eles são eventos disjuntos com a mesma probabilidade.&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>0</v>
+      </c>
+      <c r="G315" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>410</v>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Raciocínio Lógico</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Relações e Operações em Probabilidade</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;&lt;b&gt;Relações de Conjuntos e Inclusão&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Contido ($B \subset A$): Todo elemento de $B$ pertence a $A$.
+				&lt;ul&gt;
+					&lt;li&gt;Probabilidade: $P(B) \le P(A)$.&lt;/li&gt;
+					&lt;li&gt;Interseção: $P(A \cap B) = P(B)$.&lt;/li&gt;
+					&lt;li&gt;União: $P(A \cup B) = P(A)$.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Mutuamente Excluentes (Disjuntos): Não possuem elementos em comum.
+				&lt;ul&gt;
+					&lt;li&gt;Interseção: $A \cap B = \emptyset \implies P(A \cap B) = 0$.&lt;/li&gt;
+					&lt;li&gt;União: $P(A \cup B) = P(A) + P(B)$.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Operações Fundamentais&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;União ($A \cup B$): Ocorrência de pelo menos um dos eventos.
+				&lt;ul&gt;
+					&lt;li&gt;Regra Geral: $P(A \cup B) = P(A) + P(B) - P(A \cap B)$.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Interseção ($A \cap B$): Ocorrência simultânea de ambos.
+				&lt;ul&gt;
+					&lt;li&gt;Cálculo via Probabilidade Condicional: $P(A \cap B) = P(A) \cdot P(B|A)$.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Dependência vs. Independência&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Eventos Independentes: A ocorrência de um não afeta o outro.
+				&lt;ul&gt;
+					&lt;li&gt;Condição: $P(A|B) = P(A)$.&lt;/li&gt;
+					&lt;li&gt;Interseção Simplificada: $P(A \cap B) = P(A) \cdot P(B)$.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;Eventos Dependentes: A ocorrência de um altera a probabilidade do outro.
+				&lt;ul&gt;
+					&lt;li&gt;Condição: $P(A|B) \neq P(A)$.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Complementariedade&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Evento Complementar ($A^c$ ou $\bar{A}$): Tudo o que não é $A$.
+				&lt;ul&gt;
+					&lt;li&gt;Soma: $P(A) + P(A^c) = 1$.&lt;/li&gt;
+					&lt;li&gt;Leis de De Morgan:
+						&lt;ul&gt;
+							&lt;li&gt;$P(A \cup B)^c = P(A^c \cap B^c)$.&lt;/li&gt;
+							&lt;li&gt;$P(A \cap B)^c = P(A^c \cup B^c)$.&lt;/li&gt;
+						&lt;/ul&gt;
+					&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>0</v>
+      </c>
+      <c r="G316" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>411</v>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Sistemas de Acumulação de Custos</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Produção Conjunta (PC)</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Classificação e Tratamento na PC&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;b&gt;Coprodutos:&lt;/b&gt; Produtos principais com alto valor de venda.
+        &lt;ul&gt;
+          &lt;li&gt;Custo: Recebem obrigatoriamente o rateio dos custos conjuntos (Método do Valor de Venda ou Volume).&lt;/li&gt;
+          &lt;li&gt;Lógica de Prova: Se não houver estoque final, o rateio é dispensável para o resultado, pois todo custo vira despesa no período.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Subprodutos:&lt;/b&gt; Itens com venda recorrente, mas de baixo valor.
+        &lt;ul&gt;
+          &lt;li&gt;Custo: &lt;b&gt;Não&lt;/b&gt; recebem rateio de custos.&lt;/li&gt;
+          &lt;li&gt;Contabilidade: Seu VRL (Valor Realizável Líquido / Net Realizable Value - Valor Realizável Líquido) é deduzido do custo do produto principal.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Sucatas:&lt;/b&gt; Resíduos eventuais sem valor expressivo.
+        &lt;ul&gt;
+          &lt;li&gt;Custo: Não possuem custo atribuído.&lt;/li&gt;
+          &lt;li&gt;Contabilidade: A receita de venda é tratada como Outras Receitas Operacionais (não reduzem o custo de produção).&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Pontos de Separação (Split-off)&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Definição: Momento em que os produtos se tornam identificáveis individualmente.&lt;/li&gt;
+      &lt;li&gt;Custos Conjuntos: Gastos incorridos até o &lt;i&gt;split-off&lt;/i&gt; que devem ser distribuídos apenas entre os coprodutos.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F317" t="n">
+        <v>0</v>
+      </c>
+      <c r="G317" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>412</v>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Equivalentes de Produção</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Identificação de Métodos de Avaliação de Estoque (IMAE)</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+	&lt;li&gt;&lt;b&gt;Status do Estoque Inicial (EI - Estoque Inicial)&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;&lt;b&gt;EI nulo ($EI = 0$):&lt;/b&gt;
+				&lt;ul&gt;
+					&lt;li&gt;Gatilho: Termos como "produção iniciada no período" ou "primeiro mês de operação".&lt;/li&gt;
+					&lt;li&gt;Regra: Os métodos PEPS (Primeiro que Entra, Primeiro que Sai / FIFO - First-In, First-Out), UEPS (Último que Entra, Primeiro que Sai / LIFO - Last-In, First-Out) e CM (Custo Médio) resultam no &lt;b&gt;mesmo valor&lt;/b&gt;.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+			&lt;li&gt;&lt;b&gt;EI positivo ($EI &gt; 0$):&lt;/b&gt;
+				&lt;ul&gt;
+					&lt;li&gt;Regra: A banca é obrigatória a indicar o método. Caso seja omissa, o Custo Médio Ponderado Móvel é o padrão contábil brasileiro.&lt;/li&gt;
+				&lt;/ul&gt;
+			&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Termos Sinalizadores no Enunciado&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;&lt;b&gt;PEPS (FIFO):&lt;/b&gt; "Venda das unidades mais antigas" ou "valorização pelo custo das últimas entradas" (o que sobra no estoque é o mais novo).&lt;/li&gt;
+			&lt;li&gt;&lt;b&gt;UEPS (LIFO):&lt;/b&gt; "Venda das unidades mais recentes" ou "valorização pelo custo das primeiras entradas" (o que sobra no estoque é o mais antigo).&lt;/li&gt;
+			&lt;li&gt;&lt;b&gt;Custo Médio (CM):&lt;/b&gt; "Média ponderada", "custo unitário médio" ou "rateio proporcional aos custos totais".&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+	&lt;li&gt;&lt;b&gt;Impacto no Lucro (Contexto Inflacionário)&lt;/b&gt;
+		&lt;ul&gt;
+			&lt;li&gt;Maior Lucro / Maior Estoque Final: PEPS.&lt;/li&gt;
+			&lt;li&gt;Menor Lucro / Menor Estoque Final: UEPS.&lt;/li&gt;
+			&lt;li&gt;Resultado Intermediário: Custo Médio.&lt;/li&gt;
+		&lt;/ul&gt;
+	&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F318" t="n">
+        <v>0</v>
+      </c>
+      <c r="G318" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>413</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Autoridade Nacional de Proteção de Dados (ANPD) e Sanções Administrativa</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;ANPD&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;natureza jurídica
+        &lt;ul&gt;
+          &lt;li&gt;autarquia de natureza especial&lt;/li&gt;
+          &lt;li&gt;dotada de autonomia funcional, técnica, decisória, administrativa e financeira&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;vínculo
+        &lt;ul&gt;
+          &lt;li&gt;Ministério da Justiça e Segurança Pública&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;sanções administrativas&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;aplicação
+        &lt;ul&gt;
+          &lt;li&gt;exclusivamente pela &lt;b&gt;ANPD&lt;/b&gt;&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;medidas aplicáveis
+        &lt;ul&gt;
+          &lt;li&gt;advertência com fixação de prazo para adoção de medidas corretivas&lt;/li&gt;
+          &lt;li&gt;publicização da infração após devidamente apurada e confirmada&lt;/li&gt;
+          &lt;li&gt;bloqueio ou eliminação dos dados pessoais a que se refere a infração&lt;/li&gt;
+          &lt;li&gt;suspensão do funcionamento do banco de dados por até 6 meses, prorrogável&lt;/li&gt;
+          &lt;li&gt;proibição parcial ou total do exercício de atividades relacionadas a tratamento&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;penalidades financeiras
+        &lt;ul&gt;
+          &lt;li&gt;multa simples
+            &lt;ul&gt;
+              &lt;li&gt;até 2% do faturamento de pessoa jurídica de direito privado, grupo ou conglomerado no Brasil no seu último exercício, excluídos os tributos&lt;/li&gt;
+              &lt;li&gt;limitada a &lt;b&gt;R$ 50.000.000,00 por infração&lt;/b&gt;&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;multa diária
+            &lt;ul&gt;
+              &lt;li&gt;observará o limite total de &lt;b&gt;R$ 50.000.000,00&lt;/b&gt;&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F319" t="n">
+        <v>0</v>
+      </c>
+      <c r="G319" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>414</v>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Responsabilidade e Ressarcimento de Danos (LGPD)</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Responsabilidade civil
+    &lt;ul&gt;
+      &lt;li&gt;controlador ou operador que causar dano em razão do tratamento
+        &lt;ul&gt;
+          &lt;li&gt;obrigação de reparar danos patrimoniais, morais, individuais ou coletivos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Inversão do ônus da prova
+    &lt;ul&gt;
+      &lt;li&gt;poder facultativo do juiz no processo civil
+        &lt;ul&gt;
+          &lt;li&gt;não é automática&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;critérios para aplicação
+        &lt;ul&gt;
+          &lt;li&gt;verossimilhança da alegação&lt;/li&gt;
+          &lt;li&gt;hipossuficiência para produção de prova&lt;/li&gt;
+          &lt;li&gt;produção de prova pelo titular excessivamente onerosa&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F320" t="n">
+        <v>0</v>
+      </c>
+      <c r="G320" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>415</v>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Dados Pessoais Sensíveis (LGPD)</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Dados Pessoais Sensíveis&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Conceito
+        &lt;ul&gt;
+          &lt;li&gt;origem racial ou étnica&lt;/li&gt;
+          &lt;li&gt;convicção religiosa e opinião política&lt;/li&gt;
+          &lt;li&gt;filiação a sindicato ou a organização de caráter religioso, filosófico ou político&lt;/li&gt;
+          &lt;li&gt;dado referente à saúde ou à vida sexual&lt;/li&gt;
+          &lt;li&gt;dado genético ou biométrico&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Tratamento
+        &lt;ul&gt;
+          &lt;li&gt;não há vedação absoluta ao tratamento&lt;/li&gt;
+          &lt;li&gt;Hipóteses permitidas
+            &lt;ul&gt;
+              &lt;li&gt;Com consentimento do titular ou responsável
+                &lt;ul&gt;
+                  &lt;li&gt;deve ser específico e destacado&lt;/li&gt;
+                  &lt;li&gt;para finalidades específicas&lt;/li&gt;
+                &lt;/ul&gt;
+              &lt;/li&gt;
+              &lt;li&gt;Sem consentimento do titular
+                &lt;ul&gt;
+                  &lt;li&gt;cumprimento de obrigação legal ou regulatória&lt;/li&gt;
+                  &lt;li&gt;execução de políticas públicas pela administração pública&lt;/li&gt;
+                  &lt;li&gt;realização de estudos por órgão de pesquisa
+                    &lt;ul&gt;
+                      &lt;li&gt;garantida a anonimização sempre que possível&lt;/li&gt;
+                    &lt;/ul&gt;
+                  &lt;/li&gt;
+                  &lt;li&gt;exercício regular de direitos em contrato ou processos&lt;/li&gt;
+                  &lt;li&gt;proteção da vida ou da incolumidade física&lt;/li&gt;
+                  &lt;li&gt;tutela da saúde em procedimentos por profissionais ou autoridade sanitária&lt;/li&gt;
+                  &lt;li&gt;garantia da prevenção à fraude e à segurança do titular&lt;/li&gt;
+                &lt;/ul&gt;
+              &lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F321" t="n">
+        <v>0</v>
+      </c>
+      <c r="G321" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>416</v>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Definições e Conceitos (LGPD)</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Dado pessoal&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;informação relacionada a pessoa natural
+        &lt;ul&gt;
+          &lt;li&gt;identificada ou identificável&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Dado anonimizado&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;relativo a titular que não possa ser identificado
+        &lt;ul&gt;
+          &lt;li&gt;utilização de meios técnicos razoáveis e disponíveis na ocasião&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Banco de dados&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;conjunto estruturado de dados pessoais
+        &lt;ul&gt;
+          &lt;li&gt;estabelecido em um ou em vários locais&lt;/li&gt;
+          &lt;li&gt;suporte eletrônico ou físico&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F322" t="n">
+        <v>0</v>
+      </c>
+      <c r="G322" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>417</v>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Hipóteses de Tratamento (Dados Comuns)</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Tratamento de dados comuns (Art. 7º)&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;pode ser realizado sem o consentimento do titular
+        &lt;ul&gt;
+          &lt;li&gt;cumprimento de obrigação legal ou regulatória&lt;/li&gt;
+          &lt;li&gt;execução de políticas públicas pela administração&lt;/li&gt;
+          &lt;li&gt;realização de estudos por órgão de pesquisa
+            &lt;ul&gt;
+              &lt;li&gt;garantida a anonimização sempre que possível&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;execução de contrato ou procedimentos preliminares&lt;/li&gt;
+          &lt;li&gt;exercício regular de direitos em processos (judiciais, adm. ou arbitrais)&lt;/li&gt;
+          &lt;li&gt;proteção da vida ou da incolumidade física&lt;/li&gt;
+          &lt;li&gt;tutela da saúde (exclusivamente por profissionais ou serviços de saúde)&lt;/li&gt;
+          &lt;li&gt;interesse legítimo do controlador ou de terceiros
+            &lt;ul&gt;
+              &lt;li&gt;exceto se prevalecerem direitos e liberdades do titular&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;proteção do crédito&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F323" t="n">
+        <v>0</v>
+      </c>
+      <c r="G323" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>418</v>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Relatório de Impacto à Proteção de Dados Pessoais (RIPD)</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Relatório de Impacto à Proteção de Dados Pessoais (RIPD)&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Conceito
+        &lt;ul&gt;
+          &lt;li&gt;documentação do controlador com descrição dos processos de tratamento&lt;/li&gt;
+          &lt;li&gt;foco em riscos às liberdades civis e aos direitos fundamentais&lt;/li&gt;
+          &lt;li&gt;inclui medidas, salvaguardas e mecanismos de mitigação&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Conteúdo mínimo
+        &lt;ul&gt;
+          &lt;li&gt;descrição dos tipos de dados coletados&lt;/li&gt;
+          &lt;li&gt;metodologia utilizada para a coleta&lt;/li&gt;
+          &lt;li&gt;metodologia utilizada para a garantia da segurança das informações&lt;/li&gt;
+          &lt;li&gt;análise do controlador sobre medidas e salvaguardas adotadas&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Exigibilidade e Publicidade
+        &lt;ul&gt;
+          &lt;li&gt;elaboração determinada pela ANPD&lt;/li&gt;
+          &lt;li&gt;referente a operações de tratamento de dados
+            &lt;ul&gt;
+              &lt;li&gt;inclusive dados sensíveis&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;deve observar segredos comercial e industrial&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F324" t="n">
+        <v>0</v>
+      </c>
+      <c r="G324" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>419</v>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Não aplicabilidade da LGPD</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Hipóteses de não aplicação da lei&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Tratamento por pessoa natural
+        &lt;ul&gt;
+          &lt;li&gt;fins exclusivamente particulares e não econômicos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Fins exclusivamente jornalísticos e artísticos&lt;/li&gt;
+      &lt;li&gt;Fins exclusivamente acadêmicos
+        &lt;ul&gt;
+          &lt;li&gt;aplicam-se apenas as hipóteses de tratamento (dados comuns e sensíveis)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Fins exclusivos de segurança e repressão
+        &lt;ul&gt;
+          &lt;li&gt;segurança pública&lt;/li&gt;
+          &lt;li&gt;defesa nacional&lt;/li&gt;
+          &lt;li&gt;segurança do Estado&lt;/li&gt;
+          &lt;li&gt;atividades de investigação e repressão de infrações penais&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Dados provenientes de fora do território nacional
+        &lt;ul&gt;
+          &lt;li&gt;desde que não sejam objeto de uso compartilhado com agentes brasileiros&lt;/li&gt;
+          &lt;li&gt;desde que o país de proveniência proporcione grau de proteção adequado&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F325" t="n">
+        <v>0</v>
+      </c>
+      <c r="G325" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>420</v>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Agentes e Figuras da LGPD</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Titular&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;pessoa natural a quem se referem os dados pessoais&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Agentes de Tratamento&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;b&gt;Controlador&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;pessoa natural ou jurídica (pública ou privada)&lt;/li&gt;
+          &lt;li&gt;detém competência para decisões sobre o tratamento&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Operador&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;pessoa natural ou jurídica (pública ou privada)&lt;/li&gt;
+          &lt;li&gt;realiza o tratamento em nome do controlador&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Encarregado (DPO)&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;pessoa indicada pelo controlador e operador&lt;/li&gt;
+      &lt;li&gt;atua como canal de comunicação entre
+        &lt;ul&gt;
+          &lt;li&gt;controlador&lt;/li&gt;
+          &lt;li&gt;titulares dos dados&lt;/li&gt;
+          &lt;li&gt;Autoridade Nacional de Proteção de Dados (ANPD)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F326" t="n">
+        <v>0</v>
+      </c>
+      <c r="G326" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>421</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Lei nº 12.527-2011</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Diretrizes e Transparência (LAI)</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Diretrizes Fundamentais&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;publicidade como preceito geral&lt;/li&gt;
+      &lt;li&gt;sigilo como exceção&lt;/li&gt;
+      &lt;li&gt;gratuidade do acesso
+        &lt;ul&gt;
+          &lt;li&gt;isento de taxas, exceto custos de reprodução&lt;/li&gt;
+&lt;li&gt;&lt;b&gt;exceção:&lt;/b&gt; cobrança permitida &lt;b&gt;exclusivamente&lt;/b&gt; para ressarcimento de custos de reprodução e materiais&lt;/li&gt;
+          &lt;li&gt;isenção da exceção: requerente que declarar pobreza (sustento próprio/família)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;divulgação de informações de interesse público
+        &lt;ul&gt;
+          &lt;li&gt;independente de solicitações&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+&lt;li&gt;uso de meios de comunicação viabilizados pela tecnologia da informação&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;li&gt;&lt;b&gt;Abrangência do Acesso (Art. 7º)&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Direitos de obter informações sobre:
+        &lt;ul&gt;
+          &lt;li&gt;orientação sobre procedimentos e atividades dos órgãos&lt;/li&gt;
+          &lt;li&gt;implementação, acompanhamento e resultados de programas e projetos&lt;/li&gt;
+          &lt;li&gt;&lt;b&gt;Resultado de inspeções, auditorias e contas&lt;/b&gt;
+            &lt;ul&gt;
+              &lt;li&gt;&lt;b&gt;Ressalva:&lt;/b&gt; não é "qualquer" resultado (exclui sigilosas e as pendentes de ato decisório)&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Tipos de Transparência&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Transparência Ativa
+        &lt;ul&gt;
+          &lt;li&gt;divulgação espontânea em sítios oficiais&lt;/li&gt;
+          &lt;li&gt;obrigatória para órgãos públicos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Transparência Passiva
+        &lt;ul&gt;
+          &lt;li&gt;atendimento a pedidos específicos (via SIC)&lt;/li&gt;
+          &lt;li&gt;proibição de exigências que inviabilizem o pedido&lt;/li&gt;
+          &lt;li&gt;vedação de exigir os motivos da solicitação&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F327" t="n">
+        <v>0</v>
+      </c>
+      <c r="G327" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>422</v>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Lei nº 12.527-2011</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Procedimento e Prazos de Acesso (LAI)</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Resposta ao Pedido&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;se disponível: acesso imediato&lt;/li&gt;
+      &lt;li&gt;se não disponível imediatamente
+        &lt;ul&gt;
+          &lt;li&gt;prazo: 20 dias&lt;/li&gt;
+          &lt;li&gt;prorrogação: + 10 dias (mediante justificativa expressa)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Negativa de Acesso&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;deve indicar razões e fundamento legal&lt;/li&gt;
+      &lt;li&gt;deve informar sobre possibilidade de recurso&lt;/li&gt;
+      &lt;li&gt;comunicar possibilidade de desclassificação (se for o caso)&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F328" t="n">
+        <v>0</v>
+      </c>
+      <c r="G328" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>423</v>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Lei nº 12.527-2011</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Classificação e Graus de Sigilo (LAI)</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Informação Sigilosa&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;imprescindível à segurança da sociedade ou do Estado&lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Graus e Prazos de Sigilo&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;Ultrassecreta: 25 anos (renovável uma única vez)&lt;/li&gt;
+          &lt;li&gt;Secreta: 15 anos&lt;/li&gt;
+          &lt;li&gt;Reservada: 5 anos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;contagem do prazo: a partir da data de sua produção&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Competência para Classificação (Federal)&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Ultrassecreta: Presidente, Vice, Ministros e equivalentes, Comandantes militares e Chefes de missões diplomáticas&lt;/li&gt;
+      &lt;li&gt;Secreta: mesmas da ultrassecreta + titulares de autarquias/fundações e servidores de alto escalão (DAS 101.6)&lt;/li&gt;
+      &lt;li&gt;Reservada: mesmas das anteriores + servidores DAS 101.5 ou superior&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F329" t="n">
+        <v>0</v>
+      </c>
+      <c r="G329" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="n">
+        <v>424</v>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Lei nº 12.527-2011</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Recursos e Instâncias (Âmbito Federal - LAI)</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Recurso por Negativa de Acesso&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;prazo para o interessado recorrer: 10 dias&lt;/li&gt;
+      &lt;li&gt;prazo para a autoridade decidir: 5 dias&lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Instâncias Administrativas&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;1ª: Autoridade superior à que proferiu a decisão&lt;/li&gt;
+          &lt;li&gt;2ª: Autoridade máxima do órgão&lt;/li&gt;
+          &lt;li&gt;3ª: Controladoria-Geral da União (CGU)&lt;/li&gt;
+          &lt;li&gt;4ª: Comissão Mista de Reavaliação de Informações (CMRI)&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Reclamação por Omissão (Falta de resposta)&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;pode ser feita se não houver resposta no prazo legal&lt;/li&gt;
+      &lt;li&gt;dirigida à Autoridade de Monitoramento&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>0</v>
+      </c>
+      <c r="G330" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="n">
+        <v>425</v>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Lei nº 12.527-2011</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Informações Pessoais e Restrições (LAI)</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Informações Pessoais&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;relativas à intimidade, vida privada, honra e imagem&lt;/li&gt;
+      &lt;li&gt;acesso restrito independente de classificação de sigilo&lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Prazo de proteção:&lt;/b&gt; até 100 anos (da data de produção)&lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Acesso por terceiros sem consentimento (Exceções)&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;prevenção e diagnóstico médico (se o titular for incapaz e houver interesse público)&lt;/li&gt;
+          &lt;li&gt;realização de estatísticas/pesquisas (vedada identificação)&lt;/li&gt;
+          &lt;li&gt;cumprimento de ordem judicial&lt;/li&gt;
+          &lt;li&gt;defesa de direitos humanos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F331" t="n">
+        <v>0</v>
+      </c>
+      <c r="G331" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="n">
+        <v>426</v>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Fundamentos da LGPD</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Fundamentos da Proteção de Dados&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;respeito à privacidade&lt;/li&gt;
+      &lt;li&gt;autodeterminação informativa&lt;/li&gt;
+      &lt;li&gt;liberdades
+        &lt;ul&gt;
+          &lt;li&gt;expressão, informação, comunicação e opinião&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;inviolabilidade
+        &lt;ul&gt;
+          &lt;li&gt;intimidade, honra e imagem&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;desenvolvimento
+        &lt;ul&gt;
+          &lt;li&gt;econômico, tecnológico e inovação&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Ordem Econômica&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;livre iniciativa&lt;/li&gt;
+          &lt;li&gt;livre concorrência&lt;/li&gt;
+          &lt;li&gt;defesa do consumidor&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Direitos humanos
+        &lt;ul&gt;
+          &lt;li&gt;livre desenvolvimento da personalidade&lt;/li&gt;
+          &lt;li&gt;dignidade e exercício da cidadania&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>0</v>
+      </c>
+      <c r="G332" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>427</v>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Princípios do Tratamento de Dados</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Boa-fé&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;princípio basilar que deve nortear todo o tratamento&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;O "Trio de Ferro" (Finalidade, Adequação, Necessidade)&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;b&gt;Finalidade&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;propósitos legítimos, específicos, explícitos e informados&lt;/li&gt;
+          &lt;li&gt;vedado tratamento posterior incompatível&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Adequação&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;compatibilidade do tratamento com as finalidades informadas&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Necessidade (Minimização)&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;limitação ao &lt;b&gt;mínimo necessário&lt;/b&gt; para as finalidades&lt;/li&gt;
+          &lt;li&gt;dados pertinentes, proporcionais e não excessivos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Transparência e Acesso&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;b&gt;Livre Acesso&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;consulta fácil, gratuita e integral sobre a forma e duração do tratamento&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Qualidade dos Dados&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;exatidão, clareza e atualização conforme a necessidade&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Transparência&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;informações claras, precisas e acessíveis sobre os agentes de tratamento&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;b&gt;Segurança e Ética&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;b&gt;Segurança&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;medidas técnicas e administrativas para proteger dados de acessos não autorizados&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Prevenção&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;adoção de medidas para evitar a ocorrência de danos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Não Discriminação&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;impossibilidade de tratamento para fins discriminatórios ilícitos ou abusivos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Responsabilização e Prestação de Contas (Accountability)&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;demonstração de medidas eficazes e capazes de comprovar a observância da lei&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F333" t="n">
+        <v>0</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>428</v>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Transferência Internacional de Dados</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Transferência Internacional&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Permitida apenas em hipóteses específicas
+        &lt;ul&gt;
+          &lt;li&gt;países ou &lt;b&gt;organismos internacionais&lt;/b&gt; com grau de proteção adequado
+            &lt;ul&gt;
+              &lt;li&gt;conforme avaliação da ANPD&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;quando o controlador oferecer garantias de conformidade
+            &lt;ul&gt;
+              &lt;li&gt;cláusulas contratuais específicas ou padrão&lt;/li&gt;
+              &lt;li&gt;normas corporativas globais&lt;/li&gt;
+              &lt;li&gt;selos, certificados e códigos de conduta regularmente emitidos&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;cooperação jurídica internacional entre órgãos de inteligência/investigação&lt;/li&gt;
+          &lt;li&gt;proteção da vida ou da incolumidade física do titular ou de terceiro&lt;/li&gt;
+          &lt;li&gt;autorização da ANPD&lt;/li&gt;
+          &lt;li&gt;mediante &lt;b&gt;consentimento específico e destacado&lt;/b&gt; do titular
+            &lt;ul&gt;
+              &lt;li&gt;com informação prévia sobre o caráter internacional da operação&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;cumprimento de obrigação legal ou regulatória&lt;/li&gt;
+          &lt;li&gt;execução de contrato ou procedimentos preliminares&lt;/li&gt;
+          &lt;li&gt;exercício regular de direitos em processos&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F334" t="n">
+        <v>0</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>429</v>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Informática</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Lei nº 13.709-2018</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Consentimento</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;b&gt;Consentimento&lt;/b&gt;
+    &lt;ul&gt;
+      &lt;li&gt;manifestação livre, informada e inequívoca&lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Revogação&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;pode ocorrer a qualquer momento&lt;/li&gt;
+          &lt;li&gt;exige manifestação expressa do titular&lt;/li&gt;
+          &lt;li&gt;deve ser por procedimento gratuito e facilitado&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Efeitos da Revogação (Ratificação)&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;os tratamentos realizados anteriormente permanecem válidos (ratificados)&lt;/li&gt;
+          &lt;li&gt;validade mantida enquanto não houver pedido de eliminação dos dados&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;b&gt;Regras Adicionais&lt;/b&gt;
+        &lt;ul&gt;
+          &lt;li&gt;ônus da prova cabe ao controlador&lt;/li&gt;
+          &lt;li&gt;vedado o consentimento genérico (é nulo)&lt;/li&gt;
+          &lt;li&gt;se houver alteração de finalidade, o titular deve ser informado e pode revogar&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F335" t="n">
+        <v>0</v>
+      </c>
+      <c r="G335" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
:checkered_flag: sistema estruturado e pronto para inicio de preparacao
</commit_message>
<xml_diff>
--- a/banco_de_dados/flashcards.xlsx
+++ b/banco_de_dados/flashcards.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G335"/>
+  <dimension ref="A1:G372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19363,6 +19363,1891 @@
         <v>0</v>
       </c>
     </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>430</v>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Gestão de Investimentos e Risco</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Valor Monetário Esperado (VME) / Expected Monetary Value (EMV)</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Métrica que calcula o resultado financeiro médio de uma decisão que envolve riscos e incertezas.&lt;/li&gt;
+  &lt;li&gt;Média ponderada de todos os ganhos e perdas possíveis, baseada na chance de cada um acontecer.&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;$$\text{VME} = \sum (P \times I)$$&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;\(P \Rightarrow \text{Probabilidade}\)&lt;/li&gt;
+  &lt;li&gt;\(I \Rightarrow \text{Impacto}\)&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F336" t="n">
+        <v>0</v>
+      </c>
+      <c r="G336" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>431</v>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Pontos de Equilíbrio</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Ponto de Equilíbrio Contábil</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Ponto de Equilíbrio em Quantidade&lt;/strong&gt;&lt;/p&gt;
+&lt;p&gt;$$\text{PEC} = \frac{\text{CF}}{\text{MCU}}$$&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Margem de Contribuição Unitária&lt;/strong&gt;&lt;/p&gt;
+&lt;p&gt;$$\text{MCU} = \text{PV} - \text{CV}$$&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Ponto de Equilíbrio em Valor (Receita)&lt;/strong&gt;&lt;/p&gt;
+&lt;p&gt;$$\text{PEC}_R = \text{PEC} \cdot \text{PV}$$&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;Legenda&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;\(\text{PEC} \Rightarrow \text{Ponto de Equilíbrio Contábil}\)&lt;/li&gt;
+  &lt;li&gt;\(\text{CF} \Rightarrow \text{Custos e Despesas Fixos}\)&lt;/li&gt;
+  &lt;li&gt;\(\text{MCU} \Rightarrow \text{Margem de Contribuição Unitária}\)&lt;/li&gt;
+  &lt;li&gt;\(\text{PV} \Rightarrow \text{Preço de Venda Unitário}\)&lt;/li&gt;
+  &lt;li&gt;\(\text{CV} \Rightarrow \text{Custos e Despesas Variáveis Unitários}\)&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F337" t="n">
+        <v>0</v>
+      </c>
+      <c r="G337" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>432</v>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Tipos de Custeio</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Custeio Por Absorção</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Apropriação de todos os custos incorridos aos produtos fabricados.&lt;/li&gt;
+  &lt;li&gt;Atende aos princípios de contabilidade.&lt;/li&gt;
+  &lt;li&gt;Uma parte dos custos fixos fica incorporada ao estoque.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F338" t="n">
+        <v>0</v>
+      </c>
+      <c r="G338" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>433</v>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Tipos de Custeio</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Custeio Variável ou Custeio Direto</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Apenas os custos variáveis são incorridos aos produtos.&lt;/li&gt;
+  &lt;li&gt;Custos fixos são tratados como despesas do período:
+    &lt;ul&gt;
+      &lt;li&gt;Lançados diretamente na DRE, como despesa.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Pode ser usado para fins gerenciais:
+    &lt;ul&gt;
+      &lt;li&gt;Mas não na contabilidade oficial:
+        &lt;ul&gt;
+          &lt;li&gt;Pois fere o princípio da competência.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F339" t="n">
+        <v>0</v>
+      </c>
+      <c r="G339" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>434</v>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Tipos de Custeio</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Custeio Baseado em Atividades (Activity Based Costing - ABC)</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Procura reduzir a arbitrariedade do rateio dos custos indiretos.&lt;/li&gt;
+  &lt;li&gt;Os custos são inicialmente atribuídos às atividades e depois aos produtos.&lt;/li&gt;
+  &lt;li&gt;Pode ser aplicado aos custos diretos:
+    &lt;ul&gt;
+      &lt;li&gt;Mas não haverá grandes diferenças em relação aos "sistemas tradicionais".&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Compreende a identificação das atividades relevantes no processo de fabricação, e a atribuição de custos a estas atividades.&lt;/li&gt;
+  &lt;li&gt;Possibilita a redução por meio do custo, por meio da eliminação ou redução das atividades que não agregam valor ao produto.&lt;/li&gt;
+  &lt;li&gt;Foi desenvolvido para fins gerenciais:
+    &lt;ul&gt;
+      &lt;li&gt;Mas pode ser adaptado para atender à legislação.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F340" t="n">
+        <v>0</v>
+      </c>
+      <c r="G340" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>435</v>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Tipos de Custeio</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Comparação entre Custeio Variável e Por Absorção</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;\(\text{Produção} &gt; \text{Vendas} \Rightarrow \text{Lucro variável} &lt; \text{Lucro por Absorção}\)&lt;/li&gt;
+  &lt;li&gt;\(\text{Produção} &lt; \text{Vendas} \Rightarrow \text{Lucro variável} &gt; \text{Lucro por Absorção}\)&lt;/li&gt;
+  &lt;li&gt;\(\text{Produção} = \text{Vendas} \Rightarrow \text{Lucros iguais}\)&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F341" t="n">
+        <v>0</v>
+      </c>
+      <c r="G341" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="n">
+        <v>436</v>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Pontos de Equilíbrio</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Ponto de Equilíbrio Econômico (PEE)</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Volume de vendas necessário para cobrir todos os custos e despesas fixas e atingir uma meta de lucro.&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;$$\text{PEE} = \frac{\text{CF} + \text{LD}}{\text{MCU}}$$&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;\(\text{CF} \Rightarrow \text{Custos e Despesas fixas}\)&lt;/li&gt;
+  &lt;li&gt;\(\text{LD} \Rightarrow \text{Lucro desejado}\)&lt;/li&gt;
+  &lt;li&gt;\(\text{MCU} \Rightarrow \text{Margem de contribuição unitária}\)&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F342" t="n">
+        <v>0</v>
+      </c>
+      <c r="G342" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="n">
+        <v>437</v>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Pontos de Equilíbrio</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Ponto de Equilíbrio Financeiro</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Também conhecido como Ponto de Caixa ou Ponto de Sobrevivência.&lt;/li&gt;
+  &lt;li&gt;Indica o volume de vendas necessário para manter a empresa operando sem faltar dinheiro em caixa.&lt;/li&gt;
+  &lt;li&gt;Gastos que não representam saída efetiva de dinheiro (como depreciação, amortização e exaustão) são chamados de "não desembolsáveis" e devem ser retirados da conta dos custos fixos.&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;$$\text{PEF} = \frac{\text{CF} - \text{GND}}{\text{MCU}}$$&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;\(\text{CF} \Rightarrow \text{Custos e despesas Fixas}\)&lt;/li&gt;
+  &lt;li&gt;\(\text{GND} \Rightarrow \text{Gastos não desembolsáveis}\)&lt;/li&gt;
+  &lt;li&gt;\(\text{MCU} \Rightarrow \text{Margem de contribuição unitária}\)&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>0</v>
+      </c>
+      <c r="G343" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="n">
+        <v>438</v>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>PESTAL</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Fatores: Políticos, Econômicos, Sociais, Tecnológicos, Ambientais e Legais&lt;/li&gt;
+  &lt;li&gt;Objetivo: Analisar o cenário (Situação atual)&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F344" t="n">
+        <v>0</v>
+      </c>
+      <c r="G344" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="n">
+        <v>439</v>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Gestão do Desempenho Organizacional</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Periódico (NÃO é contínuo)&lt;/li&gt;
+  &lt;li&gt;Visa: identificar, medir e desenvolver o desempenho de cada colaborador, por meio da análise de metas e competências alinhadas com os objetivos estratégicos da empresa&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F345" t="n">
+        <v>0</v>
+      </c>
+      <c r="G345" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="n">
+        <v>440</v>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Gestão Patrimonial</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Conjunto de práticas e processos voltados à administração e controle físico e contábil de todos os bens tangíveis.&lt;/li&gt;
+  &lt;li&gt;Bens utilizados na manutenção das atividades e que não se destinam à comercialização direta.&lt;/li&gt;
+  &lt;li&gt;Etapas do Ciclo de Vida do Bem Patrimonial:
+    &lt;ol&gt;
+      &lt;li&gt;&lt;strong&gt;Aquisição e Recebimento:&lt;/strong&gt; Entrada física e documental do bem na organização.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Tombamento:&lt;/strong&gt; Registro inicial do bem no sistema operacional patrimonial.
+        &lt;ul&gt;
+          &lt;li&gt;Identificação física e a criação de um número de registro único.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Carga:&lt;/strong&gt; Documento que formaliza a entrega do bem a um setor ou servidor, que passa a responder por sua guarda, uso adequado e conservação.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Movimentação:&lt;/strong&gt; Troca formal de responsabilidade física ou de localização do bem entre diferentes áreas da organização.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Depreciação e Manutenção:&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;&lt;strong&gt;Depreciação:&lt;/strong&gt; Registro contábil da perda de valor do bem ao longo do tempo.&lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Manutenção:&lt;/strong&gt; Ações para garantir que o bem atinja sua vida útil projetada.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Alienação e Baixa:&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;&lt;strong&gt;Alienação:&lt;/strong&gt; Transferência do direito de propriedade a terceiros.&lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Baixa:&lt;/strong&gt; Exclusão dos registros patrimoniais e contábeis.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ol&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Relação com a Logística:
+    &lt;ul&gt;
+      &lt;li&gt;A logística é altamente dependente de infraestrutura física (instalação de armazenagem, empilhadeiras, esteiras, frota de caminhões e sistemas de refrigeração).&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Sinergia:
+    &lt;ul&gt;
+      &lt;li&gt;Garantia de disponibilidade&lt;/li&gt;
+      &lt;li&gt;Decisão de substituição e custos&lt;/li&gt;
+      &lt;li&gt;Controle de inventário físico&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>0</v>
+      </c>
+      <c r="G346" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="n">
+        <v>441</v>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Modelo de Excelência em Gestão (MEG)</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Dimensões:&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;Pensamento sistêmico;&lt;/li&gt;
+  &lt;li&gt;Aprendizado organizacional e inovação;&lt;/li&gt;
+  &lt;li&gt;Liderança transformadora;&lt;/li&gt;
+  &lt;li&gt;Compromisso com as partes interessadas;&lt;/li&gt;
+  &lt;li&gt;Adaptabilidade;&lt;/li&gt;
+  &lt;li&gt;Desenvolvimento sustentável;&lt;/li&gt;
+  &lt;li&gt;Orientação por processos; e&lt;/li&gt;
+  &lt;li&gt;Geração de valor.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>0</v>
+      </c>
+      <c r="G347" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="n">
+        <v>442</v>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Filosofia Lean</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Maximização do valor para o cliente com o mínimo de recursos possível.&lt;/li&gt;
+  &lt;li&gt;Eliminação sistemática de desperdícios.&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;5 Princípios do Lean:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Valor&lt;/li&gt;
+      &lt;li&gt;Fluxo de Valor (VSM)&lt;/li&gt;
+      &lt;li&gt;Fluxo contínuo&lt;/li&gt;
+      &lt;li&gt;Produção puxada&lt;/li&gt;
+      &lt;li&gt;Perfeição (Kaizen)&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;8 Desperdícios:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Superprodução&lt;/li&gt;
+      &lt;li&gt;Espera&lt;/li&gt;
+      &lt;li&gt;Transporte&lt;/li&gt;
+      &lt;li&gt;Processamento Excessivo&lt;/li&gt;
+      &lt;li&gt;Estoque&lt;/li&gt;
+      &lt;li&gt;Movimento&lt;/li&gt;
+      &lt;li&gt;Defeitos&lt;/li&gt;
+      &lt;li&gt;Habilidades Subutilizadas&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Aplicação no Serviço Público (Lean Management):&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Cliente&lt;/li&gt;
+      &lt;li&gt;Produto&lt;/li&gt;
+      &lt;li&gt;Estoque&lt;/li&gt;
+      &lt;li&gt;Transporte e Movimento&lt;/li&gt;
+      &lt;li&gt;Processamento excessivo&lt;/li&gt;
+      &lt;li&gt;Fluxo contínuo e Puxado&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>0</v>
+      </c>
+      <c r="G348" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="n">
+        <v>443</v>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Indústria 3.0</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Máquinas controladas por computadores&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F349" t="n">
+        <v>0</v>
+      </c>
+      <c r="G349" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="n">
+        <v>444</v>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Indústria 4.0</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Máquinas realizam o trabalho de forma autônoma&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F350" t="n">
+        <v>0</v>
+      </c>
+      <c r="G350" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>445</v>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas por Competências</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Modelo gerencial que foca em identificar, gerenciar e desenvolver o CHA dos colaboradores:
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Conhecimento:&lt;/strong&gt; Saber – domínio teórico&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Habilidade:&lt;/strong&gt; Saber fazer – aplicação prática&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Atitude:&lt;/strong&gt; Querer fazer – comportamento e motivação&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Objetiva garantir que as competências individuais e coletivas estejam alinhadas aos objetivos e à estratégia geral&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Características Principais:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Flexibilidade:&lt;/strong&gt; O foco sai da tarefa fixa e vai para a capacidade do indivíduo de entregar resultados em diferentes cenários&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Desenvolvimento Contínuo:&lt;/strong&gt; Atrelada à avaliação de desempenho, treinamento e gestão do conhecimento.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Contraponto ao Modelo Tradicional:&lt;/strong&gt; Rompe com a rigidez, a padronização excessiva e a descrição engessada de cargos típica do modelo burocrático.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F351" t="n">
+        <v>0</v>
+      </c>
+      <c r="G351" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>446</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Gestão de Projetos</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Kanban</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Baseado em um sistema puxado
+    &lt;ul&gt;
+      &lt;li&gt;Fluxo contínuo&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;O objetivo central é limitar o trabalho em andamento para evitar gargalos e maximizar a eficiência&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Origem:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Criado pela Toyota (Taiichi Ohno) no Japão (década de 1940)&lt;/li&gt;
+      &lt;li&gt;Faz parte do STP&lt;/li&gt;
+      &lt;li&gt;Tradução literal: "Cartão Visual" ou "Sinalização"&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Componentes Visuais:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Quadro (Board):&lt;/strong&gt; Representa todo o fluxo de valor do sistema&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Colunas:&lt;/strong&gt; A fazer, Em Andamento, Feito&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Cartões:&lt;/strong&gt; Tarefas ou pacotes de trabalho&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Cores:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Categorização, priorização e identificação
+        &lt;ul&gt;
+          &lt;li&gt;Tipos de demanda&lt;/li&gt;
+          &lt;li&gt;Classes de Serviços:
+            &lt;ul&gt;
+              &lt;li&gt;Urgente: vermelho&lt;/li&gt;
+              &lt;li&gt;Data fixa: cores diversas&lt;/li&gt;
+              &lt;li&gt;Padrão: cores neutras
+                &lt;ul&gt;
+                  &lt;li&gt;Seguem o FIFO&lt;/li&gt;
+                &lt;/ul&gt;
+              &lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Métricas:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Lead Time:&lt;/strong&gt; tempo desde a ideia/solicitação até a entrega ao cliente&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Cycle Time (Tempo de Ciclo):&lt;/strong&gt; Tempo que uma tarefa leva para ser concluída&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;WIP (Work in Progress):&lt;/strong&gt; Quantidade de tarefas ativas simultaneamente&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Throughput (Vazão):&lt;/strong&gt; Número de itens de trabalho efetivamente entregues por unidade de tempo&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F352" t="n">
+        <v>0</v>
+      </c>
+      <c r="G352" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="n">
+        <v>447</v>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Teorias e Modelos de Liderança</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>&lt;ol&gt;
+  &lt;li&gt;&lt;strong&gt;Teorias dos Traços de Personalidade (A abordagem mais antiga):&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;O líder "já nasce líder". A liderança é baseada em características inatas.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Teorias dos Estilos Comportamentais (Foco no que o líder faz):&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;A liderança pode ser ensinada.&lt;/li&gt;
+      &lt;li&gt;O foco está no comportamento do líder em relação aos subordinados.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Principais modelos (Estudos de Kurt Lewin / White e Lippitt):&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;&lt;strong&gt;Autocrática:&lt;/strong&gt;
+            &lt;ul&gt;
+              &lt;li&gt;Líder centraliza decisões, dita regras&lt;/li&gt;
+              &lt;li&gt;Foco na tarefa&lt;/li&gt;
+              &lt;li&gt;Gera tensão e frustração&lt;/li&gt;
+              &lt;li&gt;Pode ser rápida em crise&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Democrática:&lt;/strong&gt;
+            &lt;ul&gt;
+              &lt;li&gt;Líder envolve o grupo nas decisões.&lt;/li&gt;
+              &lt;li&gt;Foco nas pessoas e nas tarefas&lt;/li&gt;
+              &lt;li&gt;Gera maior satisfação e qualidade no trabalho&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Laissez-Faire (Liberal):&lt;/strong&gt;
+            &lt;ul&gt;
+              &lt;li&gt;Liberdade total ao grupo&lt;/li&gt;
+              &lt;li&gt;O líder só atua se solicitado&lt;/li&gt;
+              &lt;li&gt;Costuma gerar baixa produtividade e desorganização se a equipe não for altamente madura.&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Grid Gerencial (Blake e Mouton):&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;Avalia o líder em duas dimensões (Orientação para Tarefa \(\times\) Orientação para Pessoas) em uma grade de 1 a 9.&lt;/li&gt;
+          &lt;li&gt;O modelo ideal (9,9) é o líder que foca ao máximo tanto na produção quanto na equipe.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Teorias Contingenciais ou Situacionais:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Não existe um estilo de liderança único e ideal para todas as situações.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Modelo de Liderança Situacional (Hersey e Blanchard):&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;Cruza o comportamento do líder (foco em tarefa vs. relacionamento) com a maturidade do liderado (capacidade técnica + motivação/vontade).&lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Maturidade M1 (Baixa):&lt;/strong&gt; Subordinado não sabe fazer e não quer fazer.
+            &lt;ul&gt;
+              &lt;li&gt;&lt;strong&gt;Estilo E1 (Determinar / Dirigir / Dar Ordem):&lt;/strong&gt; Muito foco na tarefa e pouco no relacionamento.&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Maturidade M2 (Média-Baixa):&lt;/strong&gt; Subordinado não sabe fazer, mas quer fazer.
+            &lt;ul&gt;
+              &lt;li&gt;&lt;strong&gt;Estilo E2 (Persuadir / Vender):&lt;/strong&gt; Muito foco na tarefa e muito foco no relacionamento.&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Maturidade M3 (Médio-Alta):&lt;/strong&gt; Subordinado sabe fazer, mas não quer fazer.
+            &lt;ul&gt;
+              &lt;li&gt;&lt;strong&gt;Estilo E3 (Compartilhar / Participar):&lt;/strong&gt; Pouco foco na tarefa e muito foco no relacionamento.&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Maturidade M4 (Alta):&lt;/strong&gt; Subordinado sabe fazer e quer fazer.
+            &lt;ul&gt;
+              &lt;li&gt;&lt;strong&gt;Estilo E4 (Delegar):&lt;/strong&gt; Foca pouco na tarefa e pouco no relacionamento.&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ol&gt;</t>
+        </is>
+      </c>
+      <c r="F353" t="n">
+        <v>0</v>
+      </c>
+      <c r="G353" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="n">
+        <v>448</v>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Teoria dos Dois Fatores de Herzberg</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Fatores Higiênicos (Extrínsecos):&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;A presença não motiva&lt;/li&gt;
+      &lt;li&gt;A ausência gera insatisfação&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Ex:&lt;/strong&gt; Salários, benefícios corporativos, segurança no emprego, condições físicas de trabalho e relacionamento com a liderança.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Fatores Motivacionais (Intrínsecos):&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Elementos que geram satisfação e motivação&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Ex:&lt;/strong&gt; Reconhecimento, grau de responsabilidade, oportunidade de crescimento profissional, desafios intelectuais e o trabalho em si.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F354" t="n">
+        <v>0</v>
+      </c>
+      <c r="G354" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="n">
+        <v>449</v>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Hierarquia das Necessidades de Maslow</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Fisiológicas (Base):&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Exigências vitais:
+        &lt;ul&gt;
+          &lt;li&gt;Alimentação, água, abrigo, descanso&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;De Segurança:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Busca por proteção, ordem, estabilidade e ausência de ameaças&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Sociais:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Interação humana, aceitação, pertencimento e amizade&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;De Estima:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Reconhecimento e valorização externa e respeito próprio&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;De Autorrealização (Topo):&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;O impulso do indivíduo de maximizar o próprio potencial, envolvendo autonomia, criatividade, superação de limites e desenvolvimento contínuo&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F355" t="n">
+        <v>0</v>
+      </c>
+      <c r="G355" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="n">
+        <v>450</v>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Dissonância Cognitiva</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Inconsistência percebida por um funcionário entre suas crenças, sentimentos e ações em relação à empresa.&lt;/li&gt;
+  &lt;li&gt;Demonstra que não apenas as emoções e atitudes levam ao comportamento, mas o oposto também pode ocorrer.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F356" t="n">
+        <v>0</v>
+      </c>
+      <c r="G356" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="n">
+        <v>451</v>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Racionalização Excessiva</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Mecanismo de defesa psicológico (tentativa de justificar comportamentos inaceitáveis com motivos lógicos).&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F357" t="n">
+        <v>0</v>
+      </c>
+      <c r="G357" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="n">
+        <v>452</v>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Teoria das Necessidades Aprendidas (David McClelland)</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Necessidade de Afiliação:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Busca contínua por aceitação social, amizade e forte aversão a atritos interpessoais.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Baixa:&lt;/strong&gt; Cargos gerenciais ou posições que exigem alocação de recursos escassos.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Necessidade de Poder:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Desejo de exercer influência, controle e impacto sobre outras pessoas e sobre o ambiente organizacional.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Necessidade de Realização:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Impulso interno para alcançar a excelência, assumir responsabilidades diretas na resolução de problemas e atingir metas desafiadoras, preferência por riscos moderados e necessidade de feedback constante.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F358" t="n">
+        <v>0</v>
+      </c>
+      <c r="G358" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="n">
+        <v>453</v>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Teoria da Expectativa (Victor Vroom)</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Expectância (Expectativa):&lt;/strong&gt; Crença de que o esforço individual dedicado à tarefa resultará no nível de desempenho desejado.&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Instrumentalidade:&lt;/strong&gt; Crença de que o nível de desempenho alcançado funcionará como o meio (instrumento) para a obtenção de uma recompensa.&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Valência:&lt;/strong&gt; Valor ou grau de importância subjetiva que o indivíduo atribui à recompensa oferecida pela organização.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F359" t="n">
+        <v>0</v>
+      </c>
+      <c r="G359" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="n">
+        <v>454</v>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Teoria da Equidade (J. Stacy Adams)</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Percepção de Justiça&lt;/li&gt;
+  &lt;li&gt;Trabalhador compara as suas contribuições com as suas recompensas e, em seguida, compara essa relação com a de outros colegas&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Comportamento em caso de Iniquidade:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Tensão que motiva o indivíduo a buscar o equilíbrio&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Ex:&lt;/strong&gt; Diminuir o ritmo de trabalho, exigir aumento, mudar de setor ou pedir demissão&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Capacidade de Previsão:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Pontos fortes:&lt;/strong&gt; Possui forte respaldo empírico para explicar e prever impactos na satisfação, no absenteísmo e na rotatividade.&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Pontos fracos:&lt;/strong&gt; Falha na previsão de assimetrias na produtividade.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F360" t="n">
+        <v>0</v>
+      </c>
+      <c r="G360" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="n">
+        <v>455</v>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Teoria do Caminho-Objetivo (Robert House)</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Estabelece que cada estilo de liderança relaciona-se com variáveis situacionais.&lt;/li&gt;
+  &lt;li&gt;O objetivo do líder é "limpar o caminho" para que os subordinados alcancem suas metas.&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Estilos de Liderança:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;&lt;strong&gt;Diretivo:&lt;/strong&gt; O líder fornece instruções rigorosas, define expectativas, cronogramas e regras claras.
+        &lt;ul&gt;
+          &lt;li&gt;Tarefa não rotineira&lt;/li&gt;
+          &lt;li&gt;Necessidade de minimizar ambiguidades de função&lt;/li&gt;
+          &lt;li&gt;Subordinados inexperientes&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Apoiador:&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;O líder demonstra preocupação genuína com o bem-estar, conforto e as necessidades da equipe.&lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Aplicação Situacional:&lt;/strong&gt; Tarefas estruturadas, rotineiras, monótonas ou sob alto nível de estresse.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Participativo:&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;O líder compartilha informações, consulta a equipe e utiliza suas sugestões antes da tomada de decisão.&lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Aplicação situacional:&lt;/strong&gt;
+            &lt;ul&gt;
+              &lt;li&gt;Subordinados experientes&lt;/li&gt;
+              &lt;li&gt;Tarefas complexas onde o envolvimento melhora a situação&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Realizador:&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;O líder define metas altamente desafiadoras, encoraja a melhoria contínua e demonstra extrema confiança na capacidade de alto desempenho da equipe.&lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Aplicação situacional:&lt;/strong&gt;
+            &lt;ul&gt;
+              &lt;li&gt;Tarefas ambíguas ou não rotineiras&lt;/li&gt;
+              &lt;li&gt;Equipes já altamente capacitadas e autônomas&lt;/li&gt;
+            &lt;/ul&gt;
+          &lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F361" t="n">
+        <v>0</v>
+      </c>
+      <c r="G361" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="n">
+        <v>456</v>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Gestão de Pessoas</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Liderança Transacional vs Transformacional (Bass e Burns)</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Líder Transacional:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Relação baseada em trocas operacionais&lt;/li&gt;
+      &lt;li&gt;Líder estabelece as regras, define as metas/tarefas e monitora o desempenho&lt;/li&gt;
+      &lt;li&gt;Premiação ou punição baseada no atingimento de metas&lt;/li&gt;
+      &lt;li&gt;Líder só intervém quando os padrões não são atingidos ou quando as coisas saem do trilho&lt;/li&gt;
+      &lt;li&gt;O objetivo é manter a estabilidade, o status quo e garantir a eficiência rotineira.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Líder Transformacional:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Líder inspira os liderados a transcenderem seus próprios interesses individuais em prol da organização&lt;/li&gt;
+      &lt;li&gt;&lt;strong&gt;Características Principais (4 I's):&lt;/strong&gt;
+        &lt;ul&gt;
+          &lt;li&gt;&lt;strong&gt;Influência Idealizada:&lt;/strong&gt; O líder é admirado e atua como um modelo moral e de conduta.&lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Inspiração Motivacional:&lt;/strong&gt; Comunica altas expectativas e dá sentido ao trabalho.&lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Estimulação Intelectual:&lt;/strong&gt; Incita novos olhares sobre problemas antigos e questiona o status quo.&lt;/li&gt;
+          &lt;li&gt;&lt;strong&gt;Consideração Individualizada:&lt;/strong&gt; Foca no desenvolvimento pessoal, atuando como mentor ou coach para cada subordinado.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Tem o objetivo de inovar, transformar o ambiente e desenvolver os liderados.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F362" t="n">
+        <v>0</v>
+      </c>
+      <c r="G362" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="n">
+        <v>457</v>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Protocolos de Avaliação Ergonômica</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Método OCRA (Occupational Repetitive Actions)&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;Avaliação de movimentos repetitivos e riscos de DORT (Distúrbios Osteomusculares Relacionados ao Trabalho)&lt;/li&gt;
+  &lt;li&gt;Desenvolvido pelos italianos Occhipinti e Colombini&lt;/li&gt;
+  &lt;li&gt;Adotado pela IEA (International Ergonomics Association)&lt;/li&gt;
+  &lt;li&gt;Avaliação semiquantitativa dividida em duas ferramentas:
+    &lt;ul&gt;
+      &lt;li&gt;Checklist: mapeamento de risco e avaliação preliminar&lt;/li&gt;
+      &lt;li&gt;Índice OCRA: Avaliação aprofundada que gera um multiplicador baseado em frequência, força, postura e períodos de recuperação&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;&lt;strong&gt;Equação do NIOSH (National Institute for Occupational Safety and Health)&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;Levantamento manual de cargas&lt;/li&gt;
+  &lt;li&gt;Objetivo primário: proteger a coluna lombar contra lesões&lt;/li&gt;
+  &lt;li&gt;Utiliza uma fórmula matemática para calcular o LPR (Limite de Peso Recomendado) para uma tarefa específica&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;&lt;strong&gt;Método OWAS (Ovako Working Posture Analysis System)&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;Análise postural do corpo inteiro&lt;/li&gt;
+  &lt;li&gt;Desenvolvido na Finlândia (Indústria do aço Ovako Oy)&lt;/li&gt;
+  &lt;li&gt;Codifica as posturas assumidas pelas costas (4 posições), braços (3 posições) e pernas (7 posições), além da carga/força suportada (3 níveis)&lt;/li&gt;
+  &lt;li&gt;Pontuação:
+    &lt;ul&gt;
+      &lt;li&gt;Categoria de risco de 1 (postura normal) a 4 (medidas corretivas imediatas)&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;&lt;strong&gt;RULA (Rapid Upper Limb Assessment)&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;Avaliação rápida de sobrecarga postural, com foco predominante em membros superiores, pescoço e tronco&lt;/li&gt;
+  &lt;li&gt;Semelhante ao OWAS na ideia de codificação de posturas, mas muito mais detalhado para braços, antebraços e pulsos.&lt;/li&gt;
+  &lt;li&gt;Amplamente utilizado para avaliar trabalhos em escritórios, uso de computadores e linhas de montagem finas.&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;&lt;strong&gt;REBA (Rapid Entire Body Assessment)&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;Avaliação rápida do corpo inteiro&lt;/li&gt;
+  &lt;li&gt;Especialmente projetado para posturas dinâmicas, imprevisíveis e movimentação de pacientes / cargas instáveis.&lt;/li&gt;
+  &lt;li&gt;Evolução direta do RULA, mas inclui uma análise muito mais robusta dos membros inferiores e do acoplamento (pega)&lt;/li&gt;
+  &lt;li&gt;Favorito para o setor de saúde (enfermagem) e construção civil&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F363" t="n">
+        <v>0</v>
+      </c>
+      <c r="G363" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>458</v>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Ergonomia (NR17): Transporte Manual de Cargas</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Limites de Peso para Mulheres e Menores (Art. 390 da CLT):
+    &lt;ul&gt;
+      &lt;li&gt;Trabalho contínuo: Máximo 20 kg&lt;/li&gt;
+      &lt;li&gt;Trabalho ocasional: Máximo 25 kg&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Limitação para Homens Adultos (Art. 198 da CLT):
+    &lt;ul&gt;
+      &lt;li&gt;Máximo 60 kg&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;A NR17 exige que o peso não comprometa a saúde ou a segurança do trabalhador, independente desse limite.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F364" t="n">
+        <v>0</v>
+      </c>
+      <c r="G364" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>459</v>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Áreas da Ergonomia</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Ergonomia Física:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Conforto no ambiente de trabalho e na prevenção de lesões musculoesqueléticas&lt;/li&gt;
+      &lt;li&gt;Características anatômicas, antropométricas, fisiológicas e biomecânicas&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Ergonomia Organizacional:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Otimização dos sistemas sociotécnicos&lt;/li&gt;
+      &lt;li&gt;Estruturas organizacionais, políticas e processos&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Ergonomia Cognitiva:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Processos mentais&lt;/li&gt;
+      &lt;li&gt;Percepção, memória, raciocínio e resposta motora&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F365" t="n">
+        <v>0</v>
+      </c>
+      <c r="G365" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>460</v>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Análise Ergonômica do Trabalho (AET)</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Estudo técnico, aprofundado e sistemático das condições de trabalho&lt;/li&gt;
+  &lt;li&gt;Exigido pela NR17&lt;/li&gt;
+  &lt;li&gt;Objetiva avaliar e garantir a adaptação das condições de trabalho às características psicofisiológicas dos trabalhadores&lt;/li&gt;
+  &lt;li&gt;Deve ser realizada sempre que:
+    &lt;ul&gt;
+      &lt;li&gt;Avaliação Ergonômica Preliminar (AEP) apontar a necessidade de um estudo mais aprofundado&lt;/li&gt;
+      &lt;li&gt;Houver recomendação médica a partir do Programa de Controle Médico de Saúde Ocupacional (PCMSO)&lt;/li&gt;
+      &lt;li&gt;For necessária a investigação de acidentes ou doenças ocupacionais com suspeita de relação com fatores ergonômicos&lt;/li&gt;
+      &lt;li&gt;Ocorrer a introdução ou modificação significativa de processos, tecnologias ou ambientes de trabalho que impactem a ergonomia&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Dispensa da elaboração:
+    &lt;ul&gt;
+      &lt;li&gt;Microempresas (ME) e Empresas de Pequeno Porte (EPP) que estejam enquadradas nos graus de risco 1 e 2&lt;/li&gt;
+      &lt;li&gt;Microempreendedor Individual (MEI)&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Observação importante:
+    &lt;ul&gt;
+      &lt;li&gt;A dispensa para ME e EPP (graus 1 e 2) cai por terra e a análise passa a ser obrigatória se:
+        &lt;ul&gt;
+          &lt;li&gt;O médico do PCMSO solicitar&lt;/li&gt;
+          &lt;li&gt;Houver fiscalização do trabalho exigindo&lt;/li&gt;
+          &lt;li&gt;A AEP (que continua sendo obrigatória para estes casos) identificar riscos que exijam uma avaliação ergonômica aprofundada&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Relatório: Deve ficar à disposição pelo prazo de 20 anos.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F366" t="n">
+        <v>0</v>
+      </c>
+      <c r="G366" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>461</v>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Adaptação do Mobiliário e Apoio para os Pés</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;O mobiliário dos postos de trabalho deve ser concebido e adaptado para atender às características psicofisiológicas dos trabalhadores e às suas dimensões antropométricas&lt;/li&gt;
+  &lt;li&gt;Regras sobre o uso do Apoio para os Pés:
+    &lt;ul&gt;
+      &lt;li&gt;Condição de fornecimento:
+        &lt;ul&gt;
+          &lt;li&gt;Não é uma exigência obrigatória para todos os postos de trabalho sentados de forma indiscriminada.&lt;/li&gt;
+          &lt;li&gt;Deve ser utilizado sempre que o trabalhador não conseguir manter a região plantar dos pés completamente apoiada no piso.&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+      &lt;li&gt;Finalidade:
+        &lt;ul&gt;
+          &lt;li&gt;Serve para a adaptação do posto de trabalho ao biotipo do trabalhador&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F367" t="n">
+        <v>0</v>
+      </c>
+      <c r="G367" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>462</v>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>NR17 (Anexo I) - Operadores de Checkout</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;strong&gt;Posto de Trabalho e Mobiliário&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;As dimensões do mobiliário devem atender às características antropométricas de 90% dos trabalhadores&lt;/li&gt;
+  &lt;li&gt;O mobiliário deve assegurar a postura para o trabalho tanto na posição sentada quanto em pé&lt;/li&gt;
+  &lt;li&gt;O apoio para os pés deve ser independente da cadeira&lt;/li&gt;
+  &lt;li&gt;Checkouts com comprimento igual ou superior a 2,7 m exigem sistema com esteira eletromecânica&lt;/li&gt;
+  &lt;li&gt;O operador deve ser protegido contra correntes de ar/vento ou grandes variações climáticas&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;&lt;strong&gt;Manipulação e Ensacamento&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;A atividade de ensacamento não deve se incorporar ao ciclo de trabalho habitual do operador&lt;/li&gt;
+  &lt;li&gt;A organização pode optar por manter, no mínimo, um ensacador a cada três checkouts em funcionamento para evitar essa sobrecarga&lt;/li&gt;
+  &lt;li&gt;A pesagem de mercadorias pelo operador só é permitida se atender simultaneamente a:
+    &lt;ul&gt;
+      &lt;li&gt;Balança frontal e nivelada com a superfície (tolerância máxima de 2 cm)&lt;/li&gt;
+      &lt;li&gt;Teclado a uma distância máxima de 45 cm&lt;/li&gt;
+      &lt;li&gt;Código de mercadoria com limite máximo de oito dígitos&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;&lt;strong&gt;Organização do Trabalho&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;Saídas para necessidades fisiológicas são garantidas a qualquer momento, mediante comunicação&lt;/li&gt;
+  &lt;li&gt;É vedado usar o número de mercadorias ou compras como base de avaliação de desempenho para fins de remuneração ou premiação&lt;/li&gt;
+  &lt;li&gt;O operador de checkout é proibido de realizar qualquer tarefa de segurança patrimonial&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;&lt;strong&gt;Aspectos Psicossociais&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;O dispositivo de identificação (crachá) é obrigatório, com nome e sobrenome escolhidos pelo trabalhador&lt;/li&gt;
+  &lt;li&gt;É vedado obrigar o uso de vestimentas, propagandas ou maquiagem temática que firam a dignidade pessoal ou causem constrangimento ao trabalhador&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;&lt;strong&gt;Treinamento e Capacitação&lt;/strong&gt;&lt;/p&gt;
+&lt;ul&gt;
+  &lt;li&gt;O treinamento deve ser ministrado durante a jornada de trabalho&lt;/li&gt;
+  &lt;li&gt;Treinamento Inicial:
+    &lt;ul&gt;
+      &lt;li&gt;Duração mínima de duas horas&lt;/li&gt;
+      &lt;li&gt;Deve ocorrer até o trigésimo dia da data de admissão&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Treinamento Periódico:
+    &lt;ul&gt;
+      &lt;li&gt;Frequência anual&lt;/li&gt;
+      &lt;li&gt;Duração mínima de duas horas&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F368" t="n">
+        <v>0</v>
+      </c>
+      <c r="G368" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>463</v>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Normas Regulamentadoras (Todas as NRs)</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>&lt;ol&gt;
+  &lt;li&gt;Disposições Gerais e Gerenciamento de Riscos Ocupacionais&lt;/li&gt;
+  &lt;li&gt;Embargo e Interdição (Revogada)&lt;/li&gt;
+  &lt;li&gt;Embargo e Interdição&lt;/li&gt;
+  &lt;li&gt;SESMT (Serviço Especializado em Segurança e em Medicina do Trabalho)&lt;/li&gt;
+  &lt;li&gt;CIPA (Comissão Interna de Prevenção de Acidentes e de Assédio)&lt;/li&gt;
+  &lt;li&gt;Equipamento de Proteção Individual (EPI)&lt;/li&gt;
+  &lt;li&gt;PCMSO (Programa de Controle Médico de Saúde Ocupacional)&lt;/li&gt;
+  &lt;li&gt;Edificações&lt;/li&gt;
+  &lt;li&gt;Avaliação e Controle das Exposições Ocupacionais a Agentes Físicos, Químicos e Biológicos&lt;/li&gt;
+  &lt;li&gt;Segurança em Instalações e Serviços em Eletricidade&lt;/li&gt;
+  &lt;li&gt;Transporte, Movimentação, Armazenagem e Manuseio de Materiais&lt;/li&gt;
+  &lt;li&gt;Segurança no Trabalho em Máquinas e Equipamentos&lt;/li&gt;
+  &lt;li&gt;Caldeiras, Vasos de Pressão, Tubulações e Tanques Metálicos de Armazenamento&lt;/li&gt;
+  &lt;li&gt;Fornos&lt;/li&gt;
+  &lt;li&gt;Atividades e Operações Insalubres&lt;/li&gt;
+  &lt;li&gt;Atividades e Operações Perigosas&lt;/li&gt;
+  &lt;li&gt;Ergonomia&lt;/li&gt;
+  &lt;li&gt;Segurança e Saúde no Trabalho na Indústria da Construção&lt;/li&gt;
+  &lt;li&gt;Explosivos&lt;/li&gt;
+  &lt;li&gt;Segurança e Saúde no Trabalho com Inflamáveis e Combustíveis&lt;/li&gt;
+  &lt;li&gt;Trabalhos a Céu Aberto&lt;/li&gt;
+  &lt;li&gt;Segurança e Saúde Ocupacional na Mineração&lt;/li&gt;
+  &lt;li&gt;Proteção Contra Incêndios&lt;/li&gt;
+  &lt;li&gt;Condições Sanitárias e de Conforto nos Locais de Trabalho&lt;/li&gt;
+  &lt;li&gt;Resíduos Industriais&lt;/li&gt;
+  &lt;li&gt;Sinalização de Segurança&lt;/li&gt;
+  &lt;li&gt;(Revogada)&lt;/li&gt;
+  &lt;li&gt;Fiscalização e Penalidades&lt;/li&gt;
+  &lt;li&gt;Segurança e Saúde no Trabalho Portuário&lt;/li&gt;
+  &lt;li&gt;Segurança e Saúde no Trabalho Aquaviário&lt;/li&gt;
+  &lt;li&gt;Segurança e Saúde no Trabalho na Agricultura, Pecuária, Silvicultura, Exploração Florestal e Aquicultura&lt;/li&gt;
+  &lt;li&gt;Segurança e Saúde no Trabalho em Serviços de Saúde&lt;/li&gt;
+  &lt;li&gt;Segurança e Saúde nos Trabalhos em Espaços Confinados&lt;/li&gt;
+  &lt;li&gt;Condições e Meio Ambiente de Trabalho na Indústria da Construção, Reparação e Desmonte Naval&lt;/li&gt;
+  &lt;li&gt;Trabalho em Altura&lt;/li&gt;
+  &lt;li&gt;Segurança e Saúde no Trabalho em Empresas de Abate e Processamento de Carnes e Derivados&lt;/li&gt;
+  &lt;li&gt;Segurança e Saúde em Plataformas de Petróleo&lt;/li&gt;
+  &lt;li&gt;Segurança e Saúde no Trabalho nas Atividades de Limpeza Urbana e Manejo de Resíduos Sólidos&lt;/li&gt;
+&lt;/ol&gt;</t>
+        </is>
+      </c>
+      <c r="F369" t="n">
+        <v>0</v>
+      </c>
+      <c r="G369" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="n">
+        <v>464</v>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>NR33 - Segurança e Saúde nos Trabalhos em Espaços Confinados</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;&lt;strong&gt;Espaço Confinado:&lt;/strong&gt; qualquer área não projetada para ocupação humana contínua, com meios limitados de entrada e saída, e com ventilação insuficiente para remover contaminantes ou onde possa existir deficiência/enriquecimento de oxigênio&lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Presença Obrigatória:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Trabalhador Autorizado&lt;/li&gt;
+      &lt;li&gt;Vigia: fica de fora monitorando e controlando acessos&lt;/li&gt;
+      &lt;li&gt;Supervisor de Entrada: emite a permissão&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Permissão de Entrada de Trabalho:&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Documento obrigatório&lt;/li&gt;
+      &lt;li&gt;Específico para cada entrada&lt;/li&gt;
+      &lt;li&gt;Validade restrita ao turno&lt;/li&gt;
+      &lt;li&gt;Deve ser arquivada por 5 anos&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;A atmosfera do ambiente deve ser monitorada de forma contínua para garantir:
+    &lt;ul&gt;
+      &lt;li&gt;Níveis de oxigênio&lt;/li&gt;
+      &lt;li&gt;Ausência de gases tóxicos e inflamáveis&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F370" t="n">
+        <v>0</v>
+      </c>
+      <c r="G370" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="n">
+        <v>465</v>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>NR35 - Trabalho em Altura</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>&lt;ul&gt;
+  &lt;li&gt;Acima de 2 m do nível inferior&lt;/li&gt;
+  &lt;li&gt;Trabalhador só pode atuar em altura após ser aprovado em treinamento:
+    &lt;ul&gt;
+      &lt;li&gt;Carga horária mínima de 8 horas&lt;/li&gt;
+      &lt;li&gt;Válido por 2 anos&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Trabalhador também deve possuir aptidão médica (atestado de aptidão médica específico para a função)&lt;/li&gt;
+  &lt;li&gt;Planejado&lt;/li&gt;
+  &lt;li&gt;Precedido por uma Análise de Risco (AR)&lt;/li&gt;
+  &lt;li&gt;Obrigatória a emissão de uma Permissão de Trabalho (PT) se não for rotineiro&lt;/li&gt;
+  &lt;li&gt;Deve ser evitada:
+    &lt;ul&gt;
+      &lt;li&gt;Impossibilidade:
+        &lt;ol&gt;
+          &lt;li&gt;Adotar medidas que eliminem o risco de queda&lt;/li&gt;
+          &lt;li&gt;Minimizar as consequências da queda&lt;/li&gt;
+        &lt;/ol&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;&lt;strong&gt;Sistema de Proteção contra Quedas (SPQ):&lt;/strong&gt;
+    &lt;ul&gt;
+      &lt;li&gt;Exigido o uso obrigatório de cinto de segurança tipo paraquedista&lt;/li&gt;
+      &lt;li&gt;Sistema de ancoragem adequado&lt;/li&gt;
+      &lt;li&gt;Talabarte ou Trava-quedas:
+        &lt;ul&gt;
+          &lt;li&gt;Deve ser fixado acima da linha de cintura&lt;/li&gt;
+        &lt;/ul&gt;
+      &lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F371" t="n">
+        <v>0</v>
+      </c>
+      <c r="G371" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="n">
+        <v>466</v>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Matemática</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Múltiplos e Divisores</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Encontrar o MDC pelo algorítmo de Euclides</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>&lt;b&gt;Passo a passo&lt;/b&gt;
+&lt;ul&gt;
+  &lt;li&gt;Trace duas linhas horizontais.
+    &lt;ul&gt;
+      &lt;li&gt;A linha superior servirá para anotar os quocientes, a do meio para os números que estão sendo divididos, e a inferior para os restos.&lt;/li&gt;
+    &lt;/ul&gt;
+  &lt;/li&gt;
+  &lt;li&gt;Na linha central, escreva o maior número na primeira coluna e o menor na segunda coluna.&lt;/li&gt;
+  &lt;li&gt;Divida o número maior pelo menor.&lt;/li&gt;
+  &lt;li&gt;Coloque o quociente na linha de cima, exatamente sobre o divisor.&lt;/li&gt;
+  &lt;li&gt;Coloque o resto da divisão na linha de baixo, exatamente sob o dividendo.&lt;/li&gt;
+  &lt;li&gt;Pegue o resto e repita-o na linha central, colocando-o imediatamente à direita do último divisor.&lt;/li&gt;
+  &lt;li&gt;Divida o número central anterior pelo novo número ao lado dele. Volte a anotar o quociente em cima e o resto embaixo.&lt;/li&gt;
+  &lt;li&gt;Repita esse processo até encontrar um resto igual a zero. O MDC será o último número da linha central.&lt;/li&gt;
+&lt;/ul&gt;</t>
+        </is>
+      </c>
+      <c r="F372" t="n">
+        <v>0</v>
+      </c>
+      <c r="G372" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>